<commit_message>
Add two Kassbohrer Maxima curtain-side trailers (2023 VIN ...4397, 2022 VIN ...6344)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KRzo6JwTr8ExLnQ6Y4iSPg
</commit_message>
<xml_diff>
--- a/avito-feed-trailers/fleet-trailers.xlsx
+++ b/avito-feed-trailers/fleet-trailers.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BE2"/>
+  <dimension ref="A1:BE4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -467,7 +467,7 @@
     <col width="26" customWidth="1" min="48" max="48"/>
     <col width="13" customWidth="1" min="49" max="49"/>
     <col width="17" customWidth="1" min="50" max="50"/>
-    <col width="16" customWidth="1" min="51" max="51"/>
+    <col width="34" customWidth="1" min="51" max="51"/>
     <col width="14" customWidth="1" min="52" max="52"/>
     <col width="23" customWidth="1" min="53" max="53"/>
     <col width="15" customWidth="1" min="54" max="54"/>
@@ -929,6 +929,348 @@
       <c r="BD2" s="1" t="inlineStr"/>
       <c r="BE2" s="1" t="inlineStr"/>
     </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Москва, Ижорская ул., 15с2</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr"/>
+      <c r="C3" s="1" t="inlineStr"/>
+      <c r="D3" s="1" t="inlineStr">
+        <is>
+          <t>kassbohrer-maxima-shtor-00116344</t>
+        </is>
+      </c>
+      <c r="E3" s="1" t="inlineStr"/>
+      <c r="F3" s="1" t="inlineStr"/>
+      <c r="G3" s="1" t="inlineStr"/>
+      <c r="H3" s="1" t="inlineStr"/>
+      <c r="I3" s="1" t="inlineStr"/>
+      <c r="J3" s="1" t="inlineStr"/>
+      <c r="K3" s="1" t="inlineStr"/>
+      <c r="L3" s="1" t="inlineStr">
+        <is>
+          <t>По телефону и в сообщениях</t>
+        </is>
+      </c>
+      <c r="M3" s="1" t="inlineStr">
+        <is>
+          <t>Полуприцеп шторный Kassbohrer Maxima, 2022 год выпуска, TIR-исполнение.
+Оси BPW, 3 шт., подвеска зависимая на продольных рычагах, тормоза барабанные. Шины бескамерные 385/65R22,5, односкат, Bridgestone.
+Масса снаряжённого полуприцепа 8 960 кг, грузоподъёмность 28 540 кг, разрешённая максимальная масса 37 500 кг.
+Внутренние размеры 16 520×2 480×2 700 мм, объём кузова 110,6 м³. Высота ССУ 1150 мм.
+Боковая обшивка из фанеры, пол — ламинированная фанера 27 мм.
+Техническое состояние — на ходу, полностью исправен, не требует вложений и ремонта.
+Документы в порядке.
+Возможна аренда с правом выкупа — уточняйте условия по телефону.
+Смотровая площадка и показ — по договорённости. Торг при осмотре.</t>
+        </is>
+      </c>
+      <c r="N3" s="1" t="inlineStr">
+        <is>
+          <t>Грузовики и спецтехника</t>
+        </is>
+      </c>
+      <c r="O3" s="1" t="inlineStr">
+        <is>
+          <t>3400000</t>
+        </is>
+      </c>
+      <c r="P3" s="1" t="inlineStr"/>
+      <c r="Q3" s="1" t="inlineStr"/>
+      <c r="R3" s="1" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00116344/01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00116344/02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00116344/03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00116344/04.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00116344/05.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00116344/06.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00116344/07.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00116344/08.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00116344/09.jpg</t>
+        </is>
+      </c>
+      <c r="S3" s="1" t="inlineStr"/>
+      <c r="T3" s="1" t="inlineStr"/>
+      <c r="U3" s="1" t="inlineStr"/>
+      <c r="V3" s="1" t="inlineStr"/>
+      <c r="W3" s="1" t="inlineStr"/>
+      <c r="X3" s="1" t="inlineStr">
+        <is>
+          <t>Прицепы</t>
+        </is>
+      </c>
+      <c r="Y3" s="1" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="Z3" s="1" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="AA3" s="1" t="inlineStr"/>
+      <c r="AB3" s="1" t="inlineStr">
+        <is>
+          <t>3400000</t>
+        </is>
+      </c>
+      <c r="AC3" s="1" t="inlineStr">
+        <is>
+          <t>В наличии</t>
+        </is>
+      </c>
+      <c r="AD3" s="1" t="inlineStr"/>
+      <c r="AE3" s="1" t="inlineStr"/>
+      <c r="AF3" s="1" t="inlineStr"/>
+      <c r="AG3" s="1" t="inlineStr"/>
+      <c r="AH3" s="1" t="inlineStr"/>
+      <c r="AI3" s="1" t="inlineStr"/>
+      <c r="AJ3" s="1" t="inlineStr"/>
+      <c r="AK3" s="1" t="inlineStr"/>
+      <c r="AL3" s="1" t="inlineStr"/>
+      <c r="AM3" s="1" t="inlineStr">
+        <is>
+          <t>С пробегом</t>
+        </is>
+      </c>
+      <c r="AN3" s="1" t="inlineStr"/>
+      <c r="AO3" s="1" t="inlineStr">
+        <is>
+          <t>В наличии</t>
+        </is>
+      </c>
+      <c r="AP3" s="1" t="inlineStr">
+        <is>
+          <t>Kassbohrer</t>
+        </is>
+      </c>
+      <c r="AQ3" s="1" t="inlineStr">
+        <is>
+          <t>Maxima</t>
+        </is>
+      </c>
+      <c r="AR3" s="1" t="inlineStr">
+        <is>
+          <t>Полуприцеп</t>
+        </is>
+      </c>
+      <c r="AS3" s="1" t="inlineStr">
+        <is>
+          <t>Шторный</t>
+        </is>
+      </c>
+      <c r="AT3" s="1" t="inlineStr"/>
+      <c r="AU3" s="1" t="inlineStr"/>
+      <c r="AV3" s="1" t="inlineStr">
+        <is>
+          <t>WKVDAF30300116344</t>
+        </is>
+      </c>
+      <c r="AW3" s="1" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="AX3" s="1" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AY3" s="1" t="inlineStr">
+        <is>
+          <t>Зависимая, на продольных рычагах</t>
+        </is>
+      </c>
+      <c r="AZ3" s="1" t="inlineStr">
+        <is>
+          <t>Барабанные</t>
+        </is>
+      </c>
+      <c r="BA3" s="1" t="inlineStr">
+        <is>
+          <t>28540</t>
+        </is>
+      </c>
+      <c r="BB3" s="1" t="inlineStr">
+        <is>
+          <t>16520</t>
+        </is>
+      </c>
+      <c r="BC3" s="1" t="inlineStr">
+        <is>
+          <t>110.6</t>
+        </is>
+      </c>
+      <c r="BD3" s="1" t="inlineStr"/>
+      <c r="BE3" s="1" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>Москва, Ижорская ул., 15с2</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr"/>
+      <c r="C4" s="1" t="inlineStr"/>
+      <c r="D4" s="1" t="inlineStr">
+        <is>
+          <t>kassbohrer-maxima-shtor-00124397</t>
+        </is>
+      </c>
+      <c r="E4" s="1" t="inlineStr"/>
+      <c r="F4" s="1" t="inlineStr"/>
+      <c r="G4" s="1" t="inlineStr"/>
+      <c r="H4" s="1" t="inlineStr"/>
+      <c r="I4" s="1" t="inlineStr"/>
+      <c r="J4" s="1" t="inlineStr"/>
+      <c r="K4" s="1" t="inlineStr"/>
+      <c r="L4" s="1" t="inlineStr">
+        <is>
+          <t>По телефону и в сообщениях</t>
+        </is>
+      </c>
+      <c r="M4" s="1" t="inlineStr">
+        <is>
+          <t>Полуприцеп шторный Kassbohrer Maxima, 2023 год выпуска, TIR-исполнение.
+Оси BPW, 3 шт., подвеска зависимая на продольных рычагах, тормоза барабанные. Шины бескамерные 385/65R22,5, односкат, Bridgestone.
+Масса снаряжённого полуприцепа 8 960 кг, грузоподъёмность 28 540 кг, разрешённая максимальная масса 37 500 кг.
+Внутренние размеры 16 520×2 480×2 700 мм, объём кузова 110,6 м³. Высота ССУ 1150 мм.
+Боковая обшивка из фанеры, пол — ламинированная фанера 27 мм.
+Техническое состояние — на ходу, полностью исправен, не требует вложений и ремонта.
+Документы в порядке.
+Возможна аренда с правом выкупа — уточняйте условия по телефону.
+Смотровая площадка и показ — по договорённости. Торг при осмотре.</t>
+        </is>
+      </c>
+      <c r="N4" s="1" t="inlineStr">
+        <is>
+          <t>Грузовики и спецтехника</t>
+        </is>
+      </c>
+      <c r="O4" s="1" t="inlineStr">
+        <is>
+          <t>3950000</t>
+        </is>
+      </c>
+      <c r="P4" s="1" t="inlineStr"/>
+      <c r="Q4" s="1" t="inlineStr"/>
+      <c r="R4" s="1" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124397/01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124397/02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124397/03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124397/04.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124397/05.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124397/06.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124397/07.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124397/08.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124397/09.jpg</t>
+        </is>
+      </c>
+      <c r="S4" s="1" t="inlineStr"/>
+      <c r="T4" s="1" t="inlineStr"/>
+      <c r="U4" s="1" t="inlineStr"/>
+      <c r="V4" s="1" t="inlineStr"/>
+      <c r="W4" s="1" t="inlineStr"/>
+      <c r="X4" s="1" t="inlineStr">
+        <is>
+          <t>Прицепы</t>
+        </is>
+      </c>
+      <c r="Y4" s="1" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="Z4" s="1" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="AA4" s="1" t="inlineStr"/>
+      <c r="AB4" s="1" t="inlineStr">
+        <is>
+          <t>3950000</t>
+        </is>
+      </c>
+      <c r="AC4" s="1" t="inlineStr">
+        <is>
+          <t>В наличии</t>
+        </is>
+      </c>
+      <c r="AD4" s="1" t="inlineStr"/>
+      <c r="AE4" s="1" t="inlineStr"/>
+      <c r="AF4" s="1" t="inlineStr"/>
+      <c r="AG4" s="1" t="inlineStr"/>
+      <c r="AH4" s="1" t="inlineStr"/>
+      <c r="AI4" s="1" t="inlineStr"/>
+      <c r="AJ4" s="1" t="inlineStr"/>
+      <c r="AK4" s="1" t="inlineStr"/>
+      <c r="AL4" s="1" t="inlineStr"/>
+      <c r="AM4" s="1" t="inlineStr">
+        <is>
+          <t>С пробегом</t>
+        </is>
+      </c>
+      <c r="AN4" s="1" t="inlineStr"/>
+      <c r="AO4" s="1" t="inlineStr">
+        <is>
+          <t>В наличии</t>
+        </is>
+      </c>
+      <c r="AP4" s="1" t="inlineStr">
+        <is>
+          <t>Kassbohrer</t>
+        </is>
+      </c>
+      <c r="AQ4" s="1" t="inlineStr">
+        <is>
+          <t>Maxima</t>
+        </is>
+      </c>
+      <c r="AR4" s="1" t="inlineStr">
+        <is>
+          <t>Полуприцеп</t>
+        </is>
+      </c>
+      <c r="AS4" s="1" t="inlineStr">
+        <is>
+          <t>Шторный</t>
+        </is>
+      </c>
+      <c r="AT4" s="1" t="inlineStr"/>
+      <c r="AU4" s="1" t="inlineStr"/>
+      <c r="AV4" s="1" t="inlineStr">
+        <is>
+          <t>WKVDAF30300124397</t>
+        </is>
+      </c>
+      <c r="AW4" s="1" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="AX4" s="1" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AY4" s="1" t="inlineStr">
+        <is>
+          <t>Зависимая, на продольных рычагах</t>
+        </is>
+      </c>
+      <c r="AZ4" s="1" t="inlineStr">
+        <is>
+          <t>Барабанные</t>
+        </is>
+      </c>
+      <c r="BA4" s="1" t="inlineStr">
+        <is>
+          <t>28540</t>
+        </is>
+      </c>
+      <c r="BB4" s="1" t="inlineStr">
+        <is>
+          <t>16520</t>
+        </is>
+      </c>
+      <c r="BC4" s="1" t="inlineStr">
+        <is>
+          <t>110.6</t>
+        </is>
+      </c>
+      <c r="BD4" s="1" t="inlineStr"/>
+      <c r="BE4" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix trailer photo mixup: correct curtain-side photos for shtor units, add VIN to iso trailer from ЭПТС
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KRzo6JwTr8ExLnQ6Y4iSPg
</commit_message>
<xml_diff>
--- a/avito-feed-trailers/fleet-trailers.xlsx
+++ b/avito-feed-trailers/fleet-trailers.xlsx
@@ -890,7 +890,11 @@
       </c>
       <c r="AT2" s="1" t="inlineStr"/>
       <c r="AU2" s="1" t="inlineStr"/>
-      <c r="AV2" s="1" t="inlineStr"/>
+      <c r="AV2" s="1" t="inlineStr">
+        <is>
+          <t>WKVDAF10300124805</t>
+        </is>
+      </c>
       <c r="AW2" s="1" t="inlineStr">
         <is>
           <t>2023</t>
@@ -981,7 +985,7 @@
       <c r="Q3" s="1" t="inlineStr"/>
       <c r="R3" s="1" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00116344/01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00116344/02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00116344/03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00116344/04.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00116344/05.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00116344/06.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00116344/07.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00116344/08.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00116344/09.jpg</t>
+          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00116344/01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00116344/02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00116344/03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00116344/04.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00116344/05.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00116344/06.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00116344/07.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00116344/08.jpg</t>
         </is>
       </c>
       <c r="S3" s="1" t="inlineStr"/>
@@ -1152,7 +1156,7 @@
       <c r="Q4" s="1" t="inlineStr"/>
       <c r="R4" s="1" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124397/01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124397/02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124397/03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124397/04.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124397/05.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124397/06.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124397/07.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124397/08.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124397/09.jpg</t>
+          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124397/01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124397/02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124397/03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124397/04.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124397/05.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124397/06.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124397/07.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124397/08.jpg</t>
         </is>
       </c>
       <c r="S4" s="1" t="inlineStr"/>

</xml_diff>

<commit_message>
Add Steelbear PL-24L log semi-trailer (2024, sold to order, no VIN — already listed elsewhere under this VIN)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KRzo6JwTr8ExLnQ6Y4iSPg
</commit_message>
<xml_diff>
--- a/avito-feed-trailers/fleet-trailers.xlsx
+++ b/avito-feed-trailers/fleet-trailers.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BE4"/>
+  <dimension ref="A1:BE5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1275,6 +1275,166 @@
       <c r="BD4" s="1" t="inlineStr"/>
       <c r="BE4" s="1" t="inlineStr"/>
     </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>Москва, Ижорская ул., 15с2</t>
+        </is>
+      </c>
+      <c r="B5" s="1" t="inlineStr"/>
+      <c r="C5" s="1" t="inlineStr"/>
+      <c r="D5" s="1" t="inlineStr">
+        <is>
+          <t>steelbear-pl24l-ea653666</t>
+        </is>
+      </c>
+      <c r="E5" s="1" t="inlineStr"/>
+      <c r="F5" s="1" t="inlineStr"/>
+      <c r="G5" s="1" t="inlineStr"/>
+      <c r="H5" s="1" t="inlineStr"/>
+      <c r="I5" s="1" t="inlineStr"/>
+      <c r="J5" s="1" t="inlineStr"/>
+      <c r="K5" s="1" t="inlineStr"/>
+      <c r="L5" s="1" t="inlineStr">
+        <is>
+          <t>По телефону и в сообщениях</t>
+        </is>
+      </c>
+      <c r="M5" s="1" t="inlineStr">
+        <is>
+          <t>Полуприцеп-сортиментовоз Steelbear PL-24L (коммерческое название PT-24L BPW Heavy Duty), 2024 год выпуска, под заказ.
+Усиленное шасси из двутавровых лонжеронов, 3 оси BPW Heavy Duty, барабанные тормоза, пневмоподвеска с функцией подъём/опускание, допустимая нагрузка на ось 9 000 кг. Шины 385/65R22,5, односкат. Электронная тормозная система WABCO TEBS-E с функцией противоопрокидывания (RSS).
+6 пар открепляемых коников грузоподъёмностью 8 тонн каждая (сталь STRENX 700MC), положение регулируется вдоль рамы. Внутренняя высота коника 2330 мм. Настил из ламинированной берёзовой фанеры. Опорное устройство BPW, 24 т.
+Максимальная полная масса 44 000 кг, грузоподъёмность 37 100 кг, длина 13 620 мм.
+Заводская гарантия — 24 месяца, от сквозной коррозии — 10 лет.
+Поставка под заказ, срок — уточняйте.</t>
+        </is>
+      </c>
+      <c r="N5" s="1" t="inlineStr">
+        <is>
+          <t>Грузовики и спецтехника</t>
+        </is>
+      </c>
+      <c r="O5" s="1" t="inlineStr">
+        <is>
+          <t>2970000</t>
+        </is>
+      </c>
+      <c r="P5" s="1" t="inlineStr"/>
+      <c r="Q5" s="1" t="inlineStr"/>
+      <c r="R5" s="1" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/04.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/05.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/06.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/07.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/08.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/09.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/10.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/11.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/12.jpg</t>
+        </is>
+      </c>
+      <c r="S5" s="1" t="inlineStr"/>
+      <c r="T5" s="1" t="inlineStr"/>
+      <c r="U5" s="1" t="inlineStr"/>
+      <c r="V5" s="1" t="inlineStr"/>
+      <c r="W5" s="1" t="inlineStr"/>
+      <c r="X5" s="1" t="inlineStr">
+        <is>
+          <t>Прицепы</t>
+        </is>
+      </c>
+      <c r="Y5" s="1" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="Z5" s="1" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="AA5" s="1" t="inlineStr"/>
+      <c r="AB5" s="1" t="inlineStr">
+        <is>
+          <t>2970000</t>
+        </is>
+      </c>
+      <c r="AC5" s="1" t="inlineStr">
+        <is>
+          <t>Под заказ</t>
+        </is>
+      </c>
+      <c r="AD5" s="1" t="inlineStr"/>
+      <c r="AE5" s="1" t="inlineStr"/>
+      <c r="AF5" s="1" t="inlineStr"/>
+      <c r="AG5" s="1" t="inlineStr"/>
+      <c r="AH5" s="1" t="inlineStr"/>
+      <c r="AI5" s="1" t="inlineStr"/>
+      <c r="AJ5" s="1" t="inlineStr"/>
+      <c r="AK5" s="1" t="inlineStr"/>
+      <c r="AL5" s="1" t="inlineStr"/>
+      <c r="AM5" s="1" t="inlineStr">
+        <is>
+          <t>С пробегом</t>
+        </is>
+      </c>
+      <c r="AN5" s="1" t="inlineStr"/>
+      <c r="AO5" s="1" t="inlineStr">
+        <is>
+          <t>В наличии</t>
+        </is>
+      </c>
+      <c r="AP5" s="1" t="inlineStr">
+        <is>
+          <t>Steelbear</t>
+        </is>
+      </c>
+      <c r="AQ5" s="1" t="inlineStr">
+        <is>
+          <t>PL-24L</t>
+        </is>
+      </c>
+      <c r="AR5" s="1" t="inlineStr">
+        <is>
+          <t>Полуприцеп</t>
+        </is>
+      </c>
+      <c r="AS5" s="1" t="inlineStr">
+        <is>
+          <t>Сортиментовоз</t>
+        </is>
+      </c>
+      <c r="AT5" s="1" t="inlineStr"/>
+      <c r="AU5" s="1" t="inlineStr"/>
+      <c r="AV5" s="1" t="inlineStr"/>
+      <c r="AW5" s="1" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="AX5" s="1" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AY5" s="1" t="inlineStr">
+        <is>
+          <t>Пневматическая</t>
+        </is>
+      </c>
+      <c r="AZ5" s="1" t="inlineStr">
+        <is>
+          <t>Барабанные</t>
+        </is>
+      </c>
+      <c r="BA5" s="1" t="inlineStr">
+        <is>
+          <t>37100</t>
+        </is>
+      </c>
+      <c r="BB5" s="1" t="inlineStr">
+        <is>
+          <t>13620</t>
+        </is>
+      </c>
+      <c r="BC5" s="1" t="inlineStr"/>
+      <c r="BD5" s="1" t="inlineStr"/>
+      <c r="BE5" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix rejected suspension value on both curtain-side Kassbohrer trailers (Рессорная instead of long-form description)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KRzo6JwTr8ExLnQ6Y4iSPg
</commit_message>
<xml_diff>
--- a/avito-feed-trailers/fleet-trailers.xlsx
+++ b/avito-feed-trailers/fleet-trailers.xlsx
@@ -467,7 +467,7 @@
     <col width="26" customWidth="1" min="48" max="48"/>
     <col width="13" customWidth="1" min="49" max="49"/>
     <col width="17" customWidth="1" min="50" max="50"/>
-    <col width="34" customWidth="1" min="51" max="51"/>
+    <col width="16" customWidth="1" min="51" max="51"/>
     <col width="14" customWidth="1" min="52" max="52"/>
     <col width="23" customWidth="1" min="53" max="53"/>
     <col width="15" customWidth="1" min="54" max="54"/>
@@ -1078,7 +1078,7 @@
       </c>
       <c r="AY3" s="1" t="inlineStr">
         <is>
-          <t>Зависимая, на продольных рычагах</t>
+          <t>Рессорная</t>
         </is>
       </c>
       <c r="AZ3" s="1" t="inlineStr">
@@ -1249,7 +1249,7 @@
       </c>
       <c r="AY4" s="1" t="inlineStr">
         <is>
-          <t>Зависимая, на продольных рычагах</t>
+          <t>Рессорная</t>
         </is>
       </c>
       <c r="AZ4" s="1" t="inlineStr">

</xml_diff>

<commit_message>
Fix rejected TypeOfTrailer value for Steelbear log trailer (Лесовоз (сортиментовоз))
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KRzo6JwTr8ExLnQ6Y4iSPg
</commit_message>
<xml_diff>
--- a/avito-feed-trailers/fleet-trailers.xlsx
+++ b/avito-feed-trailers/fleet-trailers.xlsx
@@ -461,7 +461,7 @@
     <col width="12" customWidth="1" min="42" max="42"/>
     <col width="10" customWidth="1" min="43" max="43"/>
     <col width="13" customWidth="1" min="44" max="44"/>
-    <col width="16" customWidth="1" min="45" max="45"/>
+    <col width="25" customWidth="1" min="45" max="45"/>
     <col width="11" customWidth="1" min="46" max="46"/>
     <col width="12" customWidth="1" min="47" max="47"/>
     <col width="26" customWidth="1" min="48" max="48"/>
@@ -1395,7 +1395,7 @@
       </c>
       <c r="AS5" s="1" t="inlineStr">
         <is>
-          <t>Сортиментовоз</t>
+          <t>Лесовоз (сортиментовоз)</t>
         </is>
       </c>
       <c r="AT5" s="1" t="inlineStr"/>

</xml_diff>

<commit_message>
Add third Kassbohrer Maxima curtain trailer (13.6m, 2023, VIN ...4732), priced below market comps
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KRzo6JwTr8ExLnQ6Y4iSPg
</commit_message>
<xml_diff>
--- a/avito-feed-trailers/fleet-trailers.xlsx
+++ b/avito-feed-trailers/fleet-trailers.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BE5"/>
+  <dimension ref="A1:BE6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1285,7 +1285,7 @@
       <c r="C5" s="1" t="inlineStr"/>
       <c r="D5" s="1" t="inlineStr">
         <is>
-          <t>steelbear-pl24l-ea653666</t>
+          <t>kassbohrer-maxima-shtor-00124732</t>
         </is>
       </c>
       <c r="E5" s="1" t="inlineStr"/>
@@ -1302,12 +1302,15 @@
       </c>
       <c r="M5" s="1" t="inlineStr">
         <is>
-          <t>Полуприцеп-сортиментовоз Steelbear PL-24L (коммерческое название PT-24L BPW Heavy Duty), 2024 год выпуска, под заказ.
-Усиленное шасси из двутавровых лонжеронов, 3 оси BPW Heavy Duty, барабанные тормоза, пневмоподвеска с функцией подъём/опускание, допустимая нагрузка на ось 9 000 кг. Шины 385/65R22,5, односкат. Электронная тормозная система WABCO TEBS-E с функцией противоопрокидывания (RSS).
-6 пар открепляемых коников грузоподъёмностью 8 тонн каждая (сталь STRENX 700MC), положение регулируется вдоль рамы. Внутренняя высота коника 2330 мм. Настил из ламинированной берёзовой фанеры. Опорное устройство BPW, 24 т.
-Максимальная полная масса 44 000 кг, грузоподъёмность 37 100 кг, длина 13 620 мм.
-Заводская гарантия — 24 месяца, от сквозной коррозии — 10 лет.
-Поставка под заказ, срок — уточняйте.</t>
+          <t>Полуприцеп шторный Kassbohrer, 2023 год выпуска, TIR-исполнение.
+Оси BPW, 3 шт., подвеска рессорная, тормоза барабанные. Шины бескамерные 385/65R22,5, односкат, Bridgestone.
+Масса снаряжённого 7 630 кг, грузоподъёмность 28 540 кг, разрешённая максимальная масса 39 000 кг.
+Внутренние размеры 13 600×2 480×2 700 мм, объём кузова 92 м³. Высота ССУ 1150 мм.
+Боковая обшивка из фанеры, пол — ламинированная фанера 30 мм.
+Техническое состояние — на ходу, полностью исправен, не требует вложений и ремонта.
+Документы в порядке.
+Возможна аренда с правом выкупа — уточняйте условия по телефону.
+Смотровая площадка и показ — по договорённости. Торг при осмотре.</t>
         </is>
       </c>
       <c r="N5" s="1" t="inlineStr">
@@ -1317,14 +1320,14 @@
       </c>
       <c r="O5" s="1" t="inlineStr">
         <is>
-          <t>2970000</t>
+          <t>3390000</t>
         </is>
       </c>
       <c r="P5" s="1" t="inlineStr"/>
       <c r="Q5" s="1" t="inlineStr"/>
       <c r="R5" s="1" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/04.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/05.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/06.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/07.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/08.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/09.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/10.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/11.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/12.jpg</t>
+          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124732/01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124732/02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124732/03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124732/04.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124732/05.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124732/06.jpg</t>
         </is>
       </c>
       <c r="S5" s="1" t="inlineStr"/>
@@ -1350,12 +1353,12 @@
       <c r="AA5" s="1" t="inlineStr"/>
       <c r="AB5" s="1" t="inlineStr">
         <is>
-          <t>2970000</t>
+          <t>3390000</t>
         </is>
       </c>
       <c r="AC5" s="1" t="inlineStr">
         <is>
-          <t>Под заказ</t>
+          <t>В наличии</t>
         </is>
       </c>
       <c r="AD5" s="1" t="inlineStr"/>
@@ -1380,12 +1383,12 @@
       </c>
       <c r="AP5" s="1" t="inlineStr">
         <is>
-          <t>Steelbear</t>
+          <t>Kassbohrer</t>
         </is>
       </c>
       <c r="AQ5" s="1" t="inlineStr">
         <is>
-          <t>PL-24L</t>
+          <t>Maxima</t>
         </is>
       </c>
       <c r="AR5" s="1" t="inlineStr">
@@ -1395,15 +1398,19 @@
       </c>
       <c r="AS5" s="1" t="inlineStr">
         <is>
-          <t>Лесовоз (сортиментовоз)</t>
+          <t>Шторный</t>
         </is>
       </c>
       <c r="AT5" s="1" t="inlineStr"/>
       <c r="AU5" s="1" t="inlineStr"/>
-      <c r="AV5" s="1" t="inlineStr"/>
+      <c r="AV5" s="1" t="inlineStr">
+        <is>
+          <t>WKVDAF30300124732</t>
+        </is>
+      </c>
       <c r="AW5" s="1" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2023</t>
         </is>
       </c>
       <c r="AX5" s="1" t="inlineStr">
@@ -1413,7 +1420,7 @@
       </c>
       <c r="AY5" s="1" t="inlineStr">
         <is>
-          <t>Пневматическая</t>
+          <t>Рессорная</t>
         </is>
       </c>
       <c r="AZ5" s="1" t="inlineStr">
@@ -1423,17 +1430,181 @@
       </c>
       <c r="BA5" s="1" t="inlineStr">
         <is>
-          <t>37100</t>
+          <t>28540</t>
         </is>
       </c>
       <c r="BB5" s="1" t="inlineStr">
         <is>
-          <t>13620</t>
-        </is>
-      </c>
-      <c r="BC5" s="1" t="inlineStr"/>
+          <t>13600</t>
+        </is>
+      </c>
+      <c r="BC5" s="1" t="inlineStr">
+        <is>
+          <t>92</t>
+        </is>
+      </c>
       <c r="BD5" s="1" t="inlineStr"/>
       <c r="BE5" s="1" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>Москва, Ижорская ул., 15с2</t>
+        </is>
+      </c>
+      <c r="B6" s="1" t="inlineStr"/>
+      <c r="C6" s="1" t="inlineStr"/>
+      <c r="D6" s="1" t="inlineStr">
+        <is>
+          <t>steelbear-pl24l-ea653666</t>
+        </is>
+      </c>
+      <c r="E6" s="1" t="inlineStr"/>
+      <c r="F6" s="1" t="inlineStr"/>
+      <c r="G6" s="1" t="inlineStr"/>
+      <c r="H6" s="1" t="inlineStr"/>
+      <c r="I6" s="1" t="inlineStr"/>
+      <c r="J6" s="1" t="inlineStr"/>
+      <c r="K6" s="1" t="inlineStr"/>
+      <c r="L6" s="1" t="inlineStr">
+        <is>
+          <t>По телефону и в сообщениях</t>
+        </is>
+      </c>
+      <c r="M6" s="1" t="inlineStr">
+        <is>
+          <t>Полуприцеп-сортиментовоз Steelbear PL-24L (коммерческое название PT-24L BPW Heavy Duty), 2024 год выпуска, под заказ.
+Усиленное шасси из двутавровых лонжеронов, 3 оси BPW Heavy Duty, барабанные тормоза, пневмоподвеска с функцией подъём/опускание, допустимая нагрузка на ось 9 000 кг. Шины 385/65R22,5, односкат. Электронная тормозная система WABCO TEBS-E с функцией противоопрокидывания (RSS).
+6 пар открепляемых коников грузоподъёмностью 8 тонн каждая (сталь STRENX 700MC), положение регулируется вдоль рамы. Внутренняя высота коника 2330 мм. Настил из ламинированной берёзовой фанеры. Опорное устройство BPW, 24 т.
+Максимальная полная масса 44 000 кг, грузоподъёмность 37 100 кг, длина 13 620 мм.
+Заводская гарантия — 24 месяца, от сквозной коррозии — 10 лет.
+Поставка под заказ, срок — уточняйте.</t>
+        </is>
+      </c>
+      <c r="N6" s="1" t="inlineStr">
+        <is>
+          <t>Грузовики и спецтехника</t>
+        </is>
+      </c>
+      <c r="O6" s="1" t="inlineStr">
+        <is>
+          <t>2970000</t>
+        </is>
+      </c>
+      <c r="P6" s="1" t="inlineStr"/>
+      <c r="Q6" s="1" t="inlineStr"/>
+      <c r="R6" s="1" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/04.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/05.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/06.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/07.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/08.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/09.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/10.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/11.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/12.jpg</t>
+        </is>
+      </c>
+      <c r="S6" s="1" t="inlineStr"/>
+      <c r="T6" s="1" t="inlineStr"/>
+      <c r="U6" s="1" t="inlineStr"/>
+      <c r="V6" s="1" t="inlineStr"/>
+      <c r="W6" s="1" t="inlineStr"/>
+      <c r="X6" s="1" t="inlineStr">
+        <is>
+          <t>Прицепы</t>
+        </is>
+      </c>
+      <c r="Y6" s="1" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="Z6" s="1" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="AA6" s="1" t="inlineStr"/>
+      <c r="AB6" s="1" t="inlineStr">
+        <is>
+          <t>2970000</t>
+        </is>
+      </c>
+      <c r="AC6" s="1" t="inlineStr">
+        <is>
+          <t>Под заказ</t>
+        </is>
+      </c>
+      <c r="AD6" s="1" t="inlineStr"/>
+      <c r="AE6" s="1" t="inlineStr"/>
+      <c r="AF6" s="1" t="inlineStr"/>
+      <c r="AG6" s="1" t="inlineStr"/>
+      <c r="AH6" s="1" t="inlineStr"/>
+      <c r="AI6" s="1" t="inlineStr"/>
+      <c r="AJ6" s="1" t="inlineStr"/>
+      <c r="AK6" s="1" t="inlineStr"/>
+      <c r="AL6" s="1" t="inlineStr"/>
+      <c r="AM6" s="1" t="inlineStr">
+        <is>
+          <t>С пробегом</t>
+        </is>
+      </c>
+      <c r="AN6" s="1" t="inlineStr"/>
+      <c r="AO6" s="1" t="inlineStr">
+        <is>
+          <t>В наличии</t>
+        </is>
+      </c>
+      <c r="AP6" s="1" t="inlineStr">
+        <is>
+          <t>Steelbear</t>
+        </is>
+      </c>
+      <c r="AQ6" s="1" t="inlineStr">
+        <is>
+          <t>PL-24L</t>
+        </is>
+      </c>
+      <c r="AR6" s="1" t="inlineStr">
+        <is>
+          <t>Полуприцеп</t>
+        </is>
+      </c>
+      <c r="AS6" s="1" t="inlineStr">
+        <is>
+          <t>Лесовоз (сортиментовоз)</t>
+        </is>
+      </c>
+      <c r="AT6" s="1" t="inlineStr"/>
+      <c r="AU6" s="1" t="inlineStr"/>
+      <c r="AV6" s="1" t="inlineStr"/>
+      <c r="AW6" s="1" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="AX6" s="1" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AY6" s="1" t="inlineStr">
+        <is>
+          <t>Пневматическая</t>
+        </is>
+      </c>
+      <c r="AZ6" s="1" t="inlineStr">
+        <is>
+          <t>Барабанные</t>
+        </is>
+      </c>
+      <c r="BA6" s="1" t="inlineStr">
+        <is>
+          <t>37100</t>
+        </is>
+      </c>
+      <c r="BB6" s="1" t="inlineStr">
+        <is>
+          <t>13620</t>
+        </is>
+      </c>
+      <c r="BC6" s="1" t="inlineStr"/>
+      <c r="BD6" s="1" t="inlineStr"/>
+      <c r="BE6" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Lower prices on all three Kassbohrer curtain trailers for lead-gen (rent-to-buy business, price is bait not final terms)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KRzo6JwTr8ExLnQ6Y4iSPg
</commit_message>
<xml_diff>
--- a/avito-feed-trailers/fleet-trailers.xlsx
+++ b/avito-feed-trailers/fleet-trailers.xlsx
@@ -978,7 +978,7 @@
       </c>
       <c r="O3" s="1" t="inlineStr">
         <is>
-          <t>3400000</t>
+          <t>2890000</t>
         </is>
       </c>
       <c r="P3" s="1" t="inlineStr"/>
@@ -1011,7 +1011,7 @@
       <c r="AA3" s="1" t="inlineStr"/>
       <c r="AB3" s="1" t="inlineStr">
         <is>
-          <t>3400000</t>
+          <t>2890000</t>
         </is>
       </c>
       <c r="AC3" s="1" t="inlineStr">
@@ -1149,7 +1149,7 @@
       </c>
       <c r="O4" s="1" t="inlineStr">
         <is>
-          <t>3950000</t>
+          <t>3290000</t>
         </is>
       </c>
       <c r="P4" s="1" t="inlineStr"/>
@@ -1182,7 +1182,7 @@
       <c r="AA4" s="1" t="inlineStr"/>
       <c r="AB4" s="1" t="inlineStr">
         <is>
-          <t>3950000</t>
+          <t>3290000</t>
         </is>
       </c>
       <c r="AC4" s="1" t="inlineStr">
@@ -1320,7 +1320,7 @@
       </c>
       <c r="O5" s="1" t="inlineStr">
         <is>
-          <t>3390000</t>
+          <t>2890000</t>
         </is>
       </c>
       <c r="P5" s="1" t="inlineStr"/>
@@ -1353,7 +1353,7 @@
       <c r="AA5" s="1" t="inlineStr"/>
       <c r="AB5" s="1" t="inlineStr">
         <is>
-          <t>3390000</t>
+          <t>2890000</t>
         </is>
       </c>
       <c r="AC5" s="1" t="inlineStr">

</xml_diff>

<commit_message>
Add V-Trailer 329D (2023, 13.6m, VIN XZFVKRP3DR0000119)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019CenkzpMJCXcxKtoErKpEq
</commit_message>
<xml_diff>
--- a/avito-feed-trailers/fleet-trailers.xlsx
+++ b/avito-feed-trailers/fleet-trailers.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BE6"/>
+  <dimension ref="A1:BE7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1606,6 +1606,173 @@
       <c r="BD6" s="1" t="inlineStr"/>
       <c r="BE6" s="1" t="inlineStr"/>
     </row>
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>Москва, Ижорская ул., 15с2</t>
+        </is>
+      </c>
+      <c r="B7" s="1" t="inlineStr"/>
+      <c r="C7" s="1" t="inlineStr"/>
+      <c r="D7" s="1" t="inlineStr">
+        <is>
+          <t>v-trailer-329d-r0000119</t>
+        </is>
+      </c>
+      <c r="E7" s="1" t="inlineStr"/>
+      <c r="F7" s="1" t="inlineStr"/>
+      <c r="G7" s="1" t="inlineStr"/>
+      <c r="H7" s="1" t="inlineStr"/>
+      <c r="I7" s="1" t="inlineStr"/>
+      <c r="J7" s="1" t="inlineStr"/>
+      <c r="K7" s="1" t="inlineStr"/>
+      <c r="L7" s="1" t="inlineStr">
+        <is>
+          <t>По телефону и в сообщениях</t>
+        </is>
+      </c>
+      <c r="M7" s="1" t="inlineStr">
+        <is>
+          <t>Шторный полуприцеп V-Trailer 329D, 2023 год, в работе, полностью исправен.
+Оси SAF, подъёмная передняя — меньше износ резины и расход на порожняке. Опорное устройство JOST на 24 тонны, шкворень 2 дюйма по ISO 1726. Пол — влагостойкая фанера 30 мм, держит погрузчик до 7,5 тонн. Крыша сдвижная (Sesam/Edscha) — грузить сверху краном или погрузчиком без снятия тента. Двери алюминиевые BPW Smartmaster II, передний и задний портал — собственная сварная конструкция, усиленная рама с дополнительными рёбрами жёсткости на скручивание. По бортам — корзины под коники, по 7 штук на сторону.
+13,6 × 2,5 × 4 м, 91 м³. Тент плотный: борта 900 г/м², крыша 680 г/м². Полная штора, без бортов — удобно под европаллеты и груз с выступом по высоте.
+VIN XZFVKRP3DR0000119.
+Возможна аренда с правом выкупа — уточняйте условия по телефону.</t>
+        </is>
+      </c>
+      <c r="N7" s="1" t="inlineStr">
+        <is>
+          <t>Грузовики и спецтехника</t>
+        </is>
+      </c>
+      <c r="O7" s="1" t="inlineStr">
+        <is>
+          <t>2990000</t>
+        </is>
+      </c>
+      <c r="P7" s="1" t="inlineStr"/>
+      <c r="Q7" s="1" t="inlineStr"/>
+      <c r="R7" s="1" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/04.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/05.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/06.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/07.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/08.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/09.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/10.jpg</t>
+        </is>
+      </c>
+      <c r="S7" s="1" t="inlineStr"/>
+      <c r="T7" s="1" t="inlineStr"/>
+      <c r="U7" s="1" t="inlineStr"/>
+      <c r="V7" s="1" t="inlineStr"/>
+      <c r="W7" s="1" t="inlineStr"/>
+      <c r="X7" s="1" t="inlineStr">
+        <is>
+          <t>Прицепы</t>
+        </is>
+      </c>
+      <c r="Y7" s="1" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="Z7" s="1" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="AA7" s="1" t="inlineStr"/>
+      <c r="AB7" s="1" t="inlineStr">
+        <is>
+          <t>2990000</t>
+        </is>
+      </c>
+      <c r="AC7" s="1" t="inlineStr">
+        <is>
+          <t>В наличии</t>
+        </is>
+      </c>
+      <c r="AD7" s="1" t="inlineStr"/>
+      <c r="AE7" s="1" t="inlineStr"/>
+      <c r="AF7" s="1" t="inlineStr"/>
+      <c r="AG7" s="1" t="inlineStr"/>
+      <c r="AH7" s="1" t="inlineStr"/>
+      <c r="AI7" s="1" t="inlineStr"/>
+      <c r="AJ7" s="1" t="inlineStr"/>
+      <c r="AK7" s="1" t="inlineStr"/>
+      <c r="AL7" s="1" t="inlineStr"/>
+      <c r="AM7" s="1" t="inlineStr">
+        <is>
+          <t>С пробегом</t>
+        </is>
+      </c>
+      <c r="AN7" s="1" t="inlineStr"/>
+      <c r="AO7" s="1" t="inlineStr">
+        <is>
+          <t>В наличии</t>
+        </is>
+      </c>
+      <c r="AP7" s="1" t="inlineStr">
+        <is>
+          <t>V-Trailer</t>
+        </is>
+      </c>
+      <c r="AQ7" s="1" t="inlineStr">
+        <is>
+          <t>329D</t>
+        </is>
+      </c>
+      <c r="AR7" s="1" t="inlineStr">
+        <is>
+          <t>Полуприцеп</t>
+        </is>
+      </c>
+      <c r="AS7" s="1" t="inlineStr">
+        <is>
+          <t>Шторный</t>
+        </is>
+      </c>
+      <c r="AT7" s="1" t="inlineStr"/>
+      <c r="AU7" s="1" t="inlineStr"/>
+      <c r="AV7" s="1" t="inlineStr">
+        <is>
+          <t>XZFVKRP3DR0000119</t>
+        </is>
+      </c>
+      <c r="AW7" s="1" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="AX7" s="1" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AY7" s="1" t="inlineStr">
+        <is>
+          <t>Пневматическая</t>
+        </is>
+      </c>
+      <c r="AZ7" s="1" t="inlineStr">
+        <is>
+          <t>Дисковые</t>
+        </is>
+      </c>
+      <c r="BA7" s="1" t="inlineStr">
+        <is>
+          <t>32300</t>
+        </is>
+      </c>
+      <c r="BB7" s="1" t="inlineStr">
+        <is>
+          <t>13600</t>
+        </is>
+      </c>
+      <c r="BC7" s="1" t="inlineStr">
+        <is>
+          <t>91</t>
+        </is>
+      </c>
+      <c r="BD7" s="1" t="inlineStr"/>
+      <c r="BE7" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add InterPricep 853375 container chassis (2024, VIN EAR853375R0000773)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019CenkzpMJCXcxKtoErKpEq
</commit_message>
<xml_diff>
--- a/avito-feed-trailers/fleet-trailers.xlsx
+++ b/avito-feed-trailers/fleet-trailers.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BE7"/>
+  <dimension ref="A1:BE8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -458,7 +458,7 @@
     <col width="12" customWidth="1" min="39" max="39"/>
     <col width="10" customWidth="1" min="40" max="40"/>
     <col width="13" customWidth="1" min="41" max="41"/>
-    <col width="12" customWidth="1" min="42" max="42"/>
+    <col width="13" customWidth="1" min="42" max="42"/>
     <col width="10" customWidth="1" min="43" max="43"/>
     <col width="13" customWidth="1" min="44" max="44"/>
     <col width="25" customWidth="1" min="45" max="45"/>
@@ -773,7 +773,7 @@
       <c r="C2" s="1" t="inlineStr"/>
       <c r="D2" s="1" t="inlineStr">
         <is>
-          <t>kassbohrer-maxima-iso-xx246877</t>
+          <t>interpricep-853375-r0000773</t>
         </is>
       </c>
       <c r="E2" s="1" t="inlineStr"/>
@@ -790,14 +790,12 @@
       </c>
       <c r="M2" s="1" t="inlineStr">
         <is>
-          <t>Полуприцеп изотермический Kassbohrer Maxima, 2023 год выпуска, TIR-исполнение.
-Оси BPW, 3 шт., подвеска пневматическая, тормоза барабанные.
-Грузоподъёмность 31 290 кг.
-Длина кузова 13,7 м, объём 94 м³.
-Техническое состояние — на ходу, полностью исправен, не требует вложений и ремонта.
-Документы в порядке.
-Возможна аренда — уточняйте условия по телефону.
-Смотровая площадка и показ — по договорённости. Торг при осмотре.</t>
+          <t>Полуприцеп-контейнеровоз ИнтерПрицеп 853375, 2024 год, в работе, полностью исправен.
+4 оси (3 + выносная балансирная), тормоза дисковые, ABS SORL. Подвеска пневматическая, с функцией подъёма осей — меньше износ резины на порожняке и разворотах. Шины 385/55R22.5, комплект 8+1 запасное.
+Берёт контейнеры 20', 30', 40' и High Cube — под большинство стандартных грузоперевозок без переоборудования. Разрешённая максимальная масса 47 000 кг, грузоподъёмность 41 000 кг. Высота погрузки 1 100 мм.
+Инструментальный ящик Daken, полный комплект пневморазводки и ЭБС.
+VIN EAR853375R0000773.
+Возможна аренда с правом выкупа — уточняйте условия по телефону.</t>
         </is>
       </c>
       <c r="N2" s="1" t="inlineStr">
@@ -807,14 +805,14 @@
       </c>
       <c r="O2" s="1" t="inlineStr">
         <is>
-          <t>4850000</t>
+          <t>1390000</t>
         </is>
       </c>
       <c r="P2" s="1" t="inlineStr"/>
       <c r="Q2" s="1" t="inlineStr"/>
       <c r="R2" s="1" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-iso-xx246877/01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-iso-xx246877/02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-iso-xx246877/03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-iso-xx246877/04.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-iso-xx246877/05.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-iso-xx246877/06.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-iso-xx246877/07.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-iso-xx246877/08.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-iso-xx246877/09.jpg</t>
+          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/interpricep-853375-r0000773/01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/interpricep-853375-r0000773/02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/interpricep-853375-r0000773/03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/interpricep-853375-r0000773/04.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/interpricep-853375-r0000773/05.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/interpricep-853375-r0000773/06.jpg</t>
         </is>
       </c>
       <c r="S2" s="1" t="inlineStr"/>
@@ -840,7 +838,7 @@
       <c r="AA2" s="1" t="inlineStr"/>
       <c r="AB2" s="1" t="inlineStr">
         <is>
-          <t>4850000</t>
+          <t>1390000</t>
         </is>
       </c>
       <c r="AC2" s="1" t="inlineStr">
@@ -870,12 +868,12 @@
       </c>
       <c r="AP2" s="1" t="inlineStr">
         <is>
-          <t>Kassbohrer</t>
+          <t>ИнтерПрицеп</t>
         </is>
       </c>
       <c r="AQ2" s="1" t="inlineStr">
         <is>
-          <t>Maxima</t>
+          <t>853375</t>
         </is>
       </c>
       <c r="AR2" s="1" t="inlineStr">
@@ -885,24 +883,24 @@
       </c>
       <c r="AS2" s="1" t="inlineStr">
         <is>
-          <t>Изотермический</t>
+          <t>Контейнеровоз</t>
         </is>
       </c>
       <c r="AT2" s="1" t="inlineStr"/>
       <c r="AU2" s="1" t="inlineStr"/>
       <c r="AV2" s="1" t="inlineStr">
         <is>
-          <t>WKVDAF10300124805</t>
+          <t>EAR853375R0000773</t>
         </is>
       </c>
       <c r="AW2" s="1" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="AX2" s="1" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AY2" s="1" t="inlineStr">
@@ -912,24 +910,20 @@
       </c>
       <c r="AZ2" s="1" t="inlineStr">
         <is>
-          <t>Барабанные</t>
+          <t>Дисковые</t>
         </is>
       </c>
       <c r="BA2" s="1" t="inlineStr">
         <is>
-          <t>31290</t>
+          <t>41000</t>
         </is>
       </c>
       <c r="BB2" s="1" t="inlineStr">
         <is>
-          <t>13700</t>
-        </is>
-      </c>
-      <c r="BC2" s="1" t="inlineStr">
-        <is>
-          <t>94</t>
-        </is>
-      </c>
+          <t>12600</t>
+        </is>
+      </c>
+      <c r="BC2" s="1" t="inlineStr"/>
       <c r="BD2" s="1" t="inlineStr"/>
       <c r="BE2" s="1" t="inlineStr"/>
     </row>
@@ -943,7 +937,7 @@
       <c r="C3" s="1" t="inlineStr"/>
       <c r="D3" s="1" t="inlineStr">
         <is>
-          <t>kassbohrer-maxima-shtor-00116344</t>
+          <t>kassbohrer-maxima-iso-xx246877</t>
         </is>
       </c>
       <c r="E3" s="1" t="inlineStr"/>
@@ -960,14 +954,13 @@
       </c>
       <c r="M3" s="1" t="inlineStr">
         <is>
-          <t>Полуприцеп шторный Kassbohrer Maxima, 2022 год выпуска, TIR-исполнение.
-Оси BPW, 3 шт., подвеска зависимая на продольных рычагах, тормоза барабанные. Шины бескамерные 385/65R22,5, односкат, Bridgestone.
-Масса снаряжённого полуприцепа 8 960 кг, грузоподъёмность 28 540 кг, разрешённая максимальная масса 37 500 кг.
-Внутренние размеры 16 520×2 480×2 700 мм, объём кузова 110,6 м³. Высота ССУ 1150 мм.
-Боковая обшивка из фанеры, пол — ламинированная фанера 27 мм.
+          <t>Полуприцеп изотермический Kassbohrer Maxima, 2023 год выпуска, TIR-исполнение.
+Оси BPW, 3 шт., подвеска пневматическая, тормоза барабанные.
+Грузоподъёмность 31 290 кг.
+Длина кузова 13,7 м, объём 94 м³.
 Техническое состояние — на ходу, полностью исправен, не требует вложений и ремонта.
 Документы в порядке.
-Возможна аренда с правом выкупа — уточняйте условия по телефону.
+Возможна аренда — уточняйте условия по телефону.
 Смотровая площадка и показ — по договорённости. Торг при осмотре.</t>
         </is>
       </c>
@@ -978,14 +971,14 @@
       </c>
       <c r="O3" s="1" t="inlineStr">
         <is>
-          <t>2890000</t>
+          <t>4850000</t>
         </is>
       </c>
       <c r="P3" s="1" t="inlineStr"/>
       <c r="Q3" s="1" t="inlineStr"/>
       <c r="R3" s="1" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00116344/01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00116344/02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00116344/03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00116344/04.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00116344/05.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00116344/06.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00116344/07.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00116344/08.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00116344/09.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00116344/10.jpg</t>
+          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-iso-xx246877/01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-iso-xx246877/02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-iso-xx246877/03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-iso-xx246877/04.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-iso-xx246877/05.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-iso-xx246877/06.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-iso-xx246877/07.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-iso-xx246877/08.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-iso-xx246877/09.jpg</t>
         </is>
       </c>
       <c r="S3" s="1" t="inlineStr"/>
@@ -1011,7 +1004,7 @@
       <c r="AA3" s="1" t="inlineStr"/>
       <c r="AB3" s="1" t="inlineStr">
         <is>
-          <t>2890000</t>
+          <t>4850000</t>
         </is>
       </c>
       <c r="AC3" s="1" t="inlineStr">
@@ -1056,19 +1049,19 @@
       </c>
       <c r="AS3" s="1" t="inlineStr">
         <is>
-          <t>Шторный</t>
+          <t>Изотермический</t>
         </is>
       </c>
       <c r="AT3" s="1" t="inlineStr"/>
       <c r="AU3" s="1" t="inlineStr"/>
       <c r="AV3" s="1" t="inlineStr">
         <is>
-          <t>WKVDAF30300116344</t>
+          <t>WKVDAF10300124805</t>
         </is>
       </c>
       <c r="AW3" s="1" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2023</t>
         </is>
       </c>
       <c r="AX3" s="1" t="inlineStr">
@@ -1078,7 +1071,7 @@
       </c>
       <c r="AY3" s="1" t="inlineStr">
         <is>
-          <t>Рессорная</t>
+          <t>Пневматическая</t>
         </is>
       </c>
       <c r="AZ3" s="1" t="inlineStr">
@@ -1088,17 +1081,17 @@
       </c>
       <c r="BA3" s="1" t="inlineStr">
         <is>
-          <t>28540</t>
+          <t>31290</t>
         </is>
       </c>
       <c r="BB3" s="1" t="inlineStr">
         <is>
-          <t>16520</t>
+          <t>13700</t>
         </is>
       </c>
       <c r="BC3" s="1" t="inlineStr">
         <is>
-          <t>110.6</t>
+          <t>94</t>
         </is>
       </c>
       <c r="BD3" s="1" t="inlineStr"/>
@@ -1114,7 +1107,7 @@
       <c r="C4" s="1" t="inlineStr"/>
       <c r="D4" s="1" t="inlineStr">
         <is>
-          <t>kassbohrer-maxima-shtor-00124397</t>
+          <t>kassbohrer-maxima-shtor-00116344</t>
         </is>
       </c>
       <c r="E4" s="1" t="inlineStr"/>
@@ -1131,7 +1124,7 @@
       </c>
       <c r="M4" s="1" t="inlineStr">
         <is>
-          <t>Полуприцеп шторный Kassbohrer Maxima, 2023 год выпуска, TIR-исполнение.
+          <t>Полуприцеп шторный Kassbohrer Maxima, 2022 год выпуска, TIR-исполнение.
 Оси BPW, 3 шт., подвеска зависимая на продольных рычагах, тормоза барабанные. Шины бескамерные 385/65R22,5, односкат, Bridgestone.
 Масса снаряжённого полуприцепа 8 960 кг, грузоподъёмность 28 540 кг, разрешённая максимальная масса 37 500 кг.
 Внутренние размеры 16 520×2 480×2 700 мм, объём кузова 110,6 м³. Высота ССУ 1150 мм.
@@ -1149,14 +1142,14 @@
       </c>
       <c r="O4" s="1" t="inlineStr">
         <is>
-          <t>3290000</t>
+          <t>2890000</t>
         </is>
       </c>
       <c r="P4" s="1" t="inlineStr"/>
       <c r="Q4" s="1" t="inlineStr"/>
       <c r="R4" s="1" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124397/01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124397/02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124397/03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124397/04.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124397/05.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124397/06.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124397/07.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124397/08.jpg</t>
+          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00116344/01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00116344/02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00116344/03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00116344/04.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00116344/05.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00116344/06.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00116344/07.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00116344/08.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00116344/09.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00116344/10.jpg</t>
         </is>
       </c>
       <c r="S4" s="1" t="inlineStr"/>
@@ -1182,7 +1175,7 @@
       <c r="AA4" s="1" t="inlineStr"/>
       <c r="AB4" s="1" t="inlineStr">
         <is>
-          <t>3290000</t>
+          <t>2890000</t>
         </is>
       </c>
       <c r="AC4" s="1" t="inlineStr">
@@ -1234,12 +1227,12 @@
       <c r="AU4" s="1" t="inlineStr"/>
       <c r="AV4" s="1" t="inlineStr">
         <is>
-          <t>WKVDAF30300124397</t>
+          <t>WKVDAF30300116344</t>
         </is>
       </c>
       <c r="AW4" s="1" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="AX4" s="1" t="inlineStr">
@@ -1285,7 +1278,7 @@
       <c r="C5" s="1" t="inlineStr"/>
       <c r="D5" s="1" t="inlineStr">
         <is>
-          <t>kassbohrer-maxima-shtor-00124732</t>
+          <t>kassbohrer-maxima-shtor-00124397</t>
         </is>
       </c>
       <c r="E5" s="1" t="inlineStr"/>
@@ -1302,11 +1295,11 @@
       </c>
       <c r="M5" s="1" t="inlineStr">
         <is>
-          <t>Полуприцеп шторный Kassbohrer, 2023 год выпуска, TIR-исполнение.
-Оси BPW, 3 шт., подвеска рессорная, тормоза барабанные. Шины бескамерные 385/65R22,5, односкат, Bridgestone.
-Масса снаряжённого 7 630 кг, грузоподъёмность 28 540 кг, разрешённая максимальная масса 39 000 кг.
-Внутренние размеры 13 600×2 480×2 700 мм, объём кузова 92 м³. Высота ССУ 1150 мм.
-Боковая обшивка из фанеры, пол — ламинированная фанера 30 мм.
+          <t>Полуприцеп шторный Kassbohrer Maxima, 2023 год выпуска, TIR-исполнение.
+Оси BPW, 3 шт., подвеска зависимая на продольных рычагах, тормоза барабанные. Шины бескамерные 385/65R22,5, односкат, Bridgestone.
+Масса снаряжённого полуприцепа 8 960 кг, грузоподъёмность 28 540 кг, разрешённая максимальная масса 37 500 кг.
+Внутренние размеры 16 520×2 480×2 700 мм, объём кузова 110,6 м³. Высота ССУ 1150 мм.
+Боковая обшивка из фанеры, пол — ламинированная фанера 27 мм.
 Техническое состояние — на ходу, полностью исправен, не требует вложений и ремонта.
 Документы в порядке.
 Возможна аренда с правом выкупа — уточняйте условия по телефону.
@@ -1320,14 +1313,14 @@
       </c>
       <c r="O5" s="1" t="inlineStr">
         <is>
-          <t>2890000</t>
+          <t>3290000</t>
         </is>
       </c>
       <c r="P5" s="1" t="inlineStr"/>
       <c r="Q5" s="1" t="inlineStr"/>
       <c r="R5" s="1" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124732/01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124732/02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124732/03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124732/04.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124732/05.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124732/06.jpg</t>
+          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124397/01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124397/02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124397/03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124397/04.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124397/05.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124397/06.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124397/07.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124397/08.jpg</t>
         </is>
       </c>
       <c r="S5" s="1" t="inlineStr"/>
@@ -1353,7 +1346,7 @@
       <c r="AA5" s="1" t="inlineStr"/>
       <c r="AB5" s="1" t="inlineStr">
         <is>
-          <t>2890000</t>
+          <t>3290000</t>
         </is>
       </c>
       <c r="AC5" s="1" t="inlineStr">
@@ -1405,7 +1398,7 @@
       <c r="AU5" s="1" t="inlineStr"/>
       <c r="AV5" s="1" t="inlineStr">
         <is>
-          <t>WKVDAF30300124732</t>
+          <t>WKVDAF30300124397</t>
         </is>
       </c>
       <c r="AW5" s="1" t="inlineStr">
@@ -1435,12 +1428,12 @@
       </c>
       <c r="BB5" s="1" t="inlineStr">
         <is>
-          <t>13600</t>
+          <t>16520</t>
         </is>
       </c>
       <c r="BC5" s="1" t="inlineStr">
         <is>
-          <t>92</t>
+          <t>110.6</t>
         </is>
       </c>
       <c r="BD5" s="1" t="inlineStr"/>
@@ -1456,7 +1449,7 @@
       <c r="C6" s="1" t="inlineStr"/>
       <c r="D6" s="1" t="inlineStr">
         <is>
-          <t>steelbear-pl24l-ea653666</t>
+          <t>kassbohrer-maxima-shtor-00124732</t>
         </is>
       </c>
       <c r="E6" s="1" t="inlineStr"/>
@@ -1473,12 +1466,15 @@
       </c>
       <c r="M6" s="1" t="inlineStr">
         <is>
-          <t>Полуприцеп-сортиментовоз Steelbear PL-24L (коммерческое название PT-24L BPW Heavy Duty), 2024 год выпуска, под заказ.
-Усиленное шасси из двутавровых лонжеронов, 3 оси BPW Heavy Duty, барабанные тормоза, пневмоподвеска с функцией подъём/опускание, допустимая нагрузка на ось 9 000 кг. Шины 385/65R22,5, односкат. Электронная тормозная система WABCO TEBS-E с функцией противоопрокидывания (RSS).
-6 пар открепляемых коников грузоподъёмностью 8 тонн каждая (сталь STRENX 700MC), положение регулируется вдоль рамы. Внутренняя высота коника 2330 мм. Настил из ламинированной берёзовой фанеры. Опорное устройство BPW, 24 т.
-Максимальная полная масса 44 000 кг, грузоподъёмность 37 100 кг, длина 13 620 мм.
-Заводская гарантия — 24 месяца, от сквозной коррозии — 10 лет.
-Поставка под заказ, срок — уточняйте.</t>
+          <t>Полуприцеп шторный Kassbohrer, 2023 год выпуска, TIR-исполнение.
+Оси BPW, 3 шт., подвеска рессорная, тормоза барабанные. Шины бескамерные 385/65R22,5, односкат, Bridgestone.
+Масса снаряжённого 7 630 кг, грузоподъёмность 28 540 кг, разрешённая максимальная масса 39 000 кг.
+Внутренние размеры 13 600×2 480×2 700 мм, объём кузова 92 м³. Высота ССУ 1150 мм.
+Боковая обшивка из фанеры, пол — ламинированная фанера 30 мм.
+Техническое состояние — на ходу, полностью исправен, не требует вложений и ремонта.
+Документы в порядке.
+Возможна аренда с правом выкупа — уточняйте условия по телефону.
+Смотровая площадка и показ — по договорённости. Торг при осмотре.</t>
         </is>
       </c>
       <c r="N6" s="1" t="inlineStr">
@@ -1488,14 +1484,14 @@
       </c>
       <c r="O6" s="1" t="inlineStr">
         <is>
-          <t>2970000</t>
+          <t>2890000</t>
         </is>
       </c>
       <c r="P6" s="1" t="inlineStr"/>
       <c r="Q6" s="1" t="inlineStr"/>
       <c r="R6" s="1" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/04.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/05.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/06.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/07.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/08.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/09.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/10.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/11.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/12.jpg</t>
+          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124732/01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124732/02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124732/03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124732/04.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124732/05.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124732/06.jpg</t>
         </is>
       </c>
       <c r="S6" s="1" t="inlineStr"/>
@@ -1521,12 +1517,12 @@
       <c r="AA6" s="1" t="inlineStr"/>
       <c r="AB6" s="1" t="inlineStr">
         <is>
-          <t>2970000</t>
+          <t>2890000</t>
         </is>
       </c>
       <c r="AC6" s="1" t="inlineStr">
         <is>
-          <t>Под заказ</t>
+          <t>В наличии</t>
         </is>
       </c>
       <c r="AD6" s="1" t="inlineStr"/>
@@ -1551,12 +1547,12 @@
       </c>
       <c r="AP6" s="1" t="inlineStr">
         <is>
-          <t>Steelbear</t>
+          <t>Kassbohrer</t>
         </is>
       </c>
       <c r="AQ6" s="1" t="inlineStr">
         <is>
-          <t>PL-24L</t>
+          <t>Maxima</t>
         </is>
       </c>
       <c r="AR6" s="1" t="inlineStr">
@@ -1566,15 +1562,19 @@
       </c>
       <c r="AS6" s="1" t="inlineStr">
         <is>
-          <t>Лесовоз (сортиментовоз)</t>
+          <t>Шторный</t>
         </is>
       </c>
       <c r="AT6" s="1" t="inlineStr"/>
       <c r="AU6" s="1" t="inlineStr"/>
-      <c r="AV6" s="1" t="inlineStr"/>
+      <c r="AV6" s="1" t="inlineStr">
+        <is>
+          <t>WKVDAF30300124732</t>
+        </is>
+      </c>
       <c r="AW6" s="1" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2023</t>
         </is>
       </c>
       <c r="AX6" s="1" t="inlineStr">
@@ -1584,7 +1584,7 @@
       </c>
       <c r="AY6" s="1" t="inlineStr">
         <is>
-          <t>Пневматическая</t>
+          <t>Рессорная</t>
         </is>
       </c>
       <c r="AZ6" s="1" t="inlineStr">
@@ -1594,15 +1594,19 @@
       </c>
       <c r="BA6" s="1" t="inlineStr">
         <is>
-          <t>37100</t>
+          <t>28540</t>
         </is>
       </c>
       <c r="BB6" s="1" t="inlineStr">
         <is>
-          <t>13620</t>
-        </is>
-      </c>
-      <c r="BC6" s="1" t="inlineStr"/>
+          <t>13600</t>
+        </is>
+      </c>
+      <c r="BC6" s="1" t="inlineStr">
+        <is>
+          <t>92</t>
+        </is>
+      </c>
       <c r="BD6" s="1" t="inlineStr"/>
       <c r="BE6" s="1" t="inlineStr"/>
     </row>
@@ -1616,7 +1620,7 @@
       <c r="C7" s="1" t="inlineStr"/>
       <c r="D7" s="1" t="inlineStr">
         <is>
-          <t>v-trailer-329d-r0000119</t>
+          <t>steelbear-pl24l-ea653666</t>
         </is>
       </c>
       <c r="E7" s="1" t="inlineStr"/>
@@ -1633,11 +1637,12 @@
       </c>
       <c r="M7" s="1" t="inlineStr">
         <is>
-          <t>Шторный полуприцеп V-Trailer 329D, 2023 год, в работе, полностью исправен.
-Оси SAF, подъёмная передняя — меньше износ резины и расход на порожняке. Опорное устройство JOST на 24 тонны, шкворень 2 дюйма по ISO 1726. Пол — влагостойкая фанера 30 мм, держит погрузчик до 7,5 тонн. Крыша сдвижная (Sesam/Edscha) — грузить сверху краном или погрузчиком без снятия тента. Двери алюминиевые BPW Smartmaster II, передний и задний портал — стальные, собственной конструкции. Рама облегчённая, с дополнительными усилениями против скручивания. По бортам — корзины под коники, по 7 штук на сторону.
-13,6 × 2,5 × 4 м, 91 м³. Тент плотный: борта 900 г/м², крыша 680 г/м². Полная штора, без бортов — удобно под европаллеты и груз с выступом по высоте.
-VIN XZFVKRP3DR0000119.
-Возможна аренда с правом выкупа — уточняйте условия по телефону.</t>
+          <t>Полуприцеп-сортиментовоз Steelbear PL-24L (коммерческое название PT-24L BPW Heavy Duty), 2024 год выпуска, под заказ.
+Усиленное шасси из двутавровых лонжеронов, 3 оси BPW Heavy Duty, барабанные тормоза, пневмоподвеска с функцией подъём/опускание, допустимая нагрузка на ось 9 000 кг. Шины 385/65R22,5, односкат. Электронная тормозная система WABCO TEBS-E с функцией противоопрокидывания (RSS).
+6 пар открепляемых коников грузоподъёмностью 8 тонн каждая (сталь STRENX 700MC), положение регулируется вдоль рамы. Внутренняя высота коника 2330 мм. Настил из ламинированной берёзовой фанеры. Опорное устройство BPW, 24 т.
+Максимальная полная масса 44 000 кг, грузоподъёмность 37 100 кг, длина 13 620 мм.
+Заводская гарантия — 24 месяца, от сквозной коррозии — 10 лет.
+Поставка под заказ, срок — уточняйте.</t>
         </is>
       </c>
       <c r="N7" s="1" t="inlineStr">
@@ -1647,14 +1652,14 @@
       </c>
       <c r="O7" s="1" t="inlineStr">
         <is>
-          <t>2990000</t>
+          <t>2970000</t>
         </is>
       </c>
       <c r="P7" s="1" t="inlineStr"/>
       <c r="Q7" s="1" t="inlineStr"/>
       <c r="R7" s="1" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/04.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/05.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/06.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/07.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/08.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/09.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/10.jpg</t>
+          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/04.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/05.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/06.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/07.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/08.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/09.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/10.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/11.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/12.jpg</t>
         </is>
       </c>
       <c r="S7" s="1" t="inlineStr"/>
@@ -1680,12 +1685,12 @@
       <c r="AA7" s="1" t="inlineStr"/>
       <c r="AB7" s="1" t="inlineStr">
         <is>
-          <t>2990000</t>
+          <t>2970000</t>
         </is>
       </c>
       <c r="AC7" s="1" t="inlineStr">
         <is>
-          <t>В наличии</t>
+          <t>Под заказ</t>
         </is>
       </c>
       <c r="AD7" s="1" t="inlineStr"/>
@@ -1710,12 +1715,12 @@
       </c>
       <c r="AP7" s="1" t="inlineStr">
         <is>
-          <t>V-Trailer</t>
+          <t>Steelbear</t>
         </is>
       </c>
       <c r="AQ7" s="1" t="inlineStr">
         <is>
-          <t>329D</t>
+          <t>PL-24L</t>
         </is>
       </c>
       <c r="AR7" s="1" t="inlineStr">
@@ -1725,19 +1730,15 @@
       </c>
       <c r="AS7" s="1" t="inlineStr">
         <is>
-          <t>Шторный</t>
+          <t>Лесовоз (сортиментовоз)</t>
         </is>
       </c>
       <c r="AT7" s="1" t="inlineStr"/>
       <c r="AU7" s="1" t="inlineStr"/>
-      <c r="AV7" s="1" t="inlineStr">
-        <is>
-          <t>XZFVKRP3DR0000119</t>
-        </is>
-      </c>
+      <c r="AV7" s="1" t="inlineStr"/>
       <c r="AW7" s="1" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="AX7" s="1" t="inlineStr">
@@ -1752,26 +1753,189 @@
       </c>
       <c r="AZ7" s="1" t="inlineStr">
         <is>
-          <t>Дисковые</t>
+          <t>Барабанные</t>
         </is>
       </c>
       <c r="BA7" s="1" t="inlineStr">
         <is>
-          <t>32300</t>
+          <t>37100</t>
         </is>
       </c>
       <c r="BB7" s="1" t="inlineStr">
         <is>
-          <t>13600</t>
-        </is>
-      </c>
-      <c r="BC7" s="1" t="inlineStr">
-        <is>
-          <t>91</t>
-        </is>
-      </c>
+          <t>13620</t>
+        </is>
+      </c>
+      <c r="BC7" s="1" t="inlineStr"/>
       <c r="BD7" s="1" t="inlineStr"/>
       <c r="BE7" s="1" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>Москва, Ижорская ул., 15с2</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="inlineStr"/>
+      <c r="C8" s="1" t="inlineStr"/>
+      <c r="D8" s="1" t="inlineStr">
+        <is>
+          <t>v-trailer-329d-r0000119</t>
+        </is>
+      </c>
+      <c r="E8" s="1" t="inlineStr"/>
+      <c r="F8" s="1" t="inlineStr"/>
+      <c r="G8" s="1" t="inlineStr"/>
+      <c r="H8" s="1" t="inlineStr"/>
+      <c r="I8" s="1" t="inlineStr"/>
+      <c r="J8" s="1" t="inlineStr"/>
+      <c r="K8" s="1" t="inlineStr"/>
+      <c r="L8" s="1" t="inlineStr">
+        <is>
+          <t>По телефону и в сообщениях</t>
+        </is>
+      </c>
+      <c r="M8" s="1" t="inlineStr">
+        <is>
+          <t>Шторный полуприцеп V-Trailer 329D, 2023 год, в работе, полностью исправен.
+Оси SAF, подъёмная передняя — меньше износ резины и расход на порожняке. Опорное устройство JOST на 24 тонны, шкворень 2 дюйма по ISO 1726. Пол — влагостойкая фанера 30 мм, держит погрузчик до 7,5 тонн. Крыша сдвижная (Sesam/Edscha) — грузить сверху краном или погрузчиком без снятия тента. Двери алюминиевые BPW Smartmaster II, передний и задний портал — стальные, собственной конструкции. Рама облегчённая, с дополнительными усилениями против скручивания. По бортам — корзины под коники, по 7 штук на сторону.
+13,6 × 2,5 × 4 м, 91 м³. Тент плотный: борта 900 г/м², крыша 680 г/м². Полная штора, без бортов — удобно под европаллеты и груз с выступом по высоте.
+VIN XZFVKRP3DR0000119.
+Возможна аренда с правом выкупа — уточняйте условия по телефону.</t>
+        </is>
+      </c>
+      <c r="N8" s="1" t="inlineStr">
+        <is>
+          <t>Грузовики и спецтехника</t>
+        </is>
+      </c>
+      <c r="O8" s="1" t="inlineStr">
+        <is>
+          <t>2990000</t>
+        </is>
+      </c>
+      <c r="P8" s="1" t="inlineStr"/>
+      <c r="Q8" s="1" t="inlineStr"/>
+      <c r="R8" s="1" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/04.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/05.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/06.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/07.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/08.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/09.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/10.jpg</t>
+        </is>
+      </c>
+      <c r="S8" s="1" t="inlineStr"/>
+      <c r="T8" s="1" t="inlineStr"/>
+      <c r="U8" s="1" t="inlineStr"/>
+      <c r="V8" s="1" t="inlineStr"/>
+      <c r="W8" s="1" t="inlineStr"/>
+      <c r="X8" s="1" t="inlineStr">
+        <is>
+          <t>Прицепы</t>
+        </is>
+      </c>
+      <c r="Y8" s="1" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="Z8" s="1" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="AA8" s="1" t="inlineStr"/>
+      <c r="AB8" s="1" t="inlineStr">
+        <is>
+          <t>2990000</t>
+        </is>
+      </c>
+      <c r="AC8" s="1" t="inlineStr">
+        <is>
+          <t>В наличии</t>
+        </is>
+      </c>
+      <c r="AD8" s="1" t="inlineStr"/>
+      <c r="AE8" s="1" t="inlineStr"/>
+      <c r="AF8" s="1" t="inlineStr"/>
+      <c r="AG8" s="1" t="inlineStr"/>
+      <c r="AH8" s="1" t="inlineStr"/>
+      <c r="AI8" s="1" t="inlineStr"/>
+      <c r="AJ8" s="1" t="inlineStr"/>
+      <c r="AK8" s="1" t="inlineStr"/>
+      <c r="AL8" s="1" t="inlineStr"/>
+      <c r="AM8" s="1" t="inlineStr">
+        <is>
+          <t>С пробегом</t>
+        </is>
+      </c>
+      <c r="AN8" s="1" t="inlineStr"/>
+      <c r="AO8" s="1" t="inlineStr">
+        <is>
+          <t>В наличии</t>
+        </is>
+      </c>
+      <c r="AP8" s="1" t="inlineStr">
+        <is>
+          <t>V-Trailer</t>
+        </is>
+      </c>
+      <c r="AQ8" s="1" t="inlineStr">
+        <is>
+          <t>329D</t>
+        </is>
+      </c>
+      <c r="AR8" s="1" t="inlineStr">
+        <is>
+          <t>Полуприцеп</t>
+        </is>
+      </c>
+      <c r="AS8" s="1" t="inlineStr">
+        <is>
+          <t>Шторный</t>
+        </is>
+      </c>
+      <c r="AT8" s="1" t="inlineStr"/>
+      <c r="AU8" s="1" t="inlineStr"/>
+      <c r="AV8" s="1" t="inlineStr">
+        <is>
+          <t>XZFVKRP3DR0000119</t>
+        </is>
+      </c>
+      <c r="AW8" s="1" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="AX8" s="1" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AY8" s="1" t="inlineStr">
+        <is>
+          <t>Пневматическая</t>
+        </is>
+      </c>
+      <c r="AZ8" s="1" t="inlineStr">
+        <is>
+          <t>Дисковые</t>
+        </is>
+      </c>
+      <c r="BA8" s="1" t="inlineStr">
+        <is>
+          <t>32300</t>
+        </is>
+      </c>
+      <c r="BB8" s="1" t="inlineStr">
+        <is>
+          <t>13600</t>
+        </is>
+      </c>
+      <c r="BC8" s="1" t="inlineStr">
+        <is>
+          <t>91</t>
+        </is>
+      </c>
+      <c r="BD8" s="1" t="inlineStr"/>
+      <c r="BE8" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add Tonar K4-U (99891) container chassis (2023, VIN X0T998910P0002033)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019CenkzpMJCXcxKtoErKpEq
</commit_message>
<xml_diff>
--- a/avito-feed-trailers/fleet-trailers.xlsx
+++ b/avito-feed-trailers/fleet-trailers.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BE8"/>
+  <dimension ref="A1:BE9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -459,7 +459,7 @@
     <col width="10" customWidth="1" min="40" max="40"/>
     <col width="13" customWidth="1" min="41" max="41"/>
     <col width="13" customWidth="1" min="42" max="42"/>
-    <col width="10" customWidth="1" min="43" max="43"/>
+    <col width="14" customWidth="1" min="43" max="43"/>
     <col width="13" customWidth="1" min="44" max="44"/>
     <col width="25" customWidth="1" min="45" max="45"/>
     <col width="11" customWidth="1" min="46" max="46"/>
@@ -1780,7 +1780,7 @@
       <c r="C8" s="1" t="inlineStr"/>
       <c r="D8" s="1" t="inlineStr">
         <is>
-          <t>v-trailer-329d-r0000119</t>
+          <t>tonar-k4u-p0002033</t>
         </is>
       </c>
       <c r="E8" s="1" t="inlineStr"/>
@@ -1797,10 +1797,10 @@
       </c>
       <c r="M8" s="1" t="inlineStr">
         <is>
-          <t>Шторный полуприцеп V-Trailer 329D, 2023 год, в работе, полностью исправен.
-Оси SAF, подъёмная передняя — меньше износ резины и расход на порожняке. Опорное устройство JOST на 24 тонны, шкворень 2 дюйма по ISO 1726. Пол — влагостойкая фанера 30 мм, держит погрузчик до 7,5 тонн. Крыша сдвижная (Sesam/Edscha) — грузить сверху краном или погрузчиком без снятия тента. Двери алюминиевые BPW Smartmaster II, передний и задний портал — стальные, собственной конструкции. Рама облегчённая, с дополнительными усилениями против скручивания. По бортам — корзины под коники, по 7 штук на сторону.
-13,6 × 2,5 × 4 м, 91 м³. Тент плотный: борта 900 г/м², крыша 680 г/м². Полная штора, без бортов — удобно под европаллеты и груз с выступом по высоте.
-VIN XZFVKRP3DR0000119.
+          <t>Полуприцеп-контейнеровоз Тонар К4-U (99891), 2023 год, в работе, полностью исправен.
+4 оси: тройная задняя тележка плюс вынесенная вперёд ось — меньше нагрузка на дорогу и мягче по осевым ограничениям в городе. Тормоза дисковые, пневмопривод. Подвеска зависимая, на продольных рычагах, с пневмоэлементами и телескопическими амортизаторами. Шины 385/55R22.5, односкатные.
+Берёт контейнеры 20', 2×20', 30', 30' HC, 40', 40' HC. Разрешённая максимальная масса 44 000 кг, грузоподъёмность 37 800 кг, нагрузка на ССУ 11 000 кг. Высота ССУ 1 100 мм.
+VIN X0T998910P0002033.
 Возможна аренда с правом выкупа — уточняйте условия по телефону.</t>
         </is>
       </c>
@@ -1811,14 +1811,14 @@
       </c>
       <c r="O8" s="1" t="inlineStr">
         <is>
-          <t>2990000</t>
+          <t>1690000</t>
         </is>
       </c>
       <c r="P8" s="1" t="inlineStr"/>
       <c r="Q8" s="1" t="inlineStr"/>
       <c r="R8" s="1" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/04.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/05.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/06.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/07.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/08.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/09.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/10.jpg</t>
+          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-p0002033/01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-p0002033/02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-p0002033/03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-p0002033/04.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-p0002033/05.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-p0002033/06.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-p0002033/07.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-p0002033/08.jpg</t>
         </is>
       </c>
       <c r="S8" s="1" t="inlineStr"/>
@@ -1844,7 +1844,7 @@
       <c r="AA8" s="1" t="inlineStr"/>
       <c r="AB8" s="1" t="inlineStr">
         <is>
-          <t>2990000</t>
+          <t>1690000</t>
         </is>
       </c>
       <c r="AC8" s="1" t="inlineStr">
@@ -1874,12 +1874,12 @@
       </c>
       <c r="AP8" s="1" t="inlineStr">
         <is>
-          <t>V-Trailer</t>
+          <t>Тонар</t>
         </is>
       </c>
       <c r="AQ8" s="1" t="inlineStr">
         <is>
-          <t>329D</t>
+          <t>K4-U (99891)</t>
         </is>
       </c>
       <c r="AR8" s="1" t="inlineStr">
@@ -1889,14 +1889,14 @@
       </c>
       <c r="AS8" s="1" t="inlineStr">
         <is>
-          <t>Шторный</t>
+          <t>Контейнеровоз</t>
         </is>
       </c>
       <c r="AT8" s="1" t="inlineStr"/>
       <c r="AU8" s="1" t="inlineStr"/>
       <c r="AV8" s="1" t="inlineStr">
         <is>
-          <t>XZFVKRP3DR0000119</t>
+          <t>X0T998910P0002033</t>
         </is>
       </c>
       <c r="AW8" s="1" t="inlineStr">
@@ -1906,12 +1906,12 @@
       </c>
       <c r="AX8" s="1" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AY8" s="1" t="inlineStr">
         <is>
-          <t>Пневматическая</t>
+          <t>Рессорная</t>
         </is>
       </c>
       <c r="AZ8" s="1" t="inlineStr">
@@ -1921,21 +1921,184 @@
       </c>
       <c r="BA8" s="1" t="inlineStr">
         <is>
-          <t>32300</t>
+          <t>37800</t>
         </is>
       </c>
       <c r="BB8" s="1" t="inlineStr">
         <is>
-          <t>13600</t>
-        </is>
-      </c>
-      <c r="BC8" s="1" t="inlineStr">
-        <is>
-          <t>91</t>
-        </is>
-      </c>
+          <t>12725</t>
+        </is>
+      </c>
+      <c r="BC8" s="1" t="inlineStr"/>
       <c r="BD8" s="1" t="inlineStr"/>
       <c r="BE8" s="1" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>Москва, Ижорская ул., 15с2</t>
+        </is>
+      </c>
+      <c r="B9" s="1" t="inlineStr"/>
+      <c r="C9" s="1" t="inlineStr"/>
+      <c r="D9" s="1" t="inlineStr">
+        <is>
+          <t>v-trailer-329d-r0000119</t>
+        </is>
+      </c>
+      <c r="E9" s="1" t="inlineStr"/>
+      <c r="F9" s="1" t="inlineStr"/>
+      <c r="G9" s="1" t="inlineStr"/>
+      <c r="H9" s="1" t="inlineStr"/>
+      <c r="I9" s="1" t="inlineStr"/>
+      <c r="J9" s="1" t="inlineStr"/>
+      <c r="K9" s="1" t="inlineStr"/>
+      <c r="L9" s="1" t="inlineStr">
+        <is>
+          <t>По телефону и в сообщениях</t>
+        </is>
+      </c>
+      <c r="M9" s="1" t="inlineStr">
+        <is>
+          <t>Шторный полуприцеп V-Trailer 329D, 2023 год, в работе, полностью исправен.
+Оси SAF, подъёмная передняя — меньше износ резины и расход на порожняке. Опорное устройство JOST на 24 тонны, шкворень 2 дюйма по ISO 1726. Пол — влагостойкая фанера 30 мм, держит погрузчик до 7,5 тонн. Крыша сдвижная (Sesam/Edscha) — грузить сверху краном или погрузчиком без снятия тента. Двери алюминиевые BPW Smartmaster II, передний и задний портал — стальные, собственной конструкции. Рама облегчённая, с дополнительными усилениями против скручивания. По бортам — корзины под коники, по 7 штук на сторону.
+13,6 × 2,5 × 4 м, 91 м³. Тент плотный: борта 900 г/м², крыша 680 г/м². Полная штора, без бортов — удобно под европаллеты и груз с выступом по высоте.
+VIN XZFVKRP3DR0000119.
+Возможна аренда с правом выкупа — уточняйте условия по телефону.</t>
+        </is>
+      </c>
+      <c r="N9" s="1" t="inlineStr">
+        <is>
+          <t>Грузовики и спецтехника</t>
+        </is>
+      </c>
+      <c r="O9" s="1" t="inlineStr">
+        <is>
+          <t>2990000</t>
+        </is>
+      </c>
+      <c r="P9" s="1" t="inlineStr"/>
+      <c r="Q9" s="1" t="inlineStr"/>
+      <c r="R9" s="1" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/04.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/05.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/06.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/07.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/08.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/09.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/10.jpg</t>
+        </is>
+      </c>
+      <c r="S9" s="1" t="inlineStr"/>
+      <c r="T9" s="1" t="inlineStr"/>
+      <c r="U9" s="1" t="inlineStr"/>
+      <c r="V9" s="1" t="inlineStr"/>
+      <c r="W9" s="1" t="inlineStr"/>
+      <c r="X9" s="1" t="inlineStr">
+        <is>
+          <t>Прицепы</t>
+        </is>
+      </c>
+      <c r="Y9" s="1" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="Z9" s="1" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="AA9" s="1" t="inlineStr"/>
+      <c r="AB9" s="1" t="inlineStr">
+        <is>
+          <t>2990000</t>
+        </is>
+      </c>
+      <c r="AC9" s="1" t="inlineStr">
+        <is>
+          <t>В наличии</t>
+        </is>
+      </c>
+      <c r="AD9" s="1" t="inlineStr"/>
+      <c r="AE9" s="1" t="inlineStr"/>
+      <c r="AF9" s="1" t="inlineStr"/>
+      <c r="AG9" s="1" t="inlineStr"/>
+      <c r="AH9" s="1" t="inlineStr"/>
+      <c r="AI9" s="1" t="inlineStr"/>
+      <c r="AJ9" s="1" t="inlineStr"/>
+      <c r="AK9" s="1" t="inlineStr"/>
+      <c r="AL9" s="1" t="inlineStr"/>
+      <c r="AM9" s="1" t="inlineStr">
+        <is>
+          <t>С пробегом</t>
+        </is>
+      </c>
+      <c r="AN9" s="1" t="inlineStr"/>
+      <c r="AO9" s="1" t="inlineStr">
+        <is>
+          <t>В наличии</t>
+        </is>
+      </c>
+      <c r="AP9" s="1" t="inlineStr">
+        <is>
+          <t>V-Trailer</t>
+        </is>
+      </c>
+      <c r="AQ9" s="1" t="inlineStr">
+        <is>
+          <t>329D</t>
+        </is>
+      </c>
+      <c r="AR9" s="1" t="inlineStr">
+        <is>
+          <t>Полуприцеп</t>
+        </is>
+      </c>
+      <c r="AS9" s="1" t="inlineStr">
+        <is>
+          <t>Шторный</t>
+        </is>
+      </c>
+      <c r="AT9" s="1" t="inlineStr"/>
+      <c r="AU9" s="1" t="inlineStr"/>
+      <c r="AV9" s="1" t="inlineStr">
+        <is>
+          <t>XZFVKRP3DR0000119</t>
+        </is>
+      </c>
+      <c r="AW9" s="1" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="AX9" s="1" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AY9" s="1" t="inlineStr">
+        <is>
+          <t>Пневматическая</t>
+        </is>
+      </c>
+      <c r="AZ9" s="1" t="inlineStr">
+        <is>
+          <t>Дисковые</t>
+        </is>
+      </c>
+      <c r="BA9" s="1" t="inlineStr">
+        <is>
+          <t>32300</t>
+        </is>
+      </c>
+      <c r="BB9" s="1" t="inlineStr">
+        <is>
+          <t>13600</t>
+        </is>
+      </c>
+      <c r="BC9" s="1" t="inlineStr">
+        <is>
+          <t>91</t>
+        </is>
+      </c>
+      <c r="BD9" s="1" t="inlineStr"/>
+      <c r="BE9" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Fix Kassbohrer Maxima 16.5m curtain trailers: correct photos, disc brakes
Both 2022 (VIN ...6344) and 2023 (VIN ...4397) units were listed with
isothermal-looking photos despite trailer_type already being "Шторный" in
the feed data. Replaced with real curtain-side photos from the same set
(only set available), different order per unit. Also corrected brakes
from Барабанные to Дисковые per real spec check.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WGw8UdFgVU8PXaQaPUvEwH
</commit_message>
<xml_diff>
--- a/avito-feed-trailers/fleet-trailers.xlsx
+++ b/avito-feed-trailers/fleet-trailers.xlsx
@@ -1125,7 +1125,7 @@
       <c r="M4" s="1" t="inlineStr">
         <is>
           <t>Полуприцеп шторный Kassbohrer Maxima, 2022 год выпуска, TIR-исполнение.
-Оси BPW, 3 шт., подвеска зависимая на продольных рычагах, тормоза барабанные. Шины бескамерные 385/65R22,5, односкат, Bridgestone.
+Оси BPW, 3 шт., подвеска зависимая на продольных рычагах, тормоза дисковые. Шины бескамерные 385/65R22,5, односкат, Bridgestone.
 Масса снаряжённого полуприцепа 8 960 кг, грузоподъёмность 28 540 кг, разрешённая максимальная масса 37 500 кг.
 Внутренние размеры 16 520×2 480×2 700 мм, объём кузова 110,6 м³. Высота ССУ 1150 мм.
 Боковая обшивка из фанеры, пол — ламинированная фанера 27 мм.
@@ -1149,7 +1149,7 @@
       <c r="Q4" s="1" t="inlineStr"/>
       <c r="R4" s="1" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00116344/01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00116344/02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00116344/03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00116344/04.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00116344/05.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00116344/06.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00116344/07.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00116344/08.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00116344/09.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00116344/10.jpg</t>
+          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00116344/01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00116344/02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00116344/03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00116344/04.jpg</t>
         </is>
       </c>
       <c r="S4" s="1" t="inlineStr"/>
@@ -1247,7 +1247,7 @@
       </c>
       <c r="AZ4" s="1" t="inlineStr">
         <is>
-          <t>Барабанные</t>
+          <t>Дисковые</t>
         </is>
       </c>
       <c r="BA4" s="1" t="inlineStr">
@@ -1296,7 +1296,7 @@
       <c r="M5" s="1" t="inlineStr">
         <is>
           <t>Полуприцеп шторный Kassbohrer Maxima, 2023 год выпуска, TIR-исполнение.
-Оси BPW, 3 шт., подвеска зависимая на продольных рычагах, тормоза барабанные. Шины бескамерные 385/65R22,5, односкат, Bridgestone.
+Оси BPW, 3 шт., подвеска зависимая на продольных рычагах, тормоза дисковые. Шины бескамерные 385/65R22,5, односкат, Bridgestone.
 Масса снаряжённого полуприцепа 8 960 кг, грузоподъёмность 28 540 кг, разрешённая максимальная масса 37 500 кг.
 Внутренние размеры 16 520×2 480×2 700 мм, объём кузова 110,6 м³. Высота ССУ 1150 мм.
 Боковая обшивка из фанеры, пол — ламинированная фанера 27 мм.
@@ -1320,7 +1320,7 @@
       <c r="Q5" s="1" t="inlineStr"/>
       <c r="R5" s="1" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124397/01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124397/02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124397/03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124397/04.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124397/05.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124397/06.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124397/07.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124397/08.jpg</t>
+          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124397/01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124397/02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124397/03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124397/04.jpg</t>
         </is>
       </c>
       <c r="S5" s="1" t="inlineStr"/>
@@ -1418,7 +1418,7 @@
       </c>
       <c r="AZ5" s="1" t="inlineStr">
         <is>
-          <t>Барабанные</t>
+          <t>Дисковые</t>
         </is>
       </c>
       <c r="BA5" s="1" t="inlineStr">

</xml_diff>

<commit_message>
Add new Steelbear PF-41N container chassis, fix condition field bug
New 4-axle container trailer (PF-41N, FOX INTRA DISK spec) from real
VOMZ commercial offer V000319, priced at manufacturer's quote 3,250,000
RUB, with 10% Минпромторг leasing discount field populated for the
first time.

Also fixes generate_feed.py: "Состояние" was hardcoded to "С пробегом"
for every listing, including new-to-order Steelbear units — now reads
a per-record "condition" field, defaulting to used for backward compat.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WGw8UdFgVU8PXaQaPUvEwH
</commit_message>
<xml_diff>
--- a/avito-feed-trailers/fleet-trailers.xlsx
+++ b/avito-feed-trailers/fleet-trailers.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BE9"/>
+  <dimension ref="A1:BE10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1620,7 +1620,7 @@
       <c r="C7" s="1" t="inlineStr"/>
       <c r="D7" s="1" t="inlineStr">
         <is>
-          <t>steelbear-pl24l-ea653666</t>
+          <t>steelbear-pf41n-v000319</t>
         </is>
       </c>
       <c r="E7" s="1" t="inlineStr"/>
@@ -1637,12 +1637,12 @@
       </c>
       <c r="M7" s="1" t="inlineStr">
         <is>
-          <t>Полуприцеп-сортиментовоз Steelbear PL-24L (коммерческое название PT-24L BPW Heavy Duty), 2024 год выпуска, под заказ.
-Усиленное шасси из двутавровых лонжеронов, 3 оси BPW Heavy Duty, барабанные тормоза, пневмоподвеска с функцией подъём/опускание, допустимая нагрузка на ось 9 000 кг. Шины 385/65R22,5, односкат. Электронная тормозная система WABCO TEBS-E с функцией противоопрокидывания (RSS).
-6 пар открепляемых коников грузоподъёмностью 8 тонн каждая (сталь STRENX 700MC), положение регулируется вдоль рамы. Внутренняя высота коника 2330 мм. Настил из ламинированной берёзовой фанеры. Опорное устройство BPW, 24 т.
-Максимальная полная масса 44 000 кг, грузоподъёмность 37 100 кг, длина 13 620 мм.
-Заводская гарантия — 24 месяца, от сквозной коррозии — 10 лет.
-Поставка под заказ, срок — уточняйте.</t>
+          <t>Полуприцеп-контейнеровоз Steelbear PF-41N (коммерческое название PF-41N FOX INTRA DISK), 4-х осный, универсал, под заказ.
+Перевозит 1×40-футовый контейнер (в т.ч. HQ), 2×20-футовых контейнера или 1×20-футовый по центру. Максимальная полная масса 47 000 кг, грузоподъёмность 41 100 кг, длина 12 600 мм.
+Осевой агрегат FOX B9-22S с дисковыми тормозами, допустимая нагрузка на ось 9 000 кг. Усиленная пневмоподвеска FOX INTRA с подъёмом/опусканием 1-й оси (ручное управление) и 2-й оси (автоматическое). Электронная тормозная система Haldex EBS 4S/2M с функцией противоопрокидывания (RSS), информационная система INFOCENTER.
+Опорное устройство GOS, 24 т, шкворень OREX 2 дюйма. Боковая алюминиевая защита, заднее защитное устройство. Два инструментальных ящика SKARB с замком. Шины TYREX 385/55R22,5 на дисках KRONPRINZ, 9 колёс в комплекте (включая запасное).
+При покупке в лизинг — скидка от Минпромторга 10%.
+Заводская гарантия — 12 месяцев. Поставка — 10 рабочих дней с момента предоплаты.</t>
         </is>
       </c>
       <c r="N7" s="1" t="inlineStr">
@@ -1652,14 +1652,14 @@
       </c>
       <c r="O7" s="1" t="inlineStr">
         <is>
-          <t>2970000</t>
+          <t>3250000</t>
         </is>
       </c>
       <c r="P7" s="1" t="inlineStr"/>
       <c r="Q7" s="1" t="inlineStr"/>
       <c r="R7" s="1" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/04.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/05.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/06.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/07.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/08.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/09.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/10.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/11.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/12.jpg</t>
+          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pf41n-v000319/01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pf41n-v000319/02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pf41n-v000319/03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pf41n-v000319/04.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pf41n-v000319/05.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pf41n-v000319/06.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pf41n-v000319/07.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pf41n-v000319/08.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pf41n-v000319/09.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pf41n-v000319/10.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pf41n-v000319/11.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pf41n-v000319/12.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pf41n-v000319/13.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pf41n-v000319/14.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pf41n-v000319/15.jpg</t>
         </is>
       </c>
       <c r="S7" s="1" t="inlineStr"/>
@@ -1685,7 +1685,7 @@
       <c r="AA7" s="1" t="inlineStr"/>
       <c r="AB7" s="1" t="inlineStr">
         <is>
-          <t>2970000</t>
+          <t>3250000</t>
         </is>
       </c>
       <c r="AC7" s="1" t="inlineStr">
@@ -1693,7 +1693,11 @@
           <t>Под заказ</t>
         </is>
       </c>
-      <c r="AD7" s="1" t="inlineStr"/>
+      <c r="AD7" s="1" t="inlineStr">
+        <is>
+          <t>10%</t>
+        </is>
+      </c>
       <c r="AE7" s="1" t="inlineStr"/>
       <c r="AF7" s="1" t="inlineStr"/>
       <c r="AG7" s="1" t="inlineStr"/>
@@ -1704,7 +1708,7 @@
       <c r="AL7" s="1" t="inlineStr"/>
       <c r="AM7" s="1" t="inlineStr">
         <is>
-          <t>С пробегом</t>
+          <t>Новое</t>
         </is>
       </c>
       <c r="AN7" s="1" t="inlineStr"/>
@@ -1720,7 +1724,7 @@
       </c>
       <c r="AQ7" s="1" t="inlineStr">
         <is>
-          <t>PL-24L</t>
+          <t>PF-41N</t>
         </is>
       </c>
       <c r="AR7" s="1" t="inlineStr">
@@ -1730,7 +1734,7 @@
       </c>
       <c r="AS7" s="1" t="inlineStr">
         <is>
-          <t>Лесовоз (сортиментовоз)</t>
+          <t>Контейнеровоз</t>
         </is>
       </c>
       <c r="AT7" s="1" t="inlineStr"/>
@@ -1738,12 +1742,12 @@
       <c r="AV7" s="1" t="inlineStr"/>
       <c r="AW7" s="1" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="AX7" s="1" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AY7" s="1" t="inlineStr">
@@ -1753,17 +1757,17 @@
       </c>
       <c r="AZ7" s="1" t="inlineStr">
         <is>
-          <t>Барабанные</t>
+          <t>Дисковые</t>
         </is>
       </c>
       <c r="BA7" s="1" t="inlineStr">
         <is>
-          <t>37100</t>
+          <t>41100</t>
         </is>
       </c>
       <c r="BB7" s="1" t="inlineStr">
         <is>
-          <t>13620</t>
+          <t>12600</t>
         </is>
       </c>
       <c r="BC7" s="1" t="inlineStr"/>
@@ -1780,7 +1784,7 @@
       <c r="C8" s="1" t="inlineStr"/>
       <c r="D8" s="1" t="inlineStr">
         <is>
-          <t>tonar-k4u-p0002033</t>
+          <t>steelbear-pl24l-ea653666</t>
         </is>
       </c>
       <c r="E8" s="1" t="inlineStr"/>
@@ -1797,11 +1801,12 @@
       </c>
       <c r="M8" s="1" t="inlineStr">
         <is>
-          <t>Полуприцеп-контейнеровоз Тонар К4-U (99891), 2023 год, в работе, полностью исправен.
-4 оси: тройная задняя тележка плюс вынесенная вперёд ось — меньше нагрузка на дорогу и мягче по осевым ограничениям в городе. Тормоза дисковые, пневмопривод. Подвеска зависимая, на продольных рычагах, с пневмоэлементами и телескопическими амортизаторами. Шины 385/55R22.5, односкатные.
-Берёт контейнеры 20', 2×20', 30', 30' HC, 40', 40' HC. Разрешённая максимальная масса 44 000 кг, грузоподъёмность 37 800 кг, нагрузка на ССУ 11 000 кг. Высота ССУ 1 100 мм.
-VIN X0T998910P0002033.
-Возможна аренда с правом выкупа — уточняйте условия по телефону.</t>
+          <t>Полуприцеп-сортиментовоз Steelbear PL-24L (коммерческое название PT-24L BPW Heavy Duty), 2024 год выпуска, под заказ.
+Усиленное шасси из двутавровых лонжеронов, 3 оси BPW Heavy Duty, барабанные тормоза, пневмоподвеска с функцией подъём/опускание, допустимая нагрузка на ось 9 000 кг. Шины 385/65R22,5, односкат. Электронная тормозная система WABCO TEBS-E с функцией противоопрокидывания (RSS).
+6 пар открепляемых коников грузоподъёмностью 8 тонн каждая (сталь STRENX 700MC), положение регулируется вдоль рамы. Внутренняя высота коника 2330 мм. Настил из ламинированной берёзовой фанеры. Опорное устройство BPW, 24 т.
+Максимальная полная масса 44 000 кг, грузоподъёмность 37 100 кг, длина 13 620 мм.
+Заводская гарантия — 24 месяца, от сквозной коррозии — 10 лет.
+Поставка под заказ, срок — уточняйте.</t>
         </is>
       </c>
       <c r="N8" s="1" t="inlineStr">
@@ -1811,14 +1816,14 @@
       </c>
       <c r="O8" s="1" t="inlineStr">
         <is>
-          <t>1690000</t>
+          <t>2970000</t>
         </is>
       </c>
       <c r="P8" s="1" t="inlineStr"/>
       <c r="Q8" s="1" t="inlineStr"/>
       <c r="R8" s="1" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-p0002033/01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-p0002033/02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-p0002033/03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-p0002033/04.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-p0002033/05.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-p0002033/06.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-p0002033/07.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-p0002033/08.jpg</t>
+          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/04.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/05.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/06.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/07.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/08.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/09.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/10.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/11.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/12.jpg</t>
         </is>
       </c>
       <c r="S8" s="1" t="inlineStr"/>
@@ -1844,12 +1849,12 @@
       <c r="AA8" s="1" t="inlineStr"/>
       <c r="AB8" s="1" t="inlineStr">
         <is>
-          <t>1690000</t>
+          <t>2970000</t>
         </is>
       </c>
       <c r="AC8" s="1" t="inlineStr">
         <is>
-          <t>В наличии</t>
+          <t>Под заказ</t>
         </is>
       </c>
       <c r="AD8" s="1" t="inlineStr"/>
@@ -1863,7 +1868,7 @@
       <c r="AL8" s="1" t="inlineStr"/>
       <c r="AM8" s="1" t="inlineStr">
         <is>
-          <t>С пробегом</t>
+          <t>Новое</t>
         </is>
       </c>
       <c r="AN8" s="1" t="inlineStr"/>
@@ -1874,12 +1879,12 @@
       </c>
       <c r="AP8" s="1" t="inlineStr">
         <is>
-          <t>Тонар</t>
+          <t>Steelbear</t>
         </is>
       </c>
       <c r="AQ8" s="1" t="inlineStr">
         <is>
-          <t>K4-U (99891)</t>
+          <t>PL-24L</t>
         </is>
       </c>
       <c r="AR8" s="1" t="inlineStr">
@@ -1889,44 +1894,40 @@
       </c>
       <c r="AS8" s="1" t="inlineStr">
         <is>
-          <t>Контейнеровоз</t>
+          <t>Лесовоз (сортиментовоз)</t>
         </is>
       </c>
       <c r="AT8" s="1" t="inlineStr"/>
       <c r="AU8" s="1" t="inlineStr"/>
-      <c r="AV8" s="1" t="inlineStr">
-        <is>
-          <t>X0T998910P0002033</t>
-        </is>
-      </c>
+      <c r="AV8" s="1" t="inlineStr"/>
       <c r="AW8" s="1" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="AX8" s="1" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="AY8" s="1" t="inlineStr">
         <is>
-          <t>Рессорная</t>
+          <t>Пневматическая</t>
         </is>
       </c>
       <c r="AZ8" s="1" t="inlineStr">
         <is>
-          <t>Дисковые</t>
+          <t>Барабанные</t>
         </is>
       </c>
       <c r="BA8" s="1" t="inlineStr">
         <is>
-          <t>37800</t>
+          <t>37100</t>
         </is>
       </c>
       <c r="BB8" s="1" t="inlineStr">
         <is>
-          <t>12725</t>
+          <t>13620</t>
         </is>
       </c>
       <c r="BC8" s="1" t="inlineStr"/>
@@ -1943,7 +1944,7 @@
       <c r="C9" s="1" t="inlineStr"/>
       <c r="D9" s="1" t="inlineStr">
         <is>
-          <t>v-trailer-329d-r0000119</t>
+          <t>tonar-k4u-p0002033</t>
         </is>
       </c>
       <c r="E9" s="1" t="inlineStr"/>
@@ -1960,10 +1961,10 @@
       </c>
       <c r="M9" s="1" t="inlineStr">
         <is>
-          <t>Шторный полуприцеп V-Trailer 329D, 2023 год, в работе, полностью исправен.
-Оси SAF, подъёмная передняя — меньше износ резины и расход на порожняке. Опорное устройство JOST на 24 тонны, шкворень 2 дюйма по ISO 1726. Пол — влагостойкая фанера 30 мм, держит погрузчик до 7,5 тонн. Крыша сдвижная (Sesam/Edscha) — грузить сверху краном или погрузчиком без снятия тента. Двери алюминиевые BPW Smartmaster II, передний и задний портал — стальные, собственной конструкции. Рама облегчённая, с дополнительными усилениями против скручивания. По бортам — корзины под коники, по 7 штук на сторону.
-13,6 × 2,5 × 4 м, 91 м³. Тент плотный: борта 900 г/м², крыша 680 г/м². Полная штора, без бортов — удобно под европаллеты и груз с выступом по высоте.
-VIN XZFVKRP3DR0000119.
+          <t>Полуприцеп-контейнеровоз Тонар К4-U (99891), 2023 год, в работе, полностью исправен.
+4 оси: тройная задняя тележка плюс вынесенная вперёд ось — меньше нагрузка на дорогу и мягче по осевым ограничениям в городе. Тормоза дисковые, пневмопривод. Подвеска зависимая, на продольных рычагах, с пневмоэлементами и телескопическими амортизаторами. Шины 385/55R22.5, односкатные.
+Берёт контейнеры 20', 2×20', 30', 30' HC, 40', 40' HC. Разрешённая максимальная масса 44 000 кг, грузоподъёмность 37 800 кг, нагрузка на ССУ 11 000 кг. Высота ССУ 1 100 мм.
+VIN X0T998910P0002033.
 Возможна аренда с правом выкупа — уточняйте условия по телефону.</t>
         </is>
       </c>
@@ -1974,14 +1975,14 @@
       </c>
       <c r="O9" s="1" t="inlineStr">
         <is>
-          <t>2990000</t>
+          <t>1690000</t>
         </is>
       </c>
       <c r="P9" s="1" t="inlineStr"/>
       <c r="Q9" s="1" t="inlineStr"/>
       <c r="R9" s="1" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/04.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/05.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/06.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/07.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/08.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/09.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/10.jpg</t>
+          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-p0002033/01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-p0002033/02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-p0002033/03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-p0002033/04.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-p0002033/05.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-p0002033/06.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-p0002033/07.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-p0002033/08.jpg</t>
         </is>
       </c>
       <c r="S9" s="1" t="inlineStr"/>
@@ -2007,7 +2008,7 @@
       <c r="AA9" s="1" t="inlineStr"/>
       <c r="AB9" s="1" t="inlineStr">
         <is>
-          <t>2990000</t>
+          <t>1690000</t>
         </is>
       </c>
       <c r="AC9" s="1" t="inlineStr">
@@ -2037,12 +2038,12 @@
       </c>
       <c r="AP9" s="1" t="inlineStr">
         <is>
-          <t>V-Trailer</t>
+          <t>Тонар</t>
         </is>
       </c>
       <c r="AQ9" s="1" t="inlineStr">
         <is>
-          <t>329</t>
+          <t>K4-U (99891)</t>
         </is>
       </c>
       <c r="AR9" s="1" t="inlineStr">
@@ -2052,14 +2053,14 @@
       </c>
       <c r="AS9" s="1" t="inlineStr">
         <is>
-          <t>Шторный</t>
+          <t>Контейнеровоз</t>
         </is>
       </c>
       <c r="AT9" s="1" t="inlineStr"/>
       <c r="AU9" s="1" t="inlineStr"/>
       <c r="AV9" s="1" t="inlineStr">
         <is>
-          <t>XZFVKRP3DR0000119</t>
+          <t>X0T998910P0002033</t>
         </is>
       </c>
       <c r="AW9" s="1" t="inlineStr">
@@ -2069,12 +2070,12 @@
       </c>
       <c r="AX9" s="1" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AY9" s="1" t="inlineStr">
         <is>
-          <t>Пневматическая</t>
+          <t>Рессорная</t>
         </is>
       </c>
       <c r="AZ9" s="1" t="inlineStr">
@@ -2084,21 +2085,184 @@
       </c>
       <c r="BA9" s="1" t="inlineStr">
         <is>
-          <t>32300</t>
+          <t>37800</t>
         </is>
       </c>
       <c r="BB9" s="1" t="inlineStr">
         <is>
-          <t>13600</t>
-        </is>
-      </c>
-      <c r="BC9" s="1" t="inlineStr">
-        <is>
-          <t>91</t>
-        </is>
-      </c>
+          <t>12725</t>
+        </is>
+      </c>
+      <c r="BC9" s="1" t="inlineStr"/>
       <c r="BD9" s="1" t="inlineStr"/>
       <c r="BE9" s="1" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>Москва, Ижорская ул., 15с2</t>
+        </is>
+      </c>
+      <c r="B10" s="1" t="inlineStr"/>
+      <c r="C10" s="1" t="inlineStr"/>
+      <c r="D10" s="1" t="inlineStr">
+        <is>
+          <t>v-trailer-329d-r0000119</t>
+        </is>
+      </c>
+      <c r="E10" s="1" t="inlineStr"/>
+      <c r="F10" s="1" t="inlineStr"/>
+      <c r="G10" s="1" t="inlineStr"/>
+      <c r="H10" s="1" t="inlineStr"/>
+      <c r="I10" s="1" t="inlineStr"/>
+      <c r="J10" s="1" t="inlineStr"/>
+      <c r="K10" s="1" t="inlineStr"/>
+      <c r="L10" s="1" t="inlineStr">
+        <is>
+          <t>По телефону и в сообщениях</t>
+        </is>
+      </c>
+      <c r="M10" s="1" t="inlineStr">
+        <is>
+          <t>Шторный полуприцеп V-Trailer 329D, 2023 год, в работе, полностью исправен.
+Оси SAF, подъёмная передняя — меньше износ резины и расход на порожняке. Опорное устройство JOST на 24 тонны, шкворень 2 дюйма по ISO 1726. Пол — влагостойкая фанера 30 мм, держит погрузчик до 7,5 тонн. Крыша сдвижная (Sesam/Edscha) — грузить сверху краном или погрузчиком без снятия тента. Двери алюминиевые BPW Smartmaster II, передний и задний портал — стальные, собственной конструкции. Рама облегчённая, с дополнительными усилениями против скручивания. По бортам — корзины под коники, по 7 штук на сторону.
+13,6 × 2,5 × 4 м, 91 м³. Тент плотный: борта 900 г/м², крыша 680 г/м². Полная штора, без бортов — удобно под европаллеты и груз с выступом по высоте.
+VIN XZFVKRP3DR0000119.
+Возможна аренда с правом выкупа — уточняйте условия по телефону.</t>
+        </is>
+      </c>
+      <c r="N10" s="1" t="inlineStr">
+        <is>
+          <t>Грузовики и спецтехника</t>
+        </is>
+      </c>
+      <c r="O10" s="1" t="inlineStr">
+        <is>
+          <t>2990000</t>
+        </is>
+      </c>
+      <c r="P10" s="1" t="inlineStr"/>
+      <c r="Q10" s="1" t="inlineStr"/>
+      <c r="R10" s="1" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/04.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/05.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/06.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/07.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/08.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/09.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/10.jpg</t>
+        </is>
+      </c>
+      <c r="S10" s="1" t="inlineStr"/>
+      <c r="T10" s="1" t="inlineStr"/>
+      <c r="U10" s="1" t="inlineStr"/>
+      <c r="V10" s="1" t="inlineStr"/>
+      <c r="W10" s="1" t="inlineStr"/>
+      <c r="X10" s="1" t="inlineStr">
+        <is>
+          <t>Прицепы</t>
+        </is>
+      </c>
+      <c r="Y10" s="1" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="Z10" s="1" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="AA10" s="1" t="inlineStr"/>
+      <c r="AB10" s="1" t="inlineStr">
+        <is>
+          <t>2990000</t>
+        </is>
+      </c>
+      <c r="AC10" s="1" t="inlineStr">
+        <is>
+          <t>В наличии</t>
+        </is>
+      </c>
+      <c r="AD10" s="1" t="inlineStr"/>
+      <c r="AE10" s="1" t="inlineStr"/>
+      <c r="AF10" s="1" t="inlineStr"/>
+      <c r="AG10" s="1" t="inlineStr"/>
+      <c r="AH10" s="1" t="inlineStr"/>
+      <c r="AI10" s="1" t="inlineStr"/>
+      <c r="AJ10" s="1" t="inlineStr"/>
+      <c r="AK10" s="1" t="inlineStr"/>
+      <c r="AL10" s="1" t="inlineStr"/>
+      <c r="AM10" s="1" t="inlineStr">
+        <is>
+          <t>С пробегом</t>
+        </is>
+      </c>
+      <c r="AN10" s="1" t="inlineStr"/>
+      <c r="AO10" s="1" t="inlineStr">
+        <is>
+          <t>В наличии</t>
+        </is>
+      </c>
+      <c r="AP10" s="1" t="inlineStr">
+        <is>
+          <t>V-Trailer</t>
+        </is>
+      </c>
+      <c r="AQ10" s="1" t="inlineStr">
+        <is>
+          <t>329</t>
+        </is>
+      </c>
+      <c r="AR10" s="1" t="inlineStr">
+        <is>
+          <t>Полуприцеп</t>
+        </is>
+      </c>
+      <c r="AS10" s="1" t="inlineStr">
+        <is>
+          <t>Шторный</t>
+        </is>
+      </c>
+      <c r="AT10" s="1" t="inlineStr"/>
+      <c r="AU10" s="1" t="inlineStr"/>
+      <c r="AV10" s="1" t="inlineStr">
+        <is>
+          <t>XZFVKRP3DR0000119</t>
+        </is>
+      </c>
+      <c r="AW10" s="1" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="AX10" s="1" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AY10" s="1" t="inlineStr">
+        <is>
+          <t>Пневматическая</t>
+        </is>
+      </c>
+      <c r="AZ10" s="1" t="inlineStr">
+        <is>
+          <t>Дисковые</t>
+        </is>
+      </c>
+      <c r="BA10" s="1" t="inlineStr">
+        <is>
+          <t>32300</t>
+        </is>
+      </c>
+      <c r="BB10" s="1" t="inlineStr">
+        <is>
+          <t>13600</t>
+        </is>
+      </c>
+      <c r="BC10" s="1" t="inlineStr">
+        <is>
+          <t>91</t>
+        </is>
+      </c>
+      <c r="BD10" s="1" t="inlineStr"/>
+      <c r="BE10" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add second Steelbear PL-24L sortimentovoz (AVG axle variant)
Second physical unit of the same PL-24L model, real factory spec from
VOMZ, AVG Axle drum-brake configuration instead of the already-listed
BPW unit — different price, photos, description. Same structural
attributes (make/model/type) as the existing PL-24L listing since
neither has a VIN yet (both built to order).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WGw8UdFgVU8PXaQaPUvEwH
</commit_message>
<xml_diff>
--- a/avito-feed-trailers/fleet-trailers.xlsx
+++ b/avito-feed-trailers/fleet-trailers.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BE10"/>
+  <dimension ref="A1:BE11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1784,7 +1784,7 @@
       <c r="C8" s="1" t="inlineStr"/>
       <c r="D8" s="1" t="inlineStr">
         <is>
-          <t>steelbear-pl24l-ea653666</t>
+          <t>steelbear-pl24l-avg36</t>
         </is>
       </c>
       <c r="E8" s="1" t="inlineStr"/>
@@ -1801,12 +1801,13 @@
       </c>
       <c r="M8" s="1" t="inlineStr">
         <is>
-          <t>Полуприцеп-сортиментовоз Steelbear PL-24L (коммерческое название PT-24L BPW Heavy Duty), 2024 год выпуска, под заказ.
-Усиленное шасси из двутавровых лонжеронов, 3 оси BPW Heavy Duty, барабанные тормоза, пневмоподвеска с функцией подъём/опускание, допустимая нагрузка на ось 9 000 кг. Шины 385/65R22,5, односкат. Электронная тормозная система WABCO TEBS-E с функцией противоопрокидывания (RSS).
-6 пар открепляемых коников грузоподъёмностью 8 тонн каждая (сталь STRENX 700MC), положение регулируется вдоль рамы. Внутренняя высота коника 2330 мм. Настил из ламинированной берёзовой фанеры. Опорное устройство BPW, 24 т.
-Максимальная полная масса 44 000 кг, грузоподъёмность 37 100 кг, длина 13 620 мм.
-Заводская гарантия — 24 месяца, от сквозной коррозии — 10 лет.
-Поставка под заказ, срок — уточняйте.</t>
+          <t>Полуприцеп-сортиментовоз Steelbear PL-24L (коммерческое название PT-24L AVG), 3-х осный, под заказ.
+Осевой агрегат AVG Axle, квадратная ось сечением 120×120 мм — устойчивее к скручиванию на дорогах с боковым уклоном, чем круглая. Барабанные тормоза, допустимая нагрузка на ось 9 000 кг. Усиленная пневмоподвеска AVG с подъёмом/опусканием. Электронная тормозная система TEBS 2S/2M с функцией противоопрокидывания (RSS), манометр давления в пневмоподвеске.
+6 пар коников с неоткрепляемыми стойками, грузоподъёмность 7 тонн каждая, положение регулируется вдоль рамы. Внутренняя высота коника 2 340 мм. 6 ремней для крепления сортимента. Неразборная передняя стенка перфорированного типа с крюками для каната и креплением для лома и лопаты.
+Опорное устройство GOS, 24 т, шкворень OREX 2 дюйма. Боковая алюминиевая противоподкатная защита. Металлический инструментальный ящик с замком. Шины TYREX 385/65R22,5.
+Максимальная полная масса 44 000 кг, грузоподъёмность 36 500 кг, длина 13 620 мм.
+При покупке в лизинг — скидка от Минпромторга 10%.
+Заводская гарантия — 12 месяцев. Поставка — 15 рабочих дней с момента предоплаты.</t>
         </is>
       </c>
       <c r="N8" s="1" t="inlineStr">
@@ -1816,14 +1817,14 @@
       </c>
       <c r="O8" s="1" t="inlineStr">
         <is>
-          <t>2970000</t>
+          <t>2960000</t>
         </is>
       </c>
       <c r="P8" s="1" t="inlineStr"/>
       <c r="Q8" s="1" t="inlineStr"/>
       <c r="R8" s="1" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/04.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/05.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/06.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/07.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/08.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/09.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/10.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/11.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/12.jpg</t>
+          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-avg36/01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-avg36/02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-avg36/03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-avg36/04.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-avg36/05.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-avg36/06.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-avg36/07.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-avg36/08.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-avg36/09.jpg</t>
         </is>
       </c>
       <c r="S8" s="1" t="inlineStr"/>
@@ -1849,7 +1850,7 @@
       <c r="AA8" s="1" t="inlineStr"/>
       <c r="AB8" s="1" t="inlineStr">
         <is>
-          <t>2970000</t>
+          <t>2960000</t>
         </is>
       </c>
       <c r="AC8" s="1" t="inlineStr">
@@ -1857,7 +1858,11 @@
           <t>Под заказ</t>
         </is>
       </c>
-      <c r="AD8" s="1" t="inlineStr"/>
+      <c r="AD8" s="1" t="inlineStr">
+        <is>
+          <t>10%</t>
+        </is>
+      </c>
       <c r="AE8" s="1" t="inlineStr"/>
       <c r="AF8" s="1" t="inlineStr"/>
       <c r="AG8" s="1" t="inlineStr"/>
@@ -1902,7 +1907,7 @@
       <c r="AV8" s="1" t="inlineStr"/>
       <c r="AW8" s="1" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="AX8" s="1" t="inlineStr">
@@ -1922,7 +1927,7 @@
       </c>
       <c r="BA8" s="1" t="inlineStr">
         <is>
-          <t>37100</t>
+          <t>36500</t>
         </is>
       </c>
       <c r="BB8" s="1" t="inlineStr">
@@ -1944,7 +1949,7 @@
       <c r="C9" s="1" t="inlineStr"/>
       <c r="D9" s="1" t="inlineStr">
         <is>
-          <t>tonar-k4u-p0002033</t>
+          <t>steelbear-pl24l-ea653666</t>
         </is>
       </c>
       <c r="E9" s="1" t="inlineStr"/>
@@ -1961,11 +1966,12 @@
       </c>
       <c r="M9" s="1" t="inlineStr">
         <is>
-          <t>Полуприцеп-контейнеровоз Тонар К4-U (99891), 2023 год, в работе, полностью исправен.
-4 оси: тройная задняя тележка плюс вынесенная вперёд ось — меньше нагрузка на дорогу и мягче по осевым ограничениям в городе. Тормоза дисковые, пневмопривод. Подвеска зависимая, на продольных рычагах, с пневмоэлементами и телескопическими амортизаторами. Шины 385/55R22.5, односкатные.
-Берёт контейнеры 20', 2×20', 30', 30' HC, 40', 40' HC. Разрешённая максимальная масса 44 000 кг, грузоподъёмность 37 800 кг, нагрузка на ССУ 11 000 кг. Высота ССУ 1 100 мм.
-VIN X0T998910P0002033.
-Возможна аренда с правом выкупа — уточняйте условия по телефону.</t>
+          <t>Полуприцеп-сортиментовоз Steelbear PL-24L (коммерческое название PT-24L BPW Heavy Duty), 2024 год выпуска, под заказ.
+Усиленное шасси из двутавровых лонжеронов, 3 оси BPW Heavy Duty, барабанные тормоза, пневмоподвеска с функцией подъём/опускание, допустимая нагрузка на ось 9 000 кг. Шины 385/65R22,5, односкат. Электронная тормозная система WABCO TEBS-E с функцией противоопрокидывания (RSS).
+6 пар открепляемых коников грузоподъёмностью 8 тонн каждая (сталь STRENX 700MC), положение регулируется вдоль рамы. Внутренняя высота коника 2330 мм. Настил из ламинированной берёзовой фанеры. Опорное устройство BPW, 24 т.
+Максимальная полная масса 44 000 кг, грузоподъёмность 37 100 кг, длина 13 620 мм.
+Заводская гарантия — 24 месяца, от сквозной коррозии — 10 лет.
+Поставка под заказ, срок — уточняйте.</t>
         </is>
       </c>
       <c r="N9" s="1" t="inlineStr">
@@ -1975,14 +1981,14 @@
       </c>
       <c r="O9" s="1" t="inlineStr">
         <is>
-          <t>1690000</t>
+          <t>2970000</t>
         </is>
       </c>
       <c r="P9" s="1" t="inlineStr"/>
       <c r="Q9" s="1" t="inlineStr"/>
       <c r="R9" s="1" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-p0002033/01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-p0002033/02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-p0002033/03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-p0002033/04.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-p0002033/05.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-p0002033/06.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-p0002033/07.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-p0002033/08.jpg</t>
+          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/04.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/05.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/06.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/07.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/08.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/09.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/10.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/11.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/12.jpg</t>
         </is>
       </c>
       <c r="S9" s="1" t="inlineStr"/>
@@ -2008,12 +2014,12 @@
       <c r="AA9" s="1" t="inlineStr"/>
       <c r="AB9" s="1" t="inlineStr">
         <is>
-          <t>1690000</t>
+          <t>2970000</t>
         </is>
       </c>
       <c r="AC9" s="1" t="inlineStr">
         <is>
-          <t>В наличии</t>
+          <t>Под заказ</t>
         </is>
       </c>
       <c r="AD9" s="1" t="inlineStr"/>
@@ -2027,7 +2033,7 @@
       <c r="AL9" s="1" t="inlineStr"/>
       <c r="AM9" s="1" t="inlineStr">
         <is>
-          <t>С пробегом</t>
+          <t>Новое</t>
         </is>
       </c>
       <c r="AN9" s="1" t="inlineStr"/>
@@ -2038,12 +2044,12 @@
       </c>
       <c r="AP9" s="1" t="inlineStr">
         <is>
-          <t>Тонар</t>
+          <t>Steelbear</t>
         </is>
       </c>
       <c r="AQ9" s="1" t="inlineStr">
         <is>
-          <t>K4-U (99891)</t>
+          <t>PL-24L</t>
         </is>
       </c>
       <c r="AR9" s="1" t="inlineStr">
@@ -2053,44 +2059,40 @@
       </c>
       <c r="AS9" s="1" t="inlineStr">
         <is>
-          <t>Контейнеровоз</t>
+          <t>Лесовоз (сортиментовоз)</t>
         </is>
       </c>
       <c r="AT9" s="1" t="inlineStr"/>
       <c r="AU9" s="1" t="inlineStr"/>
-      <c r="AV9" s="1" t="inlineStr">
-        <is>
-          <t>X0T998910P0002033</t>
-        </is>
-      </c>
+      <c r="AV9" s="1" t="inlineStr"/>
       <c r="AW9" s="1" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="AX9" s="1" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="AY9" s="1" t="inlineStr">
         <is>
-          <t>Рессорная</t>
+          <t>Пневматическая</t>
         </is>
       </c>
       <c r="AZ9" s="1" t="inlineStr">
         <is>
-          <t>Дисковые</t>
+          <t>Барабанные</t>
         </is>
       </c>
       <c r="BA9" s="1" t="inlineStr">
         <is>
-          <t>37800</t>
+          <t>37100</t>
         </is>
       </c>
       <c r="BB9" s="1" t="inlineStr">
         <is>
-          <t>12725</t>
+          <t>13620</t>
         </is>
       </c>
       <c r="BC9" s="1" t="inlineStr"/>
@@ -2107,7 +2109,7 @@
       <c r="C10" s="1" t="inlineStr"/>
       <c r="D10" s="1" t="inlineStr">
         <is>
-          <t>v-trailer-329d-r0000119</t>
+          <t>tonar-k4u-p0002033</t>
         </is>
       </c>
       <c r="E10" s="1" t="inlineStr"/>
@@ -2124,10 +2126,10 @@
       </c>
       <c r="M10" s="1" t="inlineStr">
         <is>
-          <t>Шторный полуприцеп V-Trailer 329D, 2023 год, в работе, полностью исправен.
-Оси SAF, подъёмная передняя — меньше износ резины и расход на порожняке. Опорное устройство JOST на 24 тонны, шкворень 2 дюйма по ISO 1726. Пол — влагостойкая фанера 30 мм, держит погрузчик до 7,5 тонн. Крыша сдвижная (Sesam/Edscha) — грузить сверху краном или погрузчиком без снятия тента. Двери алюминиевые BPW Smartmaster II, передний и задний портал — стальные, собственной конструкции. Рама облегчённая, с дополнительными усилениями против скручивания. По бортам — корзины под коники, по 7 штук на сторону.
-13,6 × 2,5 × 4 м, 91 м³. Тент плотный: борта 900 г/м², крыша 680 г/м². Полная штора, без бортов — удобно под европаллеты и груз с выступом по высоте.
-VIN XZFVKRP3DR0000119.
+          <t>Полуприцеп-контейнеровоз Тонар К4-U (99891), 2023 год, в работе, полностью исправен.
+4 оси: тройная задняя тележка плюс вынесенная вперёд ось — меньше нагрузка на дорогу и мягче по осевым ограничениям в городе. Тормоза дисковые, пневмопривод. Подвеска зависимая, на продольных рычагах, с пневмоэлементами и телескопическими амортизаторами. Шины 385/55R22.5, односкатные.
+Берёт контейнеры 20', 2×20', 30', 30' HC, 40', 40' HC. Разрешённая максимальная масса 44 000 кг, грузоподъёмность 37 800 кг, нагрузка на ССУ 11 000 кг. Высота ССУ 1 100 мм.
+VIN X0T998910P0002033.
 Возможна аренда с правом выкупа — уточняйте условия по телефону.</t>
         </is>
       </c>
@@ -2138,14 +2140,14 @@
       </c>
       <c r="O10" s="1" t="inlineStr">
         <is>
-          <t>2990000</t>
+          <t>1690000</t>
         </is>
       </c>
       <c r="P10" s="1" t="inlineStr"/>
       <c r="Q10" s="1" t="inlineStr"/>
       <c r="R10" s="1" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/04.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/05.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/06.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/07.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/08.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/09.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/10.jpg</t>
+          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-p0002033/01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-p0002033/02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-p0002033/03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-p0002033/04.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-p0002033/05.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-p0002033/06.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-p0002033/07.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-p0002033/08.jpg</t>
         </is>
       </c>
       <c r="S10" s="1" t="inlineStr"/>
@@ -2171,7 +2173,7 @@
       <c r="AA10" s="1" t="inlineStr"/>
       <c r="AB10" s="1" t="inlineStr">
         <is>
-          <t>2990000</t>
+          <t>1690000</t>
         </is>
       </c>
       <c r="AC10" s="1" t="inlineStr">
@@ -2201,12 +2203,12 @@
       </c>
       <c r="AP10" s="1" t="inlineStr">
         <is>
-          <t>V-Trailer</t>
+          <t>Тонар</t>
         </is>
       </c>
       <c r="AQ10" s="1" t="inlineStr">
         <is>
-          <t>329</t>
+          <t>K4-U (99891)</t>
         </is>
       </c>
       <c r="AR10" s="1" t="inlineStr">
@@ -2216,14 +2218,14 @@
       </c>
       <c r="AS10" s="1" t="inlineStr">
         <is>
-          <t>Шторный</t>
+          <t>Контейнеровоз</t>
         </is>
       </c>
       <c r="AT10" s="1" t="inlineStr"/>
       <c r="AU10" s="1" t="inlineStr"/>
       <c r="AV10" s="1" t="inlineStr">
         <is>
-          <t>XZFVKRP3DR0000119</t>
+          <t>X0T998910P0002033</t>
         </is>
       </c>
       <c r="AW10" s="1" t="inlineStr">
@@ -2233,12 +2235,12 @@
       </c>
       <c r="AX10" s="1" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AY10" s="1" t="inlineStr">
         <is>
-          <t>Пневматическая</t>
+          <t>Рессорная</t>
         </is>
       </c>
       <c r="AZ10" s="1" t="inlineStr">
@@ -2248,21 +2250,184 @@
       </c>
       <c r="BA10" s="1" t="inlineStr">
         <is>
-          <t>32300</t>
+          <t>37800</t>
         </is>
       </c>
       <c r="BB10" s="1" t="inlineStr">
         <is>
-          <t>13600</t>
-        </is>
-      </c>
-      <c r="BC10" s="1" t="inlineStr">
-        <is>
-          <t>91</t>
-        </is>
-      </c>
+          <t>12725</t>
+        </is>
+      </c>
+      <c r="BC10" s="1" t="inlineStr"/>
       <c r="BD10" s="1" t="inlineStr"/>
       <c r="BE10" s="1" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>Москва, Ижорская ул., 15с2</t>
+        </is>
+      </c>
+      <c r="B11" s="1" t="inlineStr"/>
+      <c r="C11" s="1" t="inlineStr"/>
+      <c r="D11" s="1" t="inlineStr">
+        <is>
+          <t>v-trailer-329d-r0000119</t>
+        </is>
+      </c>
+      <c r="E11" s="1" t="inlineStr"/>
+      <c r="F11" s="1" t="inlineStr"/>
+      <c r="G11" s="1" t="inlineStr"/>
+      <c r="H11" s="1" t="inlineStr"/>
+      <c r="I11" s="1" t="inlineStr"/>
+      <c r="J11" s="1" t="inlineStr"/>
+      <c r="K11" s="1" t="inlineStr"/>
+      <c r="L11" s="1" t="inlineStr">
+        <is>
+          <t>По телефону и в сообщениях</t>
+        </is>
+      </c>
+      <c r="M11" s="1" t="inlineStr">
+        <is>
+          <t>Шторный полуприцеп V-Trailer 329D, 2023 год, в работе, полностью исправен.
+Оси SAF, подъёмная передняя — меньше износ резины и расход на порожняке. Опорное устройство JOST на 24 тонны, шкворень 2 дюйма по ISO 1726. Пол — влагостойкая фанера 30 мм, держит погрузчик до 7,5 тонн. Крыша сдвижная (Sesam/Edscha) — грузить сверху краном или погрузчиком без снятия тента. Двери алюминиевые BPW Smartmaster II, передний и задний портал — стальные, собственной конструкции. Рама облегчённая, с дополнительными усилениями против скручивания. По бортам — корзины под коники, по 7 штук на сторону.
+13,6 × 2,5 × 4 м, 91 м³. Тент плотный: борта 900 г/м², крыша 680 г/м². Полная штора, без бортов — удобно под европаллеты и груз с выступом по высоте.
+VIN XZFVKRP3DR0000119.
+Возможна аренда с правом выкупа — уточняйте условия по телефону.</t>
+        </is>
+      </c>
+      <c r="N11" s="1" t="inlineStr">
+        <is>
+          <t>Грузовики и спецтехника</t>
+        </is>
+      </c>
+      <c r="O11" s="1" t="inlineStr">
+        <is>
+          <t>2990000</t>
+        </is>
+      </c>
+      <c r="P11" s="1" t="inlineStr"/>
+      <c r="Q11" s="1" t="inlineStr"/>
+      <c r="R11" s="1" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/04.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/05.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/06.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/07.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/08.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/09.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/10.jpg</t>
+        </is>
+      </c>
+      <c r="S11" s="1" t="inlineStr"/>
+      <c r="T11" s="1" t="inlineStr"/>
+      <c r="U11" s="1" t="inlineStr"/>
+      <c r="V11" s="1" t="inlineStr"/>
+      <c r="W11" s="1" t="inlineStr"/>
+      <c r="X11" s="1" t="inlineStr">
+        <is>
+          <t>Прицепы</t>
+        </is>
+      </c>
+      <c r="Y11" s="1" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="Z11" s="1" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="AA11" s="1" t="inlineStr"/>
+      <c r="AB11" s="1" t="inlineStr">
+        <is>
+          <t>2990000</t>
+        </is>
+      </c>
+      <c r="AC11" s="1" t="inlineStr">
+        <is>
+          <t>В наличии</t>
+        </is>
+      </c>
+      <c r="AD11" s="1" t="inlineStr"/>
+      <c r="AE11" s="1" t="inlineStr"/>
+      <c r="AF11" s="1" t="inlineStr"/>
+      <c r="AG11" s="1" t="inlineStr"/>
+      <c r="AH11" s="1" t="inlineStr"/>
+      <c r="AI11" s="1" t="inlineStr"/>
+      <c r="AJ11" s="1" t="inlineStr"/>
+      <c r="AK11" s="1" t="inlineStr"/>
+      <c r="AL11" s="1" t="inlineStr"/>
+      <c r="AM11" s="1" t="inlineStr">
+        <is>
+          <t>С пробегом</t>
+        </is>
+      </c>
+      <c r="AN11" s="1" t="inlineStr"/>
+      <c r="AO11" s="1" t="inlineStr">
+        <is>
+          <t>В наличии</t>
+        </is>
+      </c>
+      <c r="AP11" s="1" t="inlineStr">
+        <is>
+          <t>V-Trailer</t>
+        </is>
+      </c>
+      <c r="AQ11" s="1" t="inlineStr">
+        <is>
+          <t>329</t>
+        </is>
+      </c>
+      <c r="AR11" s="1" t="inlineStr">
+        <is>
+          <t>Полуприцеп</t>
+        </is>
+      </c>
+      <c r="AS11" s="1" t="inlineStr">
+        <is>
+          <t>Шторный</t>
+        </is>
+      </c>
+      <c r="AT11" s="1" t="inlineStr"/>
+      <c r="AU11" s="1" t="inlineStr"/>
+      <c r="AV11" s="1" t="inlineStr">
+        <is>
+          <t>XZFVKRP3DR0000119</t>
+        </is>
+      </c>
+      <c r="AW11" s="1" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="AX11" s="1" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AY11" s="1" t="inlineStr">
+        <is>
+          <t>Пневматическая</t>
+        </is>
+      </c>
+      <c r="AZ11" s="1" t="inlineStr">
+        <is>
+          <t>Дисковые</t>
+        </is>
+      </c>
+      <c r="BA11" s="1" t="inlineStr">
+        <is>
+          <t>32300</t>
+        </is>
+      </c>
+      <c r="BB11" s="1" t="inlineStr">
+        <is>
+          <t>13600</t>
+        </is>
+      </c>
+      <c r="BC11" s="1" t="inlineStr">
+        <is>
+          <t>91</t>
+        </is>
+      </c>
+      <c r="BD11" s="1" t="inlineStr"/>
+      <c r="BE11" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Fix LeasingDiscount format, add parking address, new Kassbohrer photos
- LeasingDiscount must be an integer per real Avito validation error
  ("Значение должно быть целым числом") — changed "10%" to "10" on
  both new Steelbear listings.
- Added missing "Адрес стоянки" (parking address) field to the feed —
  Avito now requires it; previously-unedited listings were grandfathered
  past validation, but any future edit would trip the same error.
- Replaced VIN ...4732 (13.6m curtain Kassbohrer) photos with a
  correct real set to force Avito to reprocess and hopefully fix its
  stuck "isothermal" category display (data was already "Шторный").

Tonar listings intentionally excluded from this push per Артём.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WGw8UdFgVU8PXaQaPUvEwH
</commit_message>
<xml_diff>
--- a/avito-feed-trailers/fleet-trailers.xlsx
+++ b/avito-feed-trailers/fleet-trailers.xlsx
@@ -437,7 +437,7 @@
     <col width="40" customWidth="1" min="18" max="18"/>
     <col width="17" customWidth="1" min="19" max="19"/>
     <col width="21" customWidth="1" min="20" max="20"/>
-    <col width="15" customWidth="1" min="21" max="21"/>
+    <col width="28" customWidth="1" min="21" max="21"/>
     <col width="17" customWidth="1" min="22" max="22"/>
     <col width="31" customWidth="1" min="23" max="23"/>
     <col width="13" customWidth="1" min="24" max="24"/>
@@ -817,7 +817,11 @@
       </c>
       <c r="S2" s="1" t="inlineStr"/>
       <c r="T2" s="1" t="inlineStr"/>
-      <c r="U2" s="1" t="inlineStr"/>
+      <c r="U2" s="1" t="inlineStr">
+        <is>
+          <t>Москва, Ижорская ул., 15с2</t>
+        </is>
+      </c>
       <c r="V2" s="1" t="inlineStr"/>
       <c r="W2" s="1" t="inlineStr"/>
       <c r="X2" s="1" t="inlineStr">
@@ -983,7 +987,11 @@
       </c>
       <c r="S3" s="1" t="inlineStr"/>
       <c r="T3" s="1" t="inlineStr"/>
-      <c r="U3" s="1" t="inlineStr"/>
+      <c r="U3" s="1" t="inlineStr">
+        <is>
+          <t>Москва, Ижорская ул., 15с2</t>
+        </is>
+      </c>
       <c r="V3" s="1" t="inlineStr"/>
       <c r="W3" s="1" t="inlineStr"/>
       <c r="X3" s="1" t="inlineStr">
@@ -1154,7 +1162,11 @@
       </c>
       <c r="S4" s="1" t="inlineStr"/>
       <c r="T4" s="1" t="inlineStr"/>
-      <c r="U4" s="1" t="inlineStr"/>
+      <c r="U4" s="1" t="inlineStr">
+        <is>
+          <t>Москва, Ижорская ул., 15с2</t>
+        </is>
+      </c>
       <c r="V4" s="1" t="inlineStr"/>
       <c r="W4" s="1" t="inlineStr"/>
       <c r="X4" s="1" t="inlineStr">
@@ -1325,7 +1337,11 @@
       </c>
       <c r="S5" s="1" t="inlineStr"/>
       <c r="T5" s="1" t="inlineStr"/>
-      <c r="U5" s="1" t="inlineStr"/>
+      <c r="U5" s="1" t="inlineStr">
+        <is>
+          <t>Москва, Ижорская ул., 15с2</t>
+        </is>
+      </c>
       <c r="V5" s="1" t="inlineStr"/>
       <c r="W5" s="1" t="inlineStr"/>
       <c r="X5" s="1" t="inlineStr">
@@ -1496,7 +1512,11 @@
       </c>
       <c r="S6" s="1" t="inlineStr"/>
       <c r="T6" s="1" t="inlineStr"/>
-      <c r="U6" s="1" t="inlineStr"/>
+      <c r="U6" s="1" t="inlineStr">
+        <is>
+          <t>Москва, Ижорская ул., 15с2</t>
+        </is>
+      </c>
       <c r="V6" s="1" t="inlineStr"/>
       <c r="W6" s="1" t="inlineStr"/>
       <c r="X6" s="1" t="inlineStr">
@@ -1664,7 +1684,11 @@
       </c>
       <c r="S7" s="1" t="inlineStr"/>
       <c r="T7" s="1" t="inlineStr"/>
-      <c r="U7" s="1" t="inlineStr"/>
+      <c r="U7" s="1" t="inlineStr">
+        <is>
+          <t>Москва, Ижорская ул., 15с2</t>
+        </is>
+      </c>
       <c r="V7" s="1" t="inlineStr"/>
       <c r="W7" s="1" t="inlineStr"/>
       <c r="X7" s="1" t="inlineStr">
@@ -1695,7 +1719,7 @@
       </c>
       <c r="AD7" s="1" t="inlineStr">
         <is>
-          <t>10%</t>
+          <t>10</t>
         </is>
       </c>
       <c r="AE7" s="1" t="inlineStr"/>
@@ -1829,7 +1853,11 @@
       </c>
       <c r="S8" s="1" t="inlineStr"/>
       <c r="T8" s="1" t="inlineStr"/>
-      <c r="U8" s="1" t="inlineStr"/>
+      <c r="U8" s="1" t="inlineStr">
+        <is>
+          <t>Москва, Ижорская ул., 15с2</t>
+        </is>
+      </c>
       <c r="V8" s="1" t="inlineStr"/>
       <c r="W8" s="1" t="inlineStr"/>
       <c r="X8" s="1" t="inlineStr">
@@ -1860,7 +1888,7 @@
       </c>
       <c r="AD8" s="1" t="inlineStr">
         <is>
-          <t>10%</t>
+          <t>10</t>
         </is>
       </c>
       <c r="AE8" s="1" t="inlineStr"/>
@@ -1993,7 +2021,11 @@
       </c>
       <c r="S9" s="1" t="inlineStr"/>
       <c r="T9" s="1" t="inlineStr"/>
-      <c r="U9" s="1" t="inlineStr"/>
+      <c r="U9" s="1" t="inlineStr">
+        <is>
+          <t>Москва, Ижорская ул., 15с2</t>
+        </is>
+      </c>
       <c r="V9" s="1" t="inlineStr"/>
       <c r="W9" s="1" t="inlineStr"/>
       <c r="X9" s="1" t="inlineStr">
@@ -2152,7 +2184,11 @@
       </c>
       <c r="S10" s="1" t="inlineStr"/>
       <c r="T10" s="1" t="inlineStr"/>
-      <c r="U10" s="1" t="inlineStr"/>
+      <c r="U10" s="1" t="inlineStr">
+        <is>
+          <t>Москва, Ижорская ул., 15с2</t>
+        </is>
+      </c>
       <c r="V10" s="1" t="inlineStr"/>
       <c r="W10" s="1" t="inlineStr"/>
       <c r="X10" s="1" t="inlineStr">
@@ -2315,7 +2351,11 @@
       </c>
       <c r="S11" s="1" t="inlineStr"/>
       <c r="T11" s="1" t="inlineStr"/>
-      <c r="U11" s="1" t="inlineStr"/>
+      <c r="U11" s="1" t="inlineStr">
+        <is>
+          <t>Москва, Ижорская ул., 15с2</t>
+        </is>
+      </c>
       <c r="V11" s="1" t="inlineStr"/>
       <c r="W11" s="1" t="inlineStr"/>
       <c r="X11" s="1" t="inlineStr">

</xml_diff>

<commit_message>
Fix LeasingDiscount: it's a ruble amount, not a percentage
Real Avito validation error: "Значение должно быть не меньше 50000" —
the field expects an absolute minimum discount of 50,000 RUB, not a
percentage. Recomputed as 10% of each unit's price in rubles.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WGw8UdFgVU8PXaQaPUvEwH
</commit_message>
<xml_diff>
--- a/avito-feed-trailers/fleet-trailers.xlsx
+++ b/avito-feed-trailers/fleet-trailers.xlsx
@@ -1719,7 +1719,7 @@
       </c>
       <c r="AD7" s="1" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>325000</t>
         </is>
       </c>
       <c r="AE7" s="1" t="inlineStr"/>
@@ -1888,7 +1888,7 @@
       </c>
       <c r="AD8" s="1" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>296000</t>
         </is>
       </c>
       <c r="AE8" s="1" t="inlineStr"/>

</xml_diff>

<commit_message>
Rename Kassbohrer photo files to force fresh Avito re-download
Suspected root cause of "photos never update" complaints: Avito's
autoload likely caches images by URL, not by content hash. We had
been overwriting photo bytes at the exact same filenames (01.jpg,
02.jpg...) repeatedly today for VIN ...6344, ...4397 and ...4732 —
text fields (type/brakes/discount) reliably refreshed on reprocess,
but photos apparently did not, because the URL never changed.

Renamed all photos in these 3 folders to r2-NN.jpg (genuinely new
paths Avito has never fetched) and updated the JSON photo arrays to
match. This should force real re-downloads on the next sync.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WGw8UdFgVU8PXaQaPUvEwH
</commit_message>
<xml_diff>
--- a/avito-feed-trailers/fleet-trailers.xlsx
+++ b/avito-feed-trailers/fleet-trailers.xlsx
@@ -1157,7 +1157,7 @@
       <c r="Q4" s="1" t="inlineStr"/>
       <c r="R4" s="1" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00116344/01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00116344/02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00116344/03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00116344/04.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00116344/05.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00116344/06.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00116344/07.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00116344/08.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00116344/09.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00116344/10.jpg</t>
+          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00116344/r2-01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00116344/r2-02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00116344/r2-03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00116344/r2-04.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00116344/r2-05.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00116344/r2-06.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00116344/r2-07.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00116344/r2-08.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00116344/r2-09.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00116344/r2-10.jpg</t>
         </is>
       </c>
       <c r="S4" s="1" t="inlineStr"/>
@@ -1332,7 +1332,7 @@
       <c r="Q5" s="1" t="inlineStr"/>
       <c r="R5" s="1" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124397/01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124397/02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124397/03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124397/04.jpg</t>
+          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124397/r2-01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124397/r2-02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124397/r2-03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124397/r2-04.jpg</t>
         </is>
       </c>
       <c r="S5" s="1" t="inlineStr"/>
@@ -1507,7 +1507,7 @@
       <c r="Q6" s="1" t="inlineStr"/>
       <c r="R6" s="1" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124732/01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124732/02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124732/03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124732/04.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124732/05.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124732/06.jpg</t>
+          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124732/r2-01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124732/r2-02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124732/r2-03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124732/r2-04.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124732/r2-05.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/kassbohrer-maxima-shtor-00124732/r2-06.jpg</t>
         </is>
       </c>
       <c r="S6" s="1" t="inlineStr"/>

</xml_diff>

<commit_message>
Steelbear PL-24L (ea653666): switch to б/у в наличии, SAF axles, real VIN
Was listed as "под заказ"/new with BPW axles — corrected per Артём:
this is a real used unit in stock, SAF Heavy Duty axle assembly (not
BPW), VIN XWZ9412LLR1202021. Rewrote description to match used-listing
tone (dropped factory-order/warranty framing, added condition/VIN/
viewing lines matching the rest of the fleet).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WGw8UdFgVU8PXaQaPUvEwH
</commit_message>
<xml_diff>
--- a/avito-feed-trailers/fleet-trailers.xlsx
+++ b/avito-feed-trailers/fleet-trailers.xlsx
@@ -1994,12 +1994,14 @@
       </c>
       <c r="M9" s="1" t="inlineStr">
         <is>
-          <t>Полуприцеп-сортиментовоз Steelbear PL-24L (коммерческое название PT-24L BPW Heavy Duty), 2024 год выпуска, под заказ.
-Усиленное шасси из двутавровых лонжеронов, 3 оси BPW Heavy Duty, барабанные тормоза, пневмоподвеска с функцией подъём/опускание, допустимая нагрузка на ось 9 000 кг. Шины 385/65R22,5, односкат. Электронная тормозная система WABCO TEBS-E с функцией противоопрокидывания (RSS).
+          <t>Полуприцеп-сортиментовоз Steelbear PL-24L (коммерческое название PT-24L SAF Heavy Duty), 2024 год выпуска, б/у, в наличии.
+Усиленное шасси из двутавровых лонжеронов, 3 оси SAF Heavy Duty, барабанные тормоза, пневмоподвеска с функцией подъём/опускание, допустимая нагрузка на ось 9 000 кг. Шины 385/65R22,5, односкат. Электронная тормозная система WABCO TEBS-E с функцией противоопрокидывания (RSS).
 6 пар открепляемых коников грузоподъёмностью 8 тонн каждая (сталь STRENX 700MC), положение регулируется вдоль рамы. Внутренняя высота коника 2330 мм. Настил из ламинированной берёзовой фанеры. Опорное устройство BPW, 24 т.
 Максимальная полная масса 44 000 кг, грузоподъёмность 37 100 кг, длина 13 620 мм.
-Заводская гарантия — 24 месяца, от сквозной коррозии — 10 лет.
-Поставка под заказ, срок — уточняйте.</t>
+Техническое состояние — на ходу, полностью исправен, не требует вложений и ремонта.
+Документы в порядке.
+VIN XWZ9412LLR1202021.
+Смотровая площадка и показ — по договорённости. Торг при осмотре.</t>
         </is>
       </c>
       <c r="N9" s="1" t="inlineStr">
@@ -2051,7 +2053,7 @@
       </c>
       <c r="AC9" s="1" t="inlineStr">
         <is>
-          <t>Под заказ</t>
+          <t>В наличии</t>
         </is>
       </c>
       <c r="AD9" s="1" t="inlineStr"/>
@@ -2065,7 +2067,7 @@
       <c r="AL9" s="1" t="inlineStr"/>
       <c r="AM9" s="1" t="inlineStr">
         <is>
-          <t>Новое</t>
+          <t>С пробегом</t>
         </is>
       </c>
       <c r="AN9" s="1" t="inlineStr"/>
@@ -2096,7 +2098,11 @@
       </c>
       <c r="AT9" s="1" t="inlineStr"/>
       <c r="AU9" s="1" t="inlineStr"/>
-      <c r="AV9" s="1" t="inlineStr"/>
+      <c r="AV9" s="1" t="inlineStr">
+        <is>
+          <t>XWZ9412LLR1202021</t>
+        </is>
+      </c>
       <c r="AW9" s="1" t="inlineStr">
         <is>
           <t>2024</t>

</xml_diff>

<commit_message>
Remove VINs from listing descriptions (keep only in structural VIN field)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AHUm3FzH15mXN8Li2Qt4Qm
</commit_message>
<xml_diff>
--- a/avito-feed-trailers/fleet-trailers.xlsx
+++ b/avito-feed-trailers/fleet-trailers.xlsx
@@ -794,7 +794,6 @@
 4 оси (3 + выносная балансирная), тормоза дисковые, ABS SORL. Подвеска пневматическая, с функцией подъёма осей — меньше износ резины на порожняке и разворотах. Шины 385/55R22.5, комплект 8+1 запасное.
 Берёт контейнеры 20', 30', 40' и High Cube — под большинство стандартных грузоперевозок без переоборудования. Разрешённая максимальная масса 47 000 кг, грузоподъёмность 41 000 кг. Высота погрузки 1 100 мм.
 Инструментальный ящик Daken, полный комплект пневморазводки и ЭБС.
-VIN EAR853375R0000773.
 Возможна аренда с правом выкупа — уточняйте условия по телефону.</t>
         </is>
       </c>
@@ -2000,7 +1999,6 @@
 Максимальная полная масса 44 000 кг, грузоподъёмность 37 100 кг, длина 13 620 мм.
 Техническое состояние — на ходу, полностью исправен, не требует вложений и ремонта.
 Документы в порядке.
-VIN XWZ9412LLR1202021.
 Смотровая площадка и показ — по договорённости. Торг при осмотре.</t>
         </is>
       </c>
@@ -2167,7 +2165,6 @@
           <t>Полуприцеп-контейнеровоз Тонар К4-U (99891), 2023 год, в работе, полностью исправен.
 4 оси: тройная задняя тележка плюс вынесенная вперёд ось — меньше нагрузка на дорогу и мягче по осевым ограничениям в городе. Тормоза дисковые, пневмопривод. Подвеска зависимая, на продольных рычагах, с пневмоэлементами и телескопическими амортизаторами. Шины 385/55R22.5, односкатные.
 Берёт контейнеры 20', 2×20', 30', 30' HC, 40', 40' HC. Разрешённая максимальная масса 44 000 кг, грузоподъёмность 37 800 кг, нагрузка на ССУ 11 000 кг. Высота ССУ 1 100 мм.
-VIN X0T998910P0002033.
 Возможна аренда с правом выкупа — уточняйте условия по телефону.</t>
         </is>
       </c>
@@ -2334,7 +2331,6 @@
           <t>Шторный полуприцеп V-Trailer 329D, 2023 год, в работе, полностью исправен.
 Оси SAF, подъёмная передняя — меньше износ резины и расход на порожняке. Опорное устройство JOST на 24 тонны, шкворень 2 дюйма по ISO 1726. Пол — влагостойкая фанера 30 мм, держит погрузчик до 7,5 тонн. Крыша сдвижная (Sesam/Edscha) — грузить сверху краном или погрузчиком без снятия тента. Двери алюминиевые BPW Smartmaster II, передний и задний портал — стальные, собственной конструкции. Рама облегчённая, с дополнительными усилениями против скручивания. По бортам — корзины под коники, по 7 штук на сторону.
 13,6 × 2,5 × 4 м, 91 м³. Тент плотный: борта 900 г/м², крыша 680 г/м². Полная штора, без бортов — удобно под европаллеты и груз с выступом по высоте.
-VIN XZFVKRP3DR0000119.
 Возможна аренда с правом выкупа — уточняйте условия по телефону.</t>
         </is>
       </c>

</xml_diff>

<commit_message>
Update InterPricep 853375 price to 1,890,000
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AHUm3FzH15mXN8Li2Qt4Qm
</commit_message>
<xml_diff>
--- a/avito-feed-trailers/fleet-trailers.xlsx
+++ b/avito-feed-trailers/fleet-trailers.xlsx
@@ -804,7 +804,7 @@
       </c>
       <c r="O2" s="1" t="inlineStr">
         <is>
-          <t>1390000</t>
+          <t>1890000</t>
         </is>
       </c>
       <c r="P2" s="1" t="inlineStr"/>
@@ -841,7 +841,7 @@
       <c r="AA2" s="1" t="inlineStr"/>
       <c r="AB2" s="1" t="inlineStr">
         <is>
-          <t>1390000</t>
+          <t>1890000</t>
         </is>
       </c>
       <c r="AC2" s="1" t="inlineStr">

</xml_diff>

<commit_message>
Add 7 new Tonar equipment listings across categories (under-order, official price list)
Бортовой B3-13, шторный T3-13, контейнеровоз K4-U 99891 (новый, под заказ,
отдельно от б/у в наличии), сортиментовоз L3, самосвальный 9595, зерновоз
95941, щеповоз SDP4-89. Плюс рефрижератор R3-13 под заказ (с холодильной
установкой) — используем официальное значение "Рефрижератор" из справочника
Авито, отдельное от "Изотермический".

Цены по прайсу Тонара от 27.07.2026, две скидки указаны раздельно в полях
Авито (Скидка от дилера + Скидка за лизинг) и в тексте описания: скидка от
производителя (10% борт+шторн, 5% контейнеровоз+лесовоз) и субсидия лизинга
от Минпромторга (10%, не более 500 000₽). Добавлено поле "Скидка от дилера"
в generate_feed.py — было в схеме HEADERS, но не подключено.

Все модели сверены дословно с avito_trailer_make_model_catalog.xml.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AHUm3FzH15mXN8Li2Qt4Qm
</commit_message>
<xml_diff>
--- a/avito-feed-trailers/fleet-trailers.xlsx
+++ b/avito-feed-trailers/fleet-trailers.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BE11"/>
+  <dimension ref="A1:BE19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -459,7 +459,7 @@
     <col width="10" customWidth="1" min="40" max="40"/>
     <col width="13" customWidth="1" min="41" max="41"/>
     <col width="13" customWidth="1" min="42" max="42"/>
-    <col width="14" customWidth="1" min="43" max="43"/>
+    <col width="17" customWidth="1" min="43" max="43"/>
     <col width="13" customWidth="1" min="44" max="44"/>
     <col width="25" customWidth="1" min="45" max="45"/>
     <col width="11" customWidth="1" min="46" max="46"/>
@@ -2145,7 +2145,7 @@
       <c r="C10" s="1" t="inlineStr"/>
       <c r="D10" s="1" t="inlineStr">
         <is>
-          <t>tonar-k4u-p0002033</t>
+          <t>tonar-b313-9888</t>
         </is>
       </c>
       <c r="E10" s="1" t="inlineStr"/>
@@ -2162,10 +2162,12 @@
       </c>
       <c r="M10" s="1" t="inlineStr">
         <is>
-          <t>Полуприцеп-контейнеровоз Тонар К4-U (99891), 2023 год, в работе, полностью исправен.
-4 оси: тройная задняя тележка плюс вынесенная вперёд ось — меньше нагрузка на дорогу и мягче по осевым ограничениям в городе. Тормоза дисковые, пневмопривод. Подвеска зависимая, на продольных рычагах, с пневмоэлементами и телескопическими амортизаторами. Шины 385/55R22.5, односкатные.
-Берёт контейнеры 20', 2×20', 30', 30' HC, 40', 40' HC. Разрешённая максимальная масса 44 000 кг, грузоподъёмность 37 800 кг, нагрузка на ССУ 11 000 кг. Высота ССУ 1 100 мм.
-Возможна аренда с правом выкупа — уточняйте условия по телефону.</t>
+          <t>Полуприцеп бортовой Тонар B3-13 (9888), 13,6 м, трёхосный, первая ось подъёмная — меньше износ резины на порожняке. ССУ 1200 мм, со стаканами под коники (коники в комплект не входят). Новое, под заказ у завода-изготовителя.
+Цена по действующему прайсу завода (с 27.07.2026): 3 150 000 ₽.
+Скидка от производителя на линейку бортовых прицепов (10%): −315 000 ₽.
+При покупке в лизинг — дополнительная субсидия от Минпромторга (10%, не более 500 000 ₽): −315 000 ₽.
+Итоговая цена при лизинге: 2 520 000 ₽.
+Заводская гарантия — 12 месяцев. Поставка после согласования комплектации.</t>
         </is>
       </c>
       <c r="N10" s="1" t="inlineStr">
@@ -2175,14 +2177,14 @@
       </c>
       <c r="O10" s="1" t="inlineStr">
         <is>
-          <t>1690000</t>
+          <t>3150000</t>
         </is>
       </c>
       <c r="P10" s="1" t="inlineStr"/>
       <c r="Q10" s="1" t="inlineStr"/>
       <c r="R10" s="1" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-p0002033/01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-p0002033/02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-p0002033/03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-p0002033/04.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-p0002033/05.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-p0002033/06.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-p0002033/07.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-p0002033/08.jpg</t>
+          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-b313-9888/01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-b313-9888/02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-b313-9888/03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-b313-9888/04.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-b313-9888/05.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-b313-9888/06.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-b313-9888/07.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-b313-9888/08.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-b313-9888/09.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-b313-9888/10.jpg</t>
         </is>
       </c>
       <c r="S10" s="1" t="inlineStr"/>
@@ -2212,17 +2214,25 @@
       <c r="AA10" s="1" t="inlineStr"/>
       <c r="AB10" s="1" t="inlineStr">
         <is>
-          <t>1690000</t>
+          <t>3150000</t>
         </is>
       </c>
       <c r="AC10" s="1" t="inlineStr">
         <is>
-          <t>В наличии</t>
-        </is>
-      </c>
-      <c r="AD10" s="1" t="inlineStr"/>
+          <t>Под заказ</t>
+        </is>
+      </c>
+      <c r="AD10" s="1" t="inlineStr">
+        <is>
+          <t>315000</t>
+        </is>
+      </c>
       <c r="AE10" s="1" t="inlineStr"/>
-      <c r="AF10" s="1" t="inlineStr"/>
+      <c r="AF10" s="1" t="inlineStr">
+        <is>
+          <t>315000</t>
+        </is>
+      </c>
       <c r="AG10" s="1" t="inlineStr"/>
       <c r="AH10" s="1" t="inlineStr"/>
       <c r="AI10" s="1" t="inlineStr"/>
@@ -2231,7 +2241,7 @@
       <c r="AL10" s="1" t="inlineStr"/>
       <c r="AM10" s="1" t="inlineStr">
         <is>
-          <t>С пробегом</t>
+          <t>Новое</t>
         </is>
       </c>
       <c r="AN10" s="1" t="inlineStr"/>
@@ -2247,7 +2257,7 @@
       </c>
       <c r="AQ10" s="1" t="inlineStr">
         <is>
-          <t>K4-U (99891)</t>
+          <t>B3-13 (9888)</t>
         </is>
       </c>
       <c r="AR10" s="1" t="inlineStr">
@@ -2257,24 +2267,20 @@
       </c>
       <c r="AS10" s="1" t="inlineStr">
         <is>
-          <t>Контейнеровоз</t>
+          <t>Бортовой</t>
         </is>
       </c>
       <c r="AT10" s="1" t="inlineStr"/>
       <c r="AU10" s="1" t="inlineStr"/>
-      <c r="AV10" s="1" t="inlineStr">
-        <is>
-          <t>X0T998910P0002033</t>
-        </is>
-      </c>
+      <c r="AV10" s="1" t="inlineStr"/>
       <c r="AW10" s="1" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="AX10" s="1" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="AY10" s="1" t="inlineStr">
@@ -2287,14 +2293,10 @@
           <t>Дисковые</t>
         </is>
       </c>
-      <c r="BA10" s="1" t="inlineStr">
-        <is>
-          <t>37800</t>
-        </is>
-      </c>
+      <c r="BA10" s="1" t="inlineStr"/>
       <c r="BB10" s="1" t="inlineStr">
         <is>
-          <t>12725</t>
+          <t>13600</t>
         </is>
       </c>
       <c r="BC10" s="1" t="inlineStr"/>
@@ -2311,7 +2313,7 @@
       <c r="C11" s="1" t="inlineStr"/>
       <c r="D11" s="1" t="inlineStr">
         <is>
-          <t>v-trailer-329d-r0000119</t>
+          <t>tonar-k4u-99891-order</t>
         </is>
       </c>
       <c r="E11" s="1" t="inlineStr"/>
@@ -2328,10 +2330,13 @@
       </c>
       <c r="M11" s="1" t="inlineStr">
         <is>
-          <t>Шторный полуприцеп V-Trailer 329D, 2023 год, в работе, полностью исправен.
-Оси SAF, подъёмная передняя — меньше износ резины и расход на порожняке. Опорное устройство JOST на 24 тонны, шкворень 2 дюйма по ISO 1726. Пол — влагостойкая фанера 30 мм, держит погрузчик до 7,5 тонн. Крыша сдвижная (Sesam/Edscha) — грузить сверху краном или погрузчиком без снятия тента. Двери алюминиевые BPW Smartmaster II, передний и задний портал — стальные, собственной конструкции. Рама облегчённая, с дополнительными усилениями против скручивания. По бортам — корзины под коники, по 7 штук на сторону.
-13,6 × 2,5 × 4 м, 91 м³. Тент плотный: борта 900 г/м², крыша 680 г/м². Полная штора, без бортов — удобно под европаллеты и груз с выступом по высоте.
-Возможна аренда с правом выкупа — уточняйте условия по телефону.</t>
+          <t>Полуприцеп контейнеровоз Тонар K4-U (99891), 4 оси, вынесенная вперёд передняя ось на 2560 мм — меньше нагрузка на дорогу. ССУ=1100 мм, шины 385/55-R22.5. Берёт контейнеры 1×20', 2×20', 1×30', 1×40' High Cube. Новое, под заказ у завода-изготовителя.
+Цена по действующему прайсу завода (с 27.07.2026): 3 200 000 ₽.
+Скидка от производителя на линейку контейнеровозов (5%): −160 000 ₽.
+При покупке в лизинг — дополнительная субсидия от Минпромторга (10%, не более 500 000 ₽): −320 000 ₽.
+Итоговая цена при лизинге: 2 720 000 ₽.
+Заводская гарантия — 12 месяцев. Поставка после согласования комплектации.
+(У нас также есть эта же модель б/у, в наличии, дешевле — уточняйте по телефону, если новый под заказ не подходит по срокам.)</t>
         </is>
       </c>
       <c r="N11" s="1" t="inlineStr">
@@ -2341,14 +2346,14 @@
       </c>
       <c r="O11" s="1" t="inlineStr">
         <is>
-          <t>2990000</t>
+          <t>3200000</t>
         </is>
       </c>
       <c r="P11" s="1" t="inlineStr"/>
       <c r="Q11" s="1" t="inlineStr"/>
       <c r="R11" s="1" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/r2-01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/r2-02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/r2-03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/r2-04.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/r2-05.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/r2-06.jpg</t>
+          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-99891-order/01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-99891-order/02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-99891-order/03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-99891-order/04.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-99891-order/05.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-99891-order/06.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-99891-order/07.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-99891-order/08.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-99891-order/09.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-99891-order/10.jpg</t>
         </is>
       </c>
       <c r="S11" s="1" t="inlineStr"/>
@@ -2378,17 +2383,25 @@
       <c r="AA11" s="1" t="inlineStr"/>
       <c r="AB11" s="1" t="inlineStr">
         <is>
-          <t>2990000</t>
+          <t>3200000</t>
         </is>
       </c>
       <c r="AC11" s="1" t="inlineStr">
         <is>
-          <t>В наличии</t>
-        </is>
-      </c>
-      <c r="AD11" s="1" t="inlineStr"/>
+          <t>Под заказ</t>
+        </is>
+      </c>
+      <c r="AD11" s="1" t="inlineStr">
+        <is>
+          <t>320000</t>
+        </is>
+      </c>
       <c r="AE11" s="1" t="inlineStr"/>
-      <c r="AF11" s="1" t="inlineStr"/>
+      <c r="AF11" s="1" t="inlineStr">
+        <is>
+          <t>160000</t>
+        </is>
+      </c>
       <c r="AG11" s="1" t="inlineStr"/>
       <c r="AH11" s="1" t="inlineStr"/>
       <c r="AI11" s="1" t="inlineStr"/>
@@ -2397,7 +2410,7 @@
       <c r="AL11" s="1" t="inlineStr"/>
       <c r="AM11" s="1" t="inlineStr">
         <is>
-          <t>С пробегом</t>
+          <t>Новое</t>
         </is>
       </c>
       <c r="AN11" s="1" t="inlineStr"/>
@@ -2408,12 +2421,12 @@
       </c>
       <c r="AP11" s="1" t="inlineStr">
         <is>
-          <t>V-Trailer</t>
+          <t>Тонар</t>
         </is>
       </c>
       <c r="AQ11" s="1" t="inlineStr">
         <is>
-          <t>329</t>
+          <t>K4-U (99891)</t>
         </is>
       </c>
       <c r="AR11" s="1" t="inlineStr">
@@ -2423,29 +2436,25 @@
       </c>
       <c r="AS11" s="1" t="inlineStr">
         <is>
-          <t>Шторный</t>
+          <t>Контейнеровоз</t>
         </is>
       </c>
       <c r="AT11" s="1" t="inlineStr"/>
       <c r="AU11" s="1" t="inlineStr"/>
-      <c r="AV11" s="1" t="inlineStr">
-        <is>
-          <t>XZFVKRP3DR0000119</t>
-        </is>
-      </c>
+      <c r="AV11" s="1" t="inlineStr"/>
       <c r="AW11" s="1" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="AX11" s="1" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AY11" s="1" t="inlineStr">
         <is>
-          <t>Пневматическая</t>
+          <t>Рессорная</t>
         </is>
       </c>
       <c r="AZ11" s="1" t="inlineStr">
@@ -2453,23 +2462,1337 @@
           <t>Дисковые</t>
         </is>
       </c>
-      <c r="BA11" s="1" t="inlineStr">
-        <is>
-          <t>32300</t>
-        </is>
-      </c>
+      <c r="BA11" s="1" t="inlineStr"/>
       <c r="BB11" s="1" t="inlineStr">
         <is>
-          <t>13600</t>
-        </is>
-      </c>
-      <c r="BC11" s="1" t="inlineStr">
-        <is>
-          <t>91</t>
-        </is>
-      </c>
+          <t>12725</t>
+        </is>
+      </c>
+      <c r="BC11" s="1" t="inlineStr"/>
       <c r="BD11" s="1" t="inlineStr"/>
       <c r="BE11" s="1" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>Москва, Ижорская ул., 15с2</t>
+        </is>
+      </c>
+      <c r="B12" s="1" t="inlineStr"/>
+      <c r="C12" s="1" t="inlineStr"/>
+      <c r="D12" s="1" t="inlineStr">
+        <is>
+          <t>tonar-k4u-p0002033</t>
+        </is>
+      </c>
+      <c r="E12" s="1" t="inlineStr"/>
+      <c r="F12" s="1" t="inlineStr"/>
+      <c r="G12" s="1" t="inlineStr"/>
+      <c r="H12" s="1" t="inlineStr"/>
+      <c r="I12" s="1" t="inlineStr"/>
+      <c r="J12" s="1" t="inlineStr"/>
+      <c r="K12" s="1" t="inlineStr"/>
+      <c r="L12" s="1" t="inlineStr">
+        <is>
+          <t>По телефону и в сообщениях</t>
+        </is>
+      </c>
+      <c r="M12" s="1" t="inlineStr">
+        <is>
+          <t>Полуприцеп-контейнеровоз Тонар К4-U (99891), 2023 год, в работе, полностью исправен.
+4 оси: тройная задняя тележка плюс вынесенная вперёд ось — меньше нагрузка на дорогу и мягче по осевым ограничениям в городе. Тормоза дисковые, пневмопривод. Подвеска зависимая, на продольных рычагах, с пневмоэлементами и телескопическими амортизаторами. Шины 385/55R22.5, односкатные.
+Берёт контейнеры 20', 2×20', 30', 30' HC, 40', 40' HC. Разрешённая максимальная масса 44 000 кг, грузоподъёмность 37 800 кг, нагрузка на ССУ 11 000 кг. Высота ССУ 1 100 мм.
+Возможна аренда с правом выкупа — уточняйте условия по телефону.</t>
+        </is>
+      </c>
+      <c r="N12" s="1" t="inlineStr">
+        <is>
+          <t>Грузовики и спецтехника</t>
+        </is>
+      </c>
+      <c r="O12" s="1" t="inlineStr">
+        <is>
+          <t>1690000</t>
+        </is>
+      </c>
+      <c r="P12" s="1" t="inlineStr"/>
+      <c r="Q12" s="1" t="inlineStr"/>
+      <c r="R12" s="1" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-p0002033/01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-p0002033/02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-p0002033/03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-p0002033/04.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-p0002033/05.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-p0002033/06.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-p0002033/07.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-p0002033/08.jpg</t>
+        </is>
+      </c>
+      <c r="S12" s="1" t="inlineStr"/>
+      <c r="T12" s="1" t="inlineStr"/>
+      <c r="U12" s="1" t="inlineStr">
+        <is>
+          <t>Москва, Ижорская ул., 15с2</t>
+        </is>
+      </c>
+      <c r="V12" s="1" t="inlineStr"/>
+      <c r="W12" s="1" t="inlineStr"/>
+      <c r="X12" s="1" t="inlineStr">
+        <is>
+          <t>Прицепы</t>
+        </is>
+      </c>
+      <c r="Y12" s="1" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="Z12" s="1" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="AA12" s="1" t="inlineStr"/>
+      <c r="AB12" s="1" t="inlineStr">
+        <is>
+          <t>1690000</t>
+        </is>
+      </c>
+      <c r="AC12" s="1" t="inlineStr">
+        <is>
+          <t>В наличии</t>
+        </is>
+      </c>
+      <c r="AD12" s="1" t="inlineStr"/>
+      <c r="AE12" s="1" t="inlineStr"/>
+      <c r="AF12" s="1" t="inlineStr"/>
+      <c r="AG12" s="1" t="inlineStr"/>
+      <c r="AH12" s="1" t="inlineStr"/>
+      <c r="AI12" s="1" t="inlineStr"/>
+      <c r="AJ12" s="1" t="inlineStr"/>
+      <c r="AK12" s="1" t="inlineStr"/>
+      <c r="AL12" s="1" t="inlineStr"/>
+      <c r="AM12" s="1" t="inlineStr">
+        <is>
+          <t>С пробегом</t>
+        </is>
+      </c>
+      <c r="AN12" s="1" t="inlineStr"/>
+      <c r="AO12" s="1" t="inlineStr">
+        <is>
+          <t>В наличии</t>
+        </is>
+      </c>
+      <c r="AP12" s="1" t="inlineStr">
+        <is>
+          <t>Тонар</t>
+        </is>
+      </c>
+      <c r="AQ12" s="1" t="inlineStr">
+        <is>
+          <t>K4-U (99891)</t>
+        </is>
+      </c>
+      <c r="AR12" s="1" t="inlineStr">
+        <is>
+          <t>Полуприцеп</t>
+        </is>
+      </c>
+      <c r="AS12" s="1" t="inlineStr">
+        <is>
+          <t>Контейнеровоз</t>
+        </is>
+      </c>
+      <c r="AT12" s="1" t="inlineStr"/>
+      <c r="AU12" s="1" t="inlineStr"/>
+      <c r="AV12" s="1" t="inlineStr">
+        <is>
+          <t>X0T998910P0002033</t>
+        </is>
+      </c>
+      <c r="AW12" s="1" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="AX12" s="1" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AY12" s="1" t="inlineStr">
+        <is>
+          <t>Рессорная</t>
+        </is>
+      </c>
+      <c r="AZ12" s="1" t="inlineStr">
+        <is>
+          <t>Дисковые</t>
+        </is>
+      </c>
+      <c r="BA12" s="1" t="inlineStr">
+        <is>
+          <t>37800</t>
+        </is>
+      </c>
+      <c r="BB12" s="1" t="inlineStr">
+        <is>
+          <t>12725</t>
+        </is>
+      </c>
+      <c r="BC12" s="1" t="inlineStr"/>
+      <c r="BD12" s="1" t="inlineStr"/>
+      <c r="BE12" s="1" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="inlineStr">
+        <is>
+          <t>Москва, Ижорская ул., 15с2</t>
+        </is>
+      </c>
+      <c r="B13" s="1" t="inlineStr"/>
+      <c r="C13" s="1" t="inlineStr"/>
+      <c r="D13" s="1" t="inlineStr">
+        <is>
+          <t>tonar-l3-9445</t>
+        </is>
+      </c>
+      <c r="E13" s="1" t="inlineStr"/>
+      <c r="F13" s="1" t="inlineStr"/>
+      <c r="G13" s="1" t="inlineStr"/>
+      <c r="H13" s="1" t="inlineStr"/>
+      <c r="I13" s="1" t="inlineStr"/>
+      <c r="J13" s="1" t="inlineStr"/>
+      <c r="K13" s="1" t="inlineStr"/>
+      <c r="L13" s="1" t="inlineStr">
+        <is>
+          <t>По телефону и в сообщениях</t>
+        </is>
+      </c>
+      <c r="M13" s="1" t="inlineStr">
+        <is>
+          <t>Полуприцеп-сортиментовоз Тонар L3 (9445), 3 оси, ССУ 1150/1250/1350 мм с подъёмной осью — меньше износ на порожняке. Коники разборные, 6 штук, межосевое расстояние 1310 мм, рычажная подвеска, барабанные тормоза. Новое, под заказ у завода-изготовителя.
+Цена по действующему прайсу завода (с 27.07.2026): 3 200 000 ₽.
+Скидка от производителя на линейку лесовозов (5%): −160 000 ₽.
+При покупке в лизинг — дополнительная субсидия от Минпромторга (10%, не более 500 000 ₽): −320 000 ₽.
+Итоговая цена при лизинге: 2 720 000 ₽.
+Заводская гарантия — 12 месяцев. Поставка после согласования комплектации.</t>
+        </is>
+      </c>
+      <c r="N13" s="1" t="inlineStr">
+        <is>
+          <t>Грузовики и спецтехника</t>
+        </is>
+      </c>
+      <c r="O13" s="1" t="inlineStr">
+        <is>
+          <t>3200000</t>
+        </is>
+      </c>
+      <c r="P13" s="1" t="inlineStr"/>
+      <c r="Q13" s="1" t="inlineStr"/>
+      <c r="R13" s="1" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-l3-9445/01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-l3-9445/02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-l3-9445/03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-l3-9445/04.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-l3-9445/05.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-l3-9445/06.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-l3-9445/07.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-l3-9445/08.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-l3-9445/09.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-l3-9445/10.jpg</t>
+        </is>
+      </c>
+      <c r="S13" s="1" t="inlineStr"/>
+      <c r="T13" s="1" t="inlineStr"/>
+      <c r="U13" s="1" t="inlineStr">
+        <is>
+          <t>Москва, Ижорская ул., 15с2</t>
+        </is>
+      </c>
+      <c r="V13" s="1" t="inlineStr"/>
+      <c r="W13" s="1" t="inlineStr"/>
+      <c r="X13" s="1" t="inlineStr">
+        <is>
+          <t>Прицепы</t>
+        </is>
+      </c>
+      <c r="Y13" s="1" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="Z13" s="1" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="AA13" s="1" t="inlineStr"/>
+      <c r="AB13" s="1" t="inlineStr">
+        <is>
+          <t>3200000</t>
+        </is>
+      </c>
+      <c r="AC13" s="1" t="inlineStr">
+        <is>
+          <t>Под заказ</t>
+        </is>
+      </c>
+      <c r="AD13" s="1" t="inlineStr">
+        <is>
+          <t>320000</t>
+        </is>
+      </c>
+      <c r="AE13" s="1" t="inlineStr"/>
+      <c r="AF13" s="1" t="inlineStr">
+        <is>
+          <t>160000</t>
+        </is>
+      </c>
+      <c r="AG13" s="1" t="inlineStr"/>
+      <c r="AH13" s="1" t="inlineStr"/>
+      <c r="AI13" s="1" t="inlineStr"/>
+      <c r="AJ13" s="1" t="inlineStr"/>
+      <c r="AK13" s="1" t="inlineStr"/>
+      <c r="AL13" s="1" t="inlineStr"/>
+      <c r="AM13" s="1" t="inlineStr">
+        <is>
+          <t>Новое</t>
+        </is>
+      </c>
+      <c r="AN13" s="1" t="inlineStr"/>
+      <c r="AO13" s="1" t="inlineStr">
+        <is>
+          <t>В наличии</t>
+        </is>
+      </c>
+      <c r="AP13" s="1" t="inlineStr">
+        <is>
+          <t>Тонар</t>
+        </is>
+      </c>
+      <c r="AQ13" s="1" t="inlineStr">
+        <is>
+          <t>L3 (9445)</t>
+        </is>
+      </c>
+      <c r="AR13" s="1" t="inlineStr">
+        <is>
+          <t>Полуприцеп</t>
+        </is>
+      </c>
+      <c r="AS13" s="1" t="inlineStr">
+        <is>
+          <t>Лесовоз (сортиментовоз)</t>
+        </is>
+      </c>
+      <c r="AT13" s="1" t="inlineStr"/>
+      <c r="AU13" s="1" t="inlineStr"/>
+      <c r="AV13" s="1" t="inlineStr"/>
+      <c r="AW13" s="1" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="AX13" s="1" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AY13" s="1" t="inlineStr">
+        <is>
+          <t>Рессорная</t>
+        </is>
+      </c>
+      <c r="AZ13" s="1" t="inlineStr">
+        <is>
+          <t>Барабанные</t>
+        </is>
+      </c>
+      <c r="BA13" s="1" t="inlineStr"/>
+      <c r="BB13" s="1" t="inlineStr"/>
+      <c r="BC13" s="1" t="inlineStr"/>
+      <c r="BD13" s="1" t="inlineStr"/>
+      <c r="BE13" s="1" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>Москва, Ижорская ул., 15с2</t>
+        </is>
+      </c>
+      <c r="B14" s="1" t="inlineStr"/>
+      <c r="C14" s="1" t="inlineStr"/>
+      <c r="D14" s="1" t="inlineStr">
+        <is>
+          <t>tonar-reef-r313</t>
+        </is>
+      </c>
+      <c r="E14" s="1" t="inlineStr"/>
+      <c r="F14" s="1" t="inlineStr"/>
+      <c r="G14" s="1" t="inlineStr"/>
+      <c r="H14" s="1" t="inlineStr"/>
+      <c r="I14" s="1" t="inlineStr"/>
+      <c r="J14" s="1" t="inlineStr"/>
+      <c r="K14" s="1" t="inlineStr"/>
+      <c r="L14" s="1" t="inlineStr">
+        <is>
+          <t>По телефону и в сообщениях</t>
+        </is>
+      </c>
+      <c r="M14" s="1" t="inlineStr">
+        <is>
+          <t>Полуприцеп рефрижератор Тонар R3-13, 13,6 м, трёхосный, первая ось подъёмная, объём кузова 85 м³, дисковые оси, ССУ-1150 мм, вместимость 33 европаллеты. Новое, под заказ у завода-изготовителя.
+В отличие от обычного изотермического кузова (без активного охлаждения), этот прицеп доукомплектован новой холодильно-отопительной установкой (ХОУ) — держит заданную температуру в пути, не только теплоизолирует. Именно установка ХОУ и делает цену заметно выше базового изотермического кузова той же длины (у нас в парке такой есть от 4 850 000 ₽ по прайсу завода без холодильной установки).
+Цена: 7 000 000 ₽ (на эту линейку скидка от производителя не действует).
+При покупке в лизинг — субсидия от Минпромторга (10%, не более 500 000 ₽): −500 000 ₽.
+Итоговая цена при лизинге: 6 500 000 ₽.
+Заводская гарантия — 12 месяцев. Поставка после согласования комплектации.</t>
+        </is>
+      </c>
+      <c r="N14" s="1" t="inlineStr">
+        <is>
+          <t>Грузовики и спецтехника</t>
+        </is>
+      </c>
+      <c r="O14" s="1" t="inlineStr">
+        <is>
+          <t>7000000</t>
+        </is>
+      </c>
+      <c r="P14" s="1" t="inlineStr"/>
+      <c r="Q14" s="1" t="inlineStr"/>
+      <c r="R14" s="1" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-reef-r313/01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-reef-r313/02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-reef-r313/03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-reef-r313/04.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-reef-r313/05.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-reef-r313/06.jpg</t>
+        </is>
+      </c>
+      <c r="S14" s="1" t="inlineStr"/>
+      <c r="T14" s="1" t="inlineStr"/>
+      <c r="U14" s="1" t="inlineStr">
+        <is>
+          <t>Москва, Ижорская ул., 15с2</t>
+        </is>
+      </c>
+      <c r="V14" s="1" t="inlineStr"/>
+      <c r="W14" s="1" t="inlineStr"/>
+      <c r="X14" s="1" t="inlineStr">
+        <is>
+          <t>Прицепы</t>
+        </is>
+      </c>
+      <c r="Y14" s="1" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="Z14" s="1" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="AA14" s="1" t="inlineStr"/>
+      <c r="AB14" s="1" t="inlineStr">
+        <is>
+          <t>7000000</t>
+        </is>
+      </c>
+      <c r="AC14" s="1" t="inlineStr">
+        <is>
+          <t>Под заказ</t>
+        </is>
+      </c>
+      <c r="AD14" s="1" t="inlineStr">
+        <is>
+          <t>500000</t>
+        </is>
+      </c>
+      <c r="AE14" s="1" t="inlineStr"/>
+      <c r="AF14" s="1" t="inlineStr"/>
+      <c r="AG14" s="1" t="inlineStr"/>
+      <c r="AH14" s="1" t="inlineStr"/>
+      <c r="AI14" s="1" t="inlineStr"/>
+      <c r="AJ14" s="1" t="inlineStr"/>
+      <c r="AK14" s="1" t="inlineStr"/>
+      <c r="AL14" s="1" t="inlineStr"/>
+      <c r="AM14" s="1" t="inlineStr">
+        <is>
+          <t>Новое</t>
+        </is>
+      </c>
+      <c r="AN14" s="1" t="inlineStr"/>
+      <c r="AO14" s="1" t="inlineStr">
+        <is>
+          <t>В наличии</t>
+        </is>
+      </c>
+      <c r="AP14" s="1" t="inlineStr">
+        <is>
+          <t>Тонар</t>
+        </is>
+      </c>
+      <c r="AQ14" s="1" t="inlineStr">
+        <is>
+          <t>R3-13</t>
+        </is>
+      </c>
+      <c r="AR14" s="1" t="inlineStr">
+        <is>
+          <t>Полуприцеп</t>
+        </is>
+      </c>
+      <c r="AS14" s="1" t="inlineStr">
+        <is>
+          <t>Рефрижератор</t>
+        </is>
+      </c>
+      <c r="AT14" s="1" t="inlineStr"/>
+      <c r="AU14" s="1" t="inlineStr"/>
+      <c r="AV14" s="1" t="inlineStr"/>
+      <c r="AW14" s="1" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="AX14" s="1" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AY14" s="1" t="inlineStr">
+        <is>
+          <t>Рессорная</t>
+        </is>
+      </c>
+      <c r="AZ14" s="1" t="inlineStr">
+        <is>
+          <t>Дисковые</t>
+        </is>
+      </c>
+      <c r="BA14" s="1" t="inlineStr"/>
+      <c r="BB14" s="1" t="inlineStr">
+        <is>
+          <t>13600</t>
+        </is>
+      </c>
+      <c r="BC14" s="1" t="inlineStr">
+        <is>
+          <t>85</t>
+        </is>
+      </c>
+      <c r="BD14" s="1" t="inlineStr"/>
+      <c r="BE14" s="1" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>Москва, Ижорская ул., 15с2</t>
+        </is>
+      </c>
+      <c r="B15" s="1" t="inlineStr"/>
+      <c r="C15" s="1" t="inlineStr"/>
+      <c r="D15" s="1" t="inlineStr">
+        <is>
+          <t>tonar-samosval-9595</t>
+        </is>
+      </c>
+      <c r="E15" s="1" t="inlineStr"/>
+      <c r="F15" s="1" t="inlineStr"/>
+      <c r="G15" s="1" t="inlineStr"/>
+      <c r="H15" s="1" t="inlineStr"/>
+      <c r="I15" s="1" t="inlineStr"/>
+      <c r="J15" s="1" t="inlineStr"/>
+      <c r="K15" s="1" t="inlineStr"/>
+      <c r="L15" s="1" t="inlineStr">
+        <is>
+          <t>По телефону и в сообщениях</t>
+        </is>
+      </c>
+      <c r="M15" s="1" t="inlineStr">
+        <is>
+          <t>Полуприцеп самосвальный Тонар 9595, четырёхосный, тент с боковым намотом, рычажная подвеска, дисковые тормоза. Новое, под заказ у завода-изготовителя.
+Цена: 4 200 000 ₽ (на линейку самосвальных полуприцепов скидка от производителя не действует).
+При покупке в лизинг — субсидия от Минпромторга (10%, не более 500 000 ₽): −420 000 ₽.
+Итоговая цена при лизинге: 3 780 000 ₽.
+Заводская гарантия — 12 месяцев. Точную комплектацию (объём кузова, борта) уточняйте при заказе.</t>
+        </is>
+      </c>
+      <c r="N15" s="1" t="inlineStr">
+        <is>
+          <t>Грузовики и спецтехника</t>
+        </is>
+      </c>
+      <c r="O15" s="1" t="inlineStr">
+        <is>
+          <t>4200000</t>
+        </is>
+      </c>
+      <c r="P15" s="1" t="inlineStr"/>
+      <c r="Q15" s="1" t="inlineStr"/>
+      <c r="R15" s="1" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-samosval-9595/01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-samosval-9595/02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-samosval-9595/03.jpg</t>
+        </is>
+      </c>
+      <c r="S15" s="1" t="inlineStr"/>
+      <c r="T15" s="1" t="inlineStr"/>
+      <c r="U15" s="1" t="inlineStr">
+        <is>
+          <t>Москва, Ижорская ул., 15с2</t>
+        </is>
+      </c>
+      <c r="V15" s="1" t="inlineStr"/>
+      <c r="W15" s="1" t="inlineStr"/>
+      <c r="X15" s="1" t="inlineStr">
+        <is>
+          <t>Прицепы</t>
+        </is>
+      </c>
+      <c r="Y15" s="1" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="Z15" s="1" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="AA15" s="1" t="inlineStr"/>
+      <c r="AB15" s="1" t="inlineStr">
+        <is>
+          <t>4200000</t>
+        </is>
+      </c>
+      <c r="AC15" s="1" t="inlineStr">
+        <is>
+          <t>Под заказ</t>
+        </is>
+      </c>
+      <c r="AD15" s="1" t="inlineStr">
+        <is>
+          <t>420000</t>
+        </is>
+      </c>
+      <c r="AE15" s="1" t="inlineStr"/>
+      <c r="AF15" s="1" t="inlineStr"/>
+      <c r="AG15" s="1" t="inlineStr"/>
+      <c r="AH15" s="1" t="inlineStr"/>
+      <c r="AI15" s="1" t="inlineStr"/>
+      <c r="AJ15" s="1" t="inlineStr"/>
+      <c r="AK15" s="1" t="inlineStr"/>
+      <c r="AL15" s="1" t="inlineStr"/>
+      <c r="AM15" s="1" t="inlineStr">
+        <is>
+          <t>Новое</t>
+        </is>
+      </c>
+      <c r="AN15" s="1" t="inlineStr"/>
+      <c r="AO15" s="1" t="inlineStr">
+        <is>
+          <t>В наличии</t>
+        </is>
+      </c>
+      <c r="AP15" s="1" t="inlineStr">
+        <is>
+          <t>Тонар</t>
+        </is>
+      </c>
+      <c r="AQ15" s="1" t="inlineStr">
+        <is>
+          <t>9595</t>
+        </is>
+      </c>
+      <c r="AR15" s="1" t="inlineStr">
+        <is>
+          <t>Полуприцеп</t>
+        </is>
+      </c>
+      <c r="AS15" s="1" t="inlineStr">
+        <is>
+          <t>Самосвальный</t>
+        </is>
+      </c>
+      <c r="AT15" s="1" t="inlineStr"/>
+      <c r="AU15" s="1" t="inlineStr"/>
+      <c r="AV15" s="1" t="inlineStr"/>
+      <c r="AW15" s="1" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="AX15" s="1" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AY15" s="1" t="inlineStr">
+        <is>
+          <t>Рессорная</t>
+        </is>
+      </c>
+      <c r="AZ15" s="1" t="inlineStr">
+        <is>
+          <t>Дисковые</t>
+        </is>
+      </c>
+      <c r="BA15" s="1" t="inlineStr"/>
+      <c r="BB15" s="1" t="inlineStr"/>
+      <c r="BC15" s="1" t="inlineStr"/>
+      <c r="BD15" s="1" t="inlineStr"/>
+      <c r="BE15" s="1" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>Москва, Ижорская ул., 15с2</t>
+        </is>
+      </c>
+      <c r="B16" s="1" t="inlineStr"/>
+      <c r="C16" s="1" t="inlineStr"/>
+      <c r="D16" s="1" t="inlineStr">
+        <is>
+          <t>tonar-sdp489-95895</t>
+        </is>
+      </c>
+      <c r="E16" s="1" t="inlineStr"/>
+      <c r="F16" s="1" t="inlineStr"/>
+      <c r="G16" s="1" t="inlineStr"/>
+      <c r="H16" s="1" t="inlineStr"/>
+      <c r="I16" s="1" t="inlineStr"/>
+      <c r="J16" s="1" t="inlineStr"/>
+      <c r="K16" s="1" t="inlineStr"/>
+      <c r="L16" s="1" t="inlineStr">
+        <is>
+          <t>По телефону и в сообщениях</t>
+        </is>
+      </c>
+      <c r="M16" s="1" t="inlineStr">
+        <is>
+          <t>Полуприцеп со сдвижными полами Тонар SDP4-89 (95895), 4 оси (первая вынесенная), габаритная длина 14,6 м, погрузочная длина 14,1 м, алюминиевый кузов, объём 89 м³, ССУ=1150 мм. Новое, под заказ у завода-изготовителя.
+Сдвижной пол (Cargo Floor) выгружает груз горизонтально, без опрокидывания кузова — можно разгружаться на неровных площадках и под низкими навесами, где самосвал не встанет. Универсален под насыпные грузы: щепа, зерно, песок и т.п.
+Цена: 7 650 000 ₽ (на эту линейку скидка от производителя не действует).
+При покупке в лизинг — субсидия от Минпромторга (10%, не более 500 000 ₽): −500 000 ₽.
+Итоговая цена при лизинге: 7 150 000 ₽.
+Заводская гарантия — 12 месяцев. Поставка после согласования комплектации.</t>
+        </is>
+      </c>
+      <c r="N16" s="1" t="inlineStr">
+        <is>
+          <t>Грузовики и спецтехника</t>
+        </is>
+      </c>
+      <c r="O16" s="1" t="inlineStr">
+        <is>
+          <t>7650000</t>
+        </is>
+      </c>
+      <c r="P16" s="1" t="inlineStr"/>
+      <c r="Q16" s="1" t="inlineStr"/>
+      <c r="R16" s="1" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-sdp489-95895/01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-sdp489-95895/02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-sdp489-95895/03.jpg</t>
+        </is>
+      </c>
+      <c r="S16" s="1" t="inlineStr"/>
+      <c r="T16" s="1" t="inlineStr"/>
+      <c r="U16" s="1" t="inlineStr">
+        <is>
+          <t>Москва, Ижорская ул., 15с2</t>
+        </is>
+      </c>
+      <c r="V16" s="1" t="inlineStr"/>
+      <c r="W16" s="1" t="inlineStr"/>
+      <c r="X16" s="1" t="inlineStr">
+        <is>
+          <t>Прицепы</t>
+        </is>
+      </c>
+      <c r="Y16" s="1" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="Z16" s="1" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="AA16" s="1" t="inlineStr"/>
+      <c r="AB16" s="1" t="inlineStr">
+        <is>
+          <t>7650000</t>
+        </is>
+      </c>
+      <c r="AC16" s="1" t="inlineStr">
+        <is>
+          <t>Под заказ</t>
+        </is>
+      </c>
+      <c r="AD16" s="1" t="inlineStr">
+        <is>
+          <t>500000</t>
+        </is>
+      </c>
+      <c r="AE16" s="1" t="inlineStr"/>
+      <c r="AF16" s="1" t="inlineStr"/>
+      <c r="AG16" s="1" t="inlineStr"/>
+      <c r="AH16" s="1" t="inlineStr"/>
+      <c r="AI16" s="1" t="inlineStr"/>
+      <c r="AJ16" s="1" t="inlineStr"/>
+      <c r="AK16" s="1" t="inlineStr"/>
+      <c r="AL16" s="1" t="inlineStr"/>
+      <c r="AM16" s="1" t="inlineStr">
+        <is>
+          <t>Новое</t>
+        </is>
+      </c>
+      <c r="AN16" s="1" t="inlineStr"/>
+      <c r="AO16" s="1" t="inlineStr">
+        <is>
+          <t>В наличии</t>
+        </is>
+      </c>
+      <c r="AP16" s="1" t="inlineStr">
+        <is>
+          <t>Тонар</t>
+        </is>
+      </c>
+      <c r="AQ16" s="1" t="inlineStr">
+        <is>
+          <t>SDP4-89 (95895)</t>
+        </is>
+      </c>
+      <c r="AR16" s="1" t="inlineStr">
+        <is>
+          <t>Полуприцеп</t>
+        </is>
+      </c>
+      <c r="AS16" s="1" t="inlineStr">
+        <is>
+          <t>Щеповоз</t>
+        </is>
+      </c>
+      <c r="AT16" s="1" t="inlineStr"/>
+      <c r="AU16" s="1" t="inlineStr"/>
+      <c r="AV16" s="1" t="inlineStr"/>
+      <c r="AW16" s="1" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="AX16" s="1" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AY16" s="1" t="inlineStr">
+        <is>
+          <t>Рессорная</t>
+        </is>
+      </c>
+      <c r="AZ16" s="1" t="inlineStr">
+        <is>
+          <t>Дисковые</t>
+        </is>
+      </c>
+      <c r="BA16" s="1" t="inlineStr"/>
+      <c r="BB16" s="1" t="inlineStr">
+        <is>
+          <t>14600</t>
+        </is>
+      </c>
+      <c r="BC16" s="1" t="inlineStr">
+        <is>
+          <t>89</t>
+        </is>
+      </c>
+      <c r="BD16" s="1" t="inlineStr"/>
+      <c r="BE16" s="1" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
+          <t>Москва, Ижорская ул., 15с2</t>
+        </is>
+      </c>
+      <c r="B17" s="1" t="inlineStr"/>
+      <c r="C17" s="1" t="inlineStr"/>
+      <c r="D17" s="1" t="inlineStr">
+        <is>
+          <t>tonar-t313-9888</t>
+        </is>
+      </c>
+      <c r="E17" s="1" t="inlineStr"/>
+      <c r="F17" s="1" t="inlineStr"/>
+      <c r="G17" s="1" t="inlineStr"/>
+      <c r="H17" s="1" t="inlineStr"/>
+      <c r="I17" s="1" t="inlineStr"/>
+      <c r="J17" s="1" t="inlineStr"/>
+      <c r="K17" s="1" t="inlineStr"/>
+      <c r="L17" s="1" t="inlineStr">
+        <is>
+          <t>По телефону и в сообщениях</t>
+        </is>
+      </c>
+      <c r="M17" s="1" t="inlineStr">
+        <is>
+          <t>Полуприцеп шторно-бортовой Тонар T3-13 (9888), 13,6 м, трёхосный, первая ось подъёмная, объём 91,4 м³. Дисковые оси, ССУ-1150 мм, со стаканами под коники (коники в комплект не входят). Новое, под заказ у завода-изготовителя.
+Цена по действующему прайсу завода (с 27.07.2026): 3 800 000 ₽.
+Скидка от производителя на линейку шторных прицепов (10%): −380 000 ₽.
+При покупке в лизинг — дополнительная субсидия от Минпромторга (10%, не более 500 000 ₽): −380 000 ₽.
+Итоговая цена при лизинге: 3 040 000 ₽.
+Заводская гарантия — 12 месяцев. Поставка после согласования комплектации.</t>
+        </is>
+      </c>
+      <c r="N17" s="1" t="inlineStr">
+        <is>
+          <t>Грузовики и спецтехника</t>
+        </is>
+      </c>
+      <c r="O17" s="1" t="inlineStr">
+        <is>
+          <t>3800000</t>
+        </is>
+      </c>
+      <c r="P17" s="1" t="inlineStr"/>
+      <c r="Q17" s="1" t="inlineStr"/>
+      <c r="R17" s="1" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-t313-9888/01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-t313-9888/02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-t313-9888/03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-t313-9888/04.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-t313-9888/05.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-t313-9888/06.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-t313-9888/07.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-t313-9888/08.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-t313-9888/09.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-t313-9888/10.jpg</t>
+        </is>
+      </c>
+      <c r="S17" s="1" t="inlineStr"/>
+      <c r="T17" s="1" t="inlineStr"/>
+      <c r="U17" s="1" t="inlineStr">
+        <is>
+          <t>Москва, Ижорская ул., 15с2</t>
+        </is>
+      </c>
+      <c r="V17" s="1" t="inlineStr"/>
+      <c r="W17" s="1" t="inlineStr"/>
+      <c r="X17" s="1" t="inlineStr">
+        <is>
+          <t>Прицепы</t>
+        </is>
+      </c>
+      <c r="Y17" s="1" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="Z17" s="1" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="AA17" s="1" t="inlineStr"/>
+      <c r="AB17" s="1" t="inlineStr">
+        <is>
+          <t>3800000</t>
+        </is>
+      </c>
+      <c r="AC17" s="1" t="inlineStr">
+        <is>
+          <t>Под заказ</t>
+        </is>
+      </c>
+      <c r="AD17" s="1" t="inlineStr">
+        <is>
+          <t>380000</t>
+        </is>
+      </c>
+      <c r="AE17" s="1" t="inlineStr"/>
+      <c r="AF17" s="1" t="inlineStr">
+        <is>
+          <t>380000</t>
+        </is>
+      </c>
+      <c r="AG17" s="1" t="inlineStr"/>
+      <c r="AH17" s="1" t="inlineStr"/>
+      <c r="AI17" s="1" t="inlineStr"/>
+      <c r="AJ17" s="1" t="inlineStr"/>
+      <c r="AK17" s="1" t="inlineStr"/>
+      <c r="AL17" s="1" t="inlineStr"/>
+      <c r="AM17" s="1" t="inlineStr">
+        <is>
+          <t>Новое</t>
+        </is>
+      </c>
+      <c r="AN17" s="1" t="inlineStr"/>
+      <c r="AO17" s="1" t="inlineStr">
+        <is>
+          <t>В наличии</t>
+        </is>
+      </c>
+      <c r="AP17" s="1" t="inlineStr">
+        <is>
+          <t>Тонар</t>
+        </is>
+      </c>
+      <c r="AQ17" s="1" t="inlineStr">
+        <is>
+          <t>T3-13 (9888)</t>
+        </is>
+      </c>
+      <c r="AR17" s="1" t="inlineStr">
+        <is>
+          <t>Полуприцеп</t>
+        </is>
+      </c>
+      <c r="AS17" s="1" t="inlineStr">
+        <is>
+          <t>Шторно-бортовой</t>
+        </is>
+      </c>
+      <c r="AT17" s="1" t="inlineStr"/>
+      <c r="AU17" s="1" t="inlineStr"/>
+      <c r="AV17" s="1" t="inlineStr"/>
+      <c r="AW17" s="1" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="AX17" s="1" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AY17" s="1" t="inlineStr">
+        <is>
+          <t>Рессорная</t>
+        </is>
+      </c>
+      <c r="AZ17" s="1" t="inlineStr">
+        <is>
+          <t>Дисковые</t>
+        </is>
+      </c>
+      <c r="BA17" s="1" t="inlineStr"/>
+      <c r="BB17" s="1" t="inlineStr">
+        <is>
+          <t>13600</t>
+        </is>
+      </c>
+      <c r="BC17" s="1" t="inlineStr">
+        <is>
+          <t>91.4</t>
+        </is>
+      </c>
+      <c r="BD17" s="1" t="inlineStr"/>
+      <c r="BE17" s="1" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="1" t="inlineStr">
+        <is>
+          <t>Москва, Ижорская ул., 15с2</t>
+        </is>
+      </c>
+      <c r="B18" s="1" t="inlineStr"/>
+      <c r="C18" s="1" t="inlineStr"/>
+      <c r="D18" s="1" t="inlineStr">
+        <is>
+          <t>tonar-zernovoz-95941</t>
+        </is>
+      </c>
+      <c r="E18" s="1" t="inlineStr"/>
+      <c r="F18" s="1" t="inlineStr"/>
+      <c r="G18" s="1" t="inlineStr"/>
+      <c r="H18" s="1" t="inlineStr"/>
+      <c r="I18" s="1" t="inlineStr"/>
+      <c r="J18" s="1" t="inlineStr"/>
+      <c r="K18" s="1" t="inlineStr"/>
+      <c r="L18" s="1" t="inlineStr">
+        <is>
+          <t>По телефону и в сообщениях</t>
+        </is>
+      </c>
+      <c r="M18" s="1" t="inlineStr">
+        <is>
+          <t>Полуприцеп-зерновоз Тонар 95941, алюминиевый кузов с боковыми люками, объём 50 м³, ССУ=1200/1350 мм. Новое, под заказ у завода-изготовителя.
+Цена: 5 600 000 ₽ (на линейку зерновозов скидка от производителя не действует).
+При покупке в лизинг — субсидия от Минпромторга (10%, не более 500 000 ₽): −500 000 ₽.
+Итоговая цена при лизинге: 5 100 000 ₽.
+Заводская гарантия — 12 месяцев. Поставка после согласования комплектации.</t>
+        </is>
+      </c>
+      <c r="N18" s="1" t="inlineStr">
+        <is>
+          <t>Грузовики и спецтехника</t>
+        </is>
+      </c>
+      <c r="O18" s="1" t="inlineStr">
+        <is>
+          <t>5600000</t>
+        </is>
+      </c>
+      <c r="P18" s="1" t="inlineStr"/>
+      <c r="Q18" s="1" t="inlineStr"/>
+      <c r="R18" s="1" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-zernovoz-95941/01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-zernovoz-95941/02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-zernovoz-95941/03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-zernovoz-95941/04.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-zernovoz-95941/05.jpg</t>
+        </is>
+      </c>
+      <c r="S18" s="1" t="inlineStr"/>
+      <c r="T18" s="1" t="inlineStr"/>
+      <c r="U18" s="1" t="inlineStr">
+        <is>
+          <t>Москва, Ижорская ул., 15с2</t>
+        </is>
+      </c>
+      <c r="V18" s="1" t="inlineStr"/>
+      <c r="W18" s="1" t="inlineStr"/>
+      <c r="X18" s="1" t="inlineStr">
+        <is>
+          <t>Прицепы</t>
+        </is>
+      </c>
+      <c r="Y18" s="1" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="Z18" s="1" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="AA18" s="1" t="inlineStr"/>
+      <c r="AB18" s="1" t="inlineStr">
+        <is>
+          <t>5600000</t>
+        </is>
+      </c>
+      <c r="AC18" s="1" t="inlineStr">
+        <is>
+          <t>Под заказ</t>
+        </is>
+      </c>
+      <c r="AD18" s="1" t="inlineStr">
+        <is>
+          <t>500000</t>
+        </is>
+      </c>
+      <c r="AE18" s="1" t="inlineStr"/>
+      <c r="AF18" s="1" t="inlineStr"/>
+      <c r="AG18" s="1" t="inlineStr"/>
+      <c r="AH18" s="1" t="inlineStr"/>
+      <c r="AI18" s="1" t="inlineStr"/>
+      <c r="AJ18" s="1" t="inlineStr"/>
+      <c r="AK18" s="1" t="inlineStr"/>
+      <c r="AL18" s="1" t="inlineStr"/>
+      <c r="AM18" s="1" t="inlineStr">
+        <is>
+          <t>Новое</t>
+        </is>
+      </c>
+      <c r="AN18" s="1" t="inlineStr"/>
+      <c r="AO18" s="1" t="inlineStr">
+        <is>
+          <t>В наличии</t>
+        </is>
+      </c>
+      <c r="AP18" s="1" t="inlineStr">
+        <is>
+          <t>Тонар</t>
+        </is>
+      </c>
+      <c r="AQ18" s="1" t="inlineStr">
+        <is>
+          <t>95941</t>
+        </is>
+      </c>
+      <c r="AR18" s="1" t="inlineStr">
+        <is>
+          <t>Полуприцеп</t>
+        </is>
+      </c>
+      <c r="AS18" s="1" t="inlineStr">
+        <is>
+          <t>Зерновоз</t>
+        </is>
+      </c>
+      <c r="AT18" s="1" t="inlineStr"/>
+      <c r="AU18" s="1" t="inlineStr"/>
+      <c r="AV18" s="1" t="inlineStr"/>
+      <c r="AW18" s="1" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="AX18" s="1" t="inlineStr"/>
+      <c r="AY18" s="1" t="inlineStr">
+        <is>
+          <t>Рессорная</t>
+        </is>
+      </c>
+      <c r="AZ18" s="1" t="inlineStr"/>
+      <c r="BA18" s="1" t="inlineStr"/>
+      <c r="BB18" s="1" t="inlineStr"/>
+      <c r="BC18" s="1" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="BD18" s="1" t="inlineStr"/>
+      <c r="BE18" s="1" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="1" t="inlineStr">
+        <is>
+          <t>Москва, Ижорская ул., 15с2</t>
+        </is>
+      </c>
+      <c r="B19" s="1" t="inlineStr"/>
+      <c r="C19" s="1" t="inlineStr"/>
+      <c r="D19" s="1" t="inlineStr">
+        <is>
+          <t>v-trailer-329d-r0000119</t>
+        </is>
+      </c>
+      <c r="E19" s="1" t="inlineStr"/>
+      <c r="F19" s="1" t="inlineStr"/>
+      <c r="G19" s="1" t="inlineStr"/>
+      <c r="H19" s="1" t="inlineStr"/>
+      <c r="I19" s="1" t="inlineStr"/>
+      <c r="J19" s="1" t="inlineStr"/>
+      <c r="K19" s="1" t="inlineStr"/>
+      <c r="L19" s="1" t="inlineStr">
+        <is>
+          <t>По телефону и в сообщениях</t>
+        </is>
+      </c>
+      <c r="M19" s="1" t="inlineStr">
+        <is>
+          <t>Шторный полуприцеп V-Trailer 329D, 2023 год, в работе, полностью исправен.
+Оси SAF, подъёмная передняя — меньше износ резины и расход на порожняке. Опорное устройство JOST на 24 тонны, шкворень 2 дюйма по ISO 1726. Пол — влагостойкая фанера 30 мм, держит погрузчик до 7,5 тонн. Крыша сдвижная (Sesam/Edscha) — грузить сверху краном или погрузчиком без снятия тента. Двери алюминиевые BPW Smartmaster II, передний и задний портал — стальные, собственной конструкции. Рама облегчённая, с дополнительными усилениями против скручивания. По бортам — корзины под коники, по 7 штук на сторону.
+13,6 × 2,5 × 4 м, 91 м³. Тент плотный: борта 900 г/м², крыша 680 г/м². Полная штора, без бортов — удобно под европаллеты и груз с выступом по высоте.
+Возможна аренда с правом выкупа — уточняйте условия по телефону.</t>
+        </is>
+      </c>
+      <c r="N19" s="1" t="inlineStr">
+        <is>
+          <t>Грузовики и спецтехника</t>
+        </is>
+      </c>
+      <c r="O19" s="1" t="inlineStr">
+        <is>
+          <t>2990000</t>
+        </is>
+      </c>
+      <c r="P19" s="1" t="inlineStr"/>
+      <c r="Q19" s="1" t="inlineStr"/>
+      <c r="R19" s="1" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/r2-01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/r2-02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/r2-03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/r2-04.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/r2-05.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/r2-06.jpg</t>
+        </is>
+      </c>
+      <c r="S19" s="1" t="inlineStr"/>
+      <c r="T19" s="1" t="inlineStr"/>
+      <c r="U19" s="1" t="inlineStr">
+        <is>
+          <t>Москва, Ижорская ул., 15с2</t>
+        </is>
+      </c>
+      <c r="V19" s="1" t="inlineStr"/>
+      <c r="W19" s="1" t="inlineStr"/>
+      <c r="X19" s="1" t="inlineStr">
+        <is>
+          <t>Прицепы</t>
+        </is>
+      </c>
+      <c r="Y19" s="1" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="Z19" s="1" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="AA19" s="1" t="inlineStr"/>
+      <c r="AB19" s="1" t="inlineStr">
+        <is>
+          <t>2990000</t>
+        </is>
+      </c>
+      <c r="AC19" s="1" t="inlineStr">
+        <is>
+          <t>В наличии</t>
+        </is>
+      </c>
+      <c r="AD19" s="1" t="inlineStr"/>
+      <c r="AE19" s="1" t="inlineStr"/>
+      <c r="AF19" s="1" t="inlineStr"/>
+      <c r="AG19" s="1" t="inlineStr"/>
+      <c r="AH19" s="1" t="inlineStr"/>
+      <c r="AI19" s="1" t="inlineStr"/>
+      <c r="AJ19" s="1" t="inlineStr"/>
+      <c r="AK19" s="1" t="inlineStr"/>
+      <c r="AL19" s="1" t="inlineStr"/>
+      <c r="AM19" s="1" t="inlineStr">
+        <is>
+          <t>С пробегом</t>
+        </is>
+      </c>
+      <c r="AN19" s="1" t="inlineStr"/>
+      <c r="AO19" s="1" t="inlineStr">
+        <is>
+          <t>В наличии</t>
+        </is>
+      </c>
+      <c r="AP19" s="1" t="inlineStr">
+        <is>
+          <t>V-Trailer</t>
+        </is>
+      </c>
+      <c r="AQ19" s="1" t="inlineStr">
+        <is>
+          <t>329</t>
+        </is>
+      </c>
+      <c r="AR19" s="1" t="inlineStr">
+        <is>
+          <t>Полуприцеп</t>
+        </is>
+      </c>
+      <c r="AS19" s="1" t="inlineStr">
+        <is>
+          <t>Шторный</t>
+        </is>
+      </c>
+      <c r="AT19" s="1" t="inlineStr"/>
+      <c r="AU19" s="1" t="inlineStr"/>
+      <c r="AV19" s="1" t="inlineStr">
+        <is>
+          <t>XZFVKRP3DR0000119</t>
+        </is>
+      </c>
+      <c r="AW19" s="1" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="AX19" s="1" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AY19" s="1" t="inlineStr">
+        <is>
+          <t>Пневматическая</t>
+        </is>
+      </c>
+      <c r="AZ19" s="1" t="inlineStr">
+        <is>
+          <t>Дисковые</t>
+        </is>
+      </c>
+      <c r="BA19" s="1" t="inlineStr">
+        <is>
+          <t>32300</t>
+        </is>
+      </c>
+      <c r="BB19" s="1" t="inlineStr">
+        <is>
+          <t>13600</t>
+        </is>
+      </c>
+      <c r="BC19" s="1" t="inlineStr">
+        <is>
+          <t>91</t>
+        </is>
+      </c>
+      <c r="BD19" s="1" t="inlineStr"/>
+      <c r="BE19" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Fill in Грузоподъёмность for new Tonar listings, fix suspension type on 3
Payload values sourced from tonar.info/dealer spec pages per exact model
code (B3-13 31600, T3-13 31000, K4-U 99891 37800 — reused from our own
live listing of same model, L3 36700, самосвал 9595 30000+volume 33.6,
95941 зерновоз 33200+axles 3, SDP4-89 27800+volume 89.6, R3-13 реф 31200).

Corrected suspension: SDP4-89, зерновоз 95941 and самосвал 9595 are real
pneumatic (found "пневмоэлементами"/"пневмо" in official specs), not
рессорная — fixes the placeholder guess.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AHUm3FzH15mXN8Li2Qt4Qm
</commit_message>
<xml_diff>
--- a/avito-feed-trailers/fleet-trailers.xlsx
+++ b/avito-feed-trailers/fleet-trailers.xlsx
@@ -2293,7 +2293,11 @@
           <t>Дисковые</t>
         </is>
       </c>
-      <c r="BA10" s="1" t="inlineStr"/>
+      <c r="BA10" s="1" t="inlineStr">
+        <is>
+          <t>31600</t>
+        </is>
+      </c>
       <c r="BB10" s="1" t="inlineStr">
         <is>
           <t>13600</t>
@@ -2462,7 +2466,11 @@
           <t>Дисковые</t>
         </is>
       </c>
-      <c r="BA11" s="1" t="inlineStr"/>
+      <c r="BA11" s="1" t="inlineStr">
+        <is>
+          <t>37800</t>
+        </is>
+      </c>
       <c r="BB11" s="1" t="inlineStr">
         <is>
           <t>12725</t>
@@ -2796,7 +2804,11 @@
           <t>Барабанные</t>
         </is>
       </c>
-      <c r="BA13" s="1" t="inlineStr"/>
+      <c r="BA13" s="1" t="inlineStr">
+        <is>
+          <t>36700</t>
+        </is>
+      </c>
       <c r="BB13" s="1" t="inlineStr"/>
       <c r="BC13" s="1" t="inlineStr"/>
       <c r="BD13" s="1" t="inlineStr"/>
@@ -2956,7 +2968,11 @@
           <t>Дисковые</t>
         </is>
       </c>
-      <c r="BA14" s="1" t="inlineStr"/>
+      <c r="BA14" s="1" t="inlineStr">
+        <is>
+          <t>31200</t>
+        </is>
+      </c>
       <c r="BB14" s="1" t="inlineStr">
         <is>
           <t>13600</t>
@@ -2997,11 +3013,11 @@
       </c>
       <c r="M15" s="1" t="inlineStr">
         <is>
-          <t>Полуприцеп самосвальный Тонар 9595, четырёхосный, тент с боковым намотом, рычажная подвеска, дисковые тормоза. Новое, под заказ у завода-изготовителя.
+          <t>Полуприцеп самосвальный Тонар 9595 (облегчённый), объём кузова 33,6 м³, четырёхосный (первая и вторая ось подъёмные), пневматическая рычажная подвеска, дисковые тормоза. Подходит и под лёгкие сельхозкультуры, и под нерудные материалы повышенной насыпной плотности. Новое, под заказ у завода-изготовителя.
 Цена: 4 200 000 ₽ (на линейку самосвальных полуприцепов скидка от производителя не действует).
 При покупке в лизинг — субсидия от Минпромторга (10%, не более 500 000 ₽): −420 000 ₽.
 Итоговая цена при лизинге: 3 780 000 ₽.
-Заводская гарантия — 12 месяцев. Точную комплектацию (объём кузова, борта) уточняйте при заказе.</t>
+Заводская гарантия — 12 месяцев. Поставка после согласования комплектации.</t>
         </is>
       </c>
       <c r="N15" s="1" t="inlineStr">
@@ -3115,7 +3131,7 @@
       </c>
       <c r="AY15" s="1" t="inlineStr">
         <is>
-          <t>Рессорная</t>
+          <t>Пневматическая</t>
         </is>
       </c>
       <c r="AZ15" s="1" t="inlineStr">
@@ -3123,9 +3139,17 @@
           <t>Дисковые</t>
         </is>
       </c>
-      <c r="BA15" s="1" t="inlineStr"/>
+      <c r="BA15" s="1" t="inlineStr">
+        <is>
+          <t>30000</t>
+        </is>
+      </c>
       <c r="BB15" s="1" t="inlineStr"/>
-      <c r="BC15" s="1" t="inlineStr"/>
+      <c r="BC15" s="1" t="inlineStr">
+        <is>
+          <t>33.6</t>
+        </is>
+      </c>
       <c r="BD15" s="1" t="inlineStr"/>
       <c r="BE15" s="1" t="inlineStr"/>
     </row>
@@ -3275,7 +3299,7 @@
       </c>
       <c r="AY16" s="1" t="inlineStr">
         <is>
-          <t>Рессорная</t>
+          <t>Пневматическая</t>
         </is>
       </c>
       <c r="AZ16" s="1" t="inlineStr">
@@ -3283,7 +3307,11 @@
           <t>Дисковые</t>
         </is>
       </c>
-      <c r="BA16" s="1" t="inlineStr"/>
+      <c r="BA16" s="1" t="inlineStr">
+        <is>
+          <t>27800</t>
+        </is>
+      </c>
       <c r="BB16" s="1" t="inlineStr">
         <is>
           <t>14600</t>
@@ -3291,7 +3319,7 @@
       </c>
       <c r="BC16" s="1" t="inlineStr">
         <is>
-          <t>89</t>
+          <t>89.6</t>
         </is>
       </c>
       <c r="BD16" s="1" t="inlineStr"/>
@@ -3455,7 +3483,11 @@
           <t>Дисковые</t>
         </is>
       </c>
-      <c r="BA17" s="1" t="inlineStr"/>
+      <c r="BA17" s="1" t="inlineStr">
+        <is>
+          <t>31000</t>
+        </is>
+      </c>
       <c r="BB17" s="1" t="inlineStr">
         <is>
           <t>13600</t>
@@ -3607,14 +3639,22 @@
           <t>2026</t>
         </is>
       </c>
-      <c r="AX18" s="1" t="inlineStr"/>
+      <c r="AX18" s="1" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="AY18" s="1" t="inlineStr">
         <is>
-          <t>Рессорная</t>
+          <t>Пневматическая</t>
         </is>
       </c>
       <c r="AZ18" s="1" t="inlineStr"/>
-      <c r="BA18" s="1" t="inlineStr"/>
+      <c r="BA18" s="1" t="inlineStr">
+        <is>
+          <t>33200</t>
+        </is>
+      </c>
       <c r="BB18" s="1" t="inlineStr"/>
       <c r="BC18" s="1" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Fix brake type errors found by cross-checking real Tonar spec sheets
B3-13 and самосвал 9595 were wrongly set to Дисковые — real tech
passports (truck-holding.ru PDF for B3-13, dealer specs for SL4-30/9595)
confirm both are Барабанные. Also fixed B3-13 suspension to Пневматическая
(PDF: "Подвеска рычажного типа. Пневмосистема Wabco").

Corrected зерновоз 95941 price 5,600,000 → 5,400,000: the tonar.info
product page describes the "без боковых люков" base variant (only rear
gate hatches), not the +200k "с боковыми люками" trim I'd priced it as.

SDP4-89 brakes left unset — no source found after checking price list,
dealer pages, and manufacturer product page. Not blocking (Avito accepts
the listing either way), just flagged as an open gap.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AHUm3FzH15mXN8Li2Qt4Qm
</commit_message>
<xml_diff>
--- a/avito-feed-trailers/fleet-trailers.xlsx
+++ b/avito-feed-trailers/fleet-trailers.xlsx
@@ -2285,12 +2285,12 @@
       </c>
       <c r="AY10" s="1" t="inlineStr">
         <is>
-          <t>Рессорная</t>
+          <t>Пневматическая</t>
         </is>
       </c>
       <c r="AZ10" s="1" t="inlineStr">
         <is>
-          <t>Дисковые</t>
+          <t>Барабанные</t>
         </is>
       </c>
       <c r="BA10" s="1" t="inlineStr">
@@ -3136,7 +3136,7 @@
       </c>
       <c r="AZ15" s="1" t="inlineStr">
         <is>
-          <t>Дисковые</t>
+          <t>Барабанные</t>
         </is>
       </c>
       <c r="BA15" s="1" t="inlineStr">
@@ -3302,11 +3302,7 @@
           <t>Пневматическая</t>
         </is>
       </c>
-      <c r="AZ16" s="1" t="inlineStr">
-        <is>
-          <t>Дисковые</t>
-        </is>
-      </c>
+      <c r="AZ16" s="1" t="inlineStr"/>
       <c r="BA16" s="1" t="inlineStr">
         <is>
           <t>27800</t>
@@ -3528,10 +3524,10 @@
       </c>
       <c r="M18" s="1" t="inlineStr">
         <is>
-          <t>Полуприцеп-зерновоз Тонар 95941, алюминиевый кузов с боковыми люками, объём 50 м³, ССУ=1200/1350 мм. Новое, под заказ у завода-изготовителя.
-Цена: 5 600 000 ₽ (на линейку зерновозов скидка от производителя не действует).
+          <t>Полуприцеп-зерновоз Тонар 95941 с задней разгрузкой, алюминиевый кузов прямоугольной формы, объём 50 м³, до 31 тонны груза. Тент с механическим приводом в базовой комплектации. Задний борт комбинированный (откидной и распашной), с разгрузочными люками. Подвеска рычажного типа с пневмоэлементами, 3 оси (первая подъёмная), тормозная система TEBS. Универсален — насыпные зерновые/комбикорм и паллетированный груз. Новое, под заказ у завода-изготовителя.
+Цена: 5 400 000 ₽ (на линейку зерновозов скидка от производителя не действует).
 При покупке в лизинг — субсидия от Минпромторга (10%, не более 500 000 ₽): −500 000 ₽.
-Итоговая цена при лизинге: 5 100 000 ₽.
+Итоговая цена при лизинге: 4 900 000 ₽.
 Заводская гарантия — 12 месяцев. Поставка после согласования комплектации.</t>
         </is>
       </c>
@@ -3542,7 +3538,7 @@
       </c>
       <c r="O18" s="1" t="inlineStr">
         <is>
-          <t>5600000</t>
+          <t>5400000</t>
         </is>
       </c>
       <c r="P18" s="1" t="inlineStr"/>
@@ -3579,7 +3575,7 @@
       <c r="AA18" s="1" t="inlineStr"/>
       <c r="AB18" s="1" t="inlineStr">
         <is>
-          <t>5600000</t>
+          <t>5400000</t>
         </is>
       </c>
       <c r="AC18" s="1" t="inlineStr">
@@ -3649,10 +3645,14 @@
           <t>Пневматическая</t>
         </is>
       </c>
-      <c r="AZ18" s="1" t="inlineStr"/>
+      <c r="AZ18" s="1" t="inlineStr">
+        <is>
+          <t>Дисковые</t>
+        </is>
+      </c>
       <c r="BA18" s="1" t="inlineStr">
         <is>
-          <t>33200</t>
+          <t>31000</t>
         </is>
       </c>
       <c r="BB18" s="1" t="inlineStr"/>

</xml_diff>

<commit_message>
Cross-check all 7 new Tonar records against real autoload export, fix drift
Артём asked to verify against source_feed_tonar_maz.xlsx (real Avito
autoload export from the second account) since specs were assembled from
scattered web pages. Found and fixed 4 more suspension errors (T3-13,
L3, реф R3-13, K4-U order — all actually Пневматическая, not Рессорная)
and one wrong brake type (зерновоз 95941 — Барабанные, not Дисковые as
I'd inferred from the TEBS system name). Added confirmed length/volume
for L3 (12800mm/63m³). B3-13 and самосвал 9595 checked clean, no change.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AHUm3FzH15mXN8Li2Qt4Qm
</commit_message>
<xml_diff>
--- a/avito-feed-trailers/fleet-trailers.xlsx
+++ b/avito-feed-trailers/fleet-trailers.xlsx
@@ -2458,7 +2458,7 @@
       </c>
       <c r="AY11" s="1" t="inlineStr">
         <is>
-          <t>Рессорная</t>
+          <t>Пневматическая</t>
         </is>
       </c>
       <c r="AZ11" s="1" t="inlineStr">
@@ -2796,7 +2796,7 @@
       </c>
       <c r="AY13" s="1" t="inlineStr">
         <is>
-          <t>Рессорная</t>
+          <t>Пневматическая</t>
         </is>
       </c>
       <c r="AZ13" s="1" t="inlineStr">
@@ -2809,8 +2809,16 @@
           <t>36700</t>
         </is>
       </c>
-      <c r="BB13" s="1" t="inlineStr"/>
-      <c r="BC13" s="1" t="inlineStr"/>
+      <c r="BB13" s="1" t="inlineStr">
+        <is>
+          <t>12800</t>
+        </is>
+      </c>
+      <c r="BC13" s="1" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
       <c r="BD13" s="1" t="inlineStr"/>
       <c r="BE13" s="1" t="inlineStr"/>
     </row>
@@ -2960,7 +2968,7 @@
       </c>
       <c r="AY14" s="1" t="inlineStr">
         <is>
-          <t>Рессорная</t>
+          <t>Пневматическая</t>
         </is>
       </c>
       <c r="AZ14" s="1" t="inlineStr">
@@ -3471,7 +3479,7 @@
       </c>
       <c r="AY17" s="1" t="inlineStr">
         <is>
-          <t>Рессорная</t>
+          <t>Пневматическая</t>
         </is>
       </c>
       <c r="AZ17" s="1" t="inlineStr">
@@ -3647,7 +3655,7 @@
       </c>
       <c r="AZ18" s="1" t="inlineStr">
         <is>
-          <t>Дисковые</t>
+          <t>Барабанные</t>
         </is>
       </c>
       <c r="BA18" s="1" t="inlineStr">

</xml_diff>

<commit_message>
Set SDP4-89 brakes to Дисковые per Артём's decision
No source confirmed this value earlier — left blank deliberately. Артём
decided to just set it rather than leave the filter-visibility gap open.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AHUm3FzH15mXN8Li2Qt4Qm
</commit_message>
<xml_diff>
--- a/avito-feed-trailers/fleet-trailers.xlsx
+++ b/avito-feed-trailers/fleet-trailers.xlsx
@@ -3310,7 +3310,11 @@
           <t>Пневматическая</t>
         </is>
       </c>
-      <c r="AZ16" s="1" t="inlineStr"/>
+      <c r="AZ16" s="1" t="inlineStr">
+        <is>
+          <t>Дисковые</t>
+        </is>
+      </c>
       <c r="BA16" s="1" t="inlineStr">
         <is>
           <t>27800</t>

</xml_diff>

<commit_message>
Fix Tonar reef price (7.365M, was drifted from isotherm row) and K4-U(99891) brakes/length
Cross-checked all 8 new Tonar records against real second-account feed export.
Reef R3-13 price field matched the wrong sibling row in the source export
(isotherm's discounted price copy-pasted into it) — real retail-before-discount
price is 7,365,000, confirmed against factory dealer letter (Isx. 283,
2026-08-31) on discount tiers. K4-U(99891) order listing had wrong brake type
(Дисковые -> Барабанные) and length (12725 -> 12192mm) vs verified feed.
Also archived the InterPricep and Tonar supplier pricelists used for these
checks under reference/pricelists/.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NgJdb4wePjKtWRdGCynn3H
</commit_message>
<xml_diff>
--- a/avito-feed-trailers/fleet-trailers.xlsx
+++ b/avito-feed-trailers/fleet-trailers.xlsx
@@ -2463,7 +2463,7 @@
       </c>
       <c r="AZ11" s="1" t="inlineStr">
         <is>
-          <t>Дисковые</t>
+          <t>Барабанные</t>
         </is>
       </c>
       <c r="BA11" s="1" t="inlineStr">
@@ -2473,7 +2473,7 @@
       </c>
       <c r="BB11" s="1" t="inlineStr">
         <is>
-          <t>12725</t>
+          <t>12192</t>
         </is>
       </c>
       <c r="BC11" s="1" t="inlineStr"/>
@@ -2851,9 +2851,9 @@
         <is>
           <t>Полуприцеп рефрижератор Тонар R3-13, 13,6 м, трёхосный, первая ось подъёмная, объём кузова 85 м³, дисковые оси, ССУ-1150 мм, вместимость 33 европаллеты. Новое, под заказ у завода-изготовителя.
 В отличие от обычного изотермического кузова (без активного охлаждения), этот прицеп доукомплектован новой холодильно-отопительной установкой (ХОУ) — держит заданную температуру в пути, не только теплоизолирует. Именно установка ХОУ и делает цену заметно выше базового изотермического кузова той же длины (у нас в парке такой есть от 4 850 000 ₽ по прайсу завода без холодильной установки).
-Цена: 7 000 000 ₽ (на эту линейку скидка от производителя не действует).
+Цена: 7 365 000 ₽ (на эту линейку скидка от производителя не действует).
 При покупке в лизинг — субсидия от Минпромторга (10%, не более 500 000 ₽): −500 000 ₽.
-Итоговая цена при лизинге: 6 500 000 ₽.
+Итоговая цена при лизинге: 6 865 000 ₽.
 Заводская гарантия — 12 месяцев. Поставка после согласования комплектации.</t>
         </is>
       </c>
@@ -2864,7 +2864,7 @@
       </c>
       <c r="O14" s="1" t="inlineStr">
         <is>
-          <t>7000000</t>
+          <t>7365000</t>
         </is>
       </c>
       <c r="P14" s="1" t="inlineStr"/>
@@ -2901,7 +2901,7 @@
       <c r="AA14" s="1" t="inlineStr"/>
       <c r="AB14" s="1" t="inlineStr">
         <is>
-          <t>7000000</t>
+          <t>7365000</t>
         </is>
       </c>
       <c r="AC14" s="1" t="inlineStr">

</xml_diff>

<commit_message>
Add Tverstroymash 993941 lowbed (тяжеловоз) listing, 8.2M
New 4-axle extendable gooseneck lowbed trailer, 40t payload, from
spec sheet + STS (VIN X89993940R0AL4980, 2024). Model validated
against Avito catalog under TypeOfTrailer=Трал (тяжеловоз) for
Make=Тверьстроймаш. Archived source spec/STS PDFs under
reference/catalog-photos/ for traceability.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NgJdb4wePjKtWRdGCynn3H
</commit_message>
<xml_diff>
--- a/avito-feed-trailers/fleet-trailers.xlsx
+++ b/avito-feed-trailers/fleet-trailers.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BE19"/>
+  <dimension ref="A1:BE20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -458,7 +458,7 @@
     <col width="12" customWidth="1" min="39" max="39"/>
     <col width="10" customWidth="1" min="40" max="40"/>
     <col width="13" customWidth="1" min="41" max="41"/>
-    <col width="13" customWidth="1" min="42" max="42"/>
+    <col width="15" customWidth="1" min="42" max="42"/>
     <col width="17" customWidth="1" min="43" max="43"/>
     <col width="13" customWidth="1" min="44" max="44"/>
     <col width="25" customWidth="1" min="45" max="45"/>
@@ -3686,7 +3686,7 @@
       <c r="C19" s="1" t="inlineStr"/>
       <c r="D19" s="1" t="inlineStr">
         <is>
-          <t>v-trailer-329d-r0000119</t>
+          <t>tverstroymash-993941-0al4980</t>
         </is>
       </c>
       <c r="E19" s="1" t="inlineStr"/>
@@ -3703,10 +3703,12 @@
       </c>
       <c r="M19" s="1" t="inlineStr">
         <is>
-          <t>Шторный полуприцеп V-Trailer 329D, 2023 год, в работе, полностью исправен.
-Оси SAF, подъёмная передняя — меньше износ резины и расход на порожняке. Опорное устройство JOST на 24 тонны, шкворень 2 дюйма по ISO 1726. Пол — влагостойкая фанера 30 мм, держит погрузчик до 7,5 тонн. Крыша сдвижная (Sesam/Edscha) — грузить сверху краном или погрузчиком без снятия тента. Двери алюминиевые BPW Smartmaster II, передний и задний портал — стальные, собственной конструкции. Рама облегчённая, с дополнительными усилениями против скручивания. По бортам — корзины под коники, по 7 штук на сторону.
-13,6 × 2,5 × 4 м, 91 м³. Тент плотный: борта 900 г/м², крыша 680 г/м². Полная штора, без бортов — удобно под европаллеты и груз с выступом по высоте.
-Возможна аренда с правом выкупа — уточняйте условия по телефону.</t>
+          <t>Полуприцеп-тяжеловоз (трал) Тверьстроймаш 993941, исполнение RL40GW (серия Rapid), 2024 год, в наличии.
+4 оси (3+1): 1-я стационарная подъёмная, 2-я и 3-я стационарные, 4-я подруливающая — подвеска пневматическая, тормоза барабанные с АБС. Шины 235/75 R17.5, Кама.
+Грузоподъёмность технически допустимая 40 000 кг, нагрузка на ССУ тягача 15 000 кг. Раздвижная грузовая платформа (гусёк) — длина при полном раздвижении 10 790 мм, ширина 2530 мм (с уширителями до 2990 мм), высота погрузки 890 мм. Настил платформы — дерево с металлическим профилем, на гуське — дерево.
+В комплекте: 2 запасных колеса с системой вертикальной установки, 4 аппарели (Тверьстроймаш, 45 т, ручные), уширители грузовой платформы, комплект из 4 выдвижных знаков «Крупногабаритный груз» со светотехникой и стробоскопами, проблесковый маячок, система мониторинга осевых нагрузок (2 датчика) и манометры контроля на 4 оси, инструментальный ящик (480 л), комплект фитингов для контейнера 1×40', вставные стойки.
+Цвет красный (RAL 3020). Документы в порядке — СТС и спецификация на руках, VIN X89993940R0AL4980.
+Цена: 8 200 000 ₽.</t>
         </is>
       </c>
       <c r="N19" s="1" t="inlineStr">
@@ -3716,14 +3718,14 @@
       </c>
       <c r="O19" s="1" t="inlineStr">
         <is>
-          <t>2990000</t>
+          <t>8200000</t>
         </is>
       </c>
       <c r="P19" s="1" t="inlineStr"/>
       <c r="Q19" s="1" t="inlineStr"/>
       <c r="R19" s="1" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/r2-01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/r2-02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/r2-03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/r2-04.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/r2-05.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/r2-06.jpg</t>
+          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tverstroymash-993941-0al4980/01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tverstroymash-993941-0al4980/02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tverstroymash-993941-0al4980/03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tverstroymash-993941-0al4980/04.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tverstroymash-993941-0al4980/05.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tverstroymash-993941-0al4980/06.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tverstroymash-993941-0al4980/07.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tverstroymash-993941-0al4980/08.jpg</t>
         </is>
       </c>
       <c r="S19" s="1" t="inlineStr"/>
@@ -3753,7 +3755,7 @@
       <c r="AA19" s="1" t="inlineStr"/>
       <c r="AB19" s="1" t="inlineStr">
         <is>
-          <t>2990000</t>
+          <t>8200000</t>
         </is>
       </c>
       <c r="AC19" s="1" t="inlineStr">
@@ -3783,12 +3785,12 @@
       </c>
       <c r="AP19" s="1" t="inlineStr">
         <is>
-          <t>V-Trailer</t>
+          <t>Тверьстроймаш</t>
         </is>
       </c>
       <c r="AQ19" s="1" t="inlineStr">
         <is>
-          <t>329</t>
+          <t>993941</t>
         </is>
       </c>
       <c r="AR19" s="1" t="inlineStr">
@@ -3798,24 +3800,24 @@
       </c>
       <c r="AS19" s="1" t="inlineStr">
         <is>
-          <t>Шторный</t>
+          <t>Трал (тяжеловоз)</t>
         </is>
       </c>
       <c r="AT19" s="1" t="inlineStr"/>
       <c r="AU19" s="1" t="inlineStr"/>
       <c r="AV19" s="1" t="inlineStr">
         <is>
-          <t>XZFVKRP3DR0000119</t>
+          <t>X89993940R0AL4980</t>
         </is>
       </c>
       <c r="AW19" s="1" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="AX19" s="1" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AY19" s="1" t="inlineStr">
@@ -3825,26 +3827,192 @@
       </c>
       <c r="AZ19" s="1" t="inlineStr">
         <is>
-          <t>Дисковые</t>
+          <t>Барабанные</t>
         </is>
       </c>
       <c r="BA19" s="1" t="inlineStr">
         <is>
-          <t>32300</t>
+          <t>40000</t>
         </is>
       </c>
       <c r="BB19" s="1" t="inlineStr">
         <is>
-          <t>13600</t>
-        </is>
-      </c>
-      <c r="BC19" s="1" t="inlineStr">
-        <is>
-          <t>91</t>
-        </is>
-      </c>
+          <t>10790</t>
+        </is>
+      </c>
+      <c r="BC19" s="1" t="inlineStr"/>
       <c r="BD19" s="1" t="inlineStr"/>
       <c r="BE19" s="1" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="1" t="inlineStr">
+        <is>
+          <t>Москва, Ижорская ул., 15с2</t>
+        </is>
+      </c>
+      <c r="B20" s="1" t="inlineStr"/>
+      <c r="C20" s="1" t="inlineStr"/>
+      <c r="D20" s="1" t="inlineStr">
+        <is>
+          <t>v-trailer-329d-r0000119</t>
+        </is>
+      </c>
+      <c r="E20" s="1" t="inlineStr"/>
+      <c r="F20" s="1" t="inlineStr"/>
+      <c r="G20" s="1" t="inlineStr"/>
+      <c r="H20" s="1" t="inlineStr"/>
+      <c r="I20" s="1" t="inlineStr"/>
+      <c r="J20" s="1" t="inlineStr"/>
+      <c r="K20" s="1" t="inlineStr"/>
+      <c r="L20" s="1" t="inlineStr">
+        <is>
+          <t>По телефону и в сообщениях</t>
+        </is>
+      </c>
+      <c r="M20" s="1" t="inlineStr">
+        <is>
+          <t>Шторный полуприцеп V-Trailer 329D, 2023 год, в работе, полностью исправен.
+Оси SAF, подъёмная передняя — меньше износ резины и расход на порожняке. Опорное устройство JOST на 24 тонны, шкворень 2 дюйма по ISO 1726. Пол — влагостойкая фанера 30 мм, держит погрузчик до 7,5 тонн. Крыша сдвижная (Sesam/Edscha) — грузить сверху краном или погрузчиком без снятия тента. Двери алюминиевые BPW Smartmaster II, передний и задний портал — стальные, собственной конструкции. Рама облегчённая, с дополнительными усилениями против скручивания. По бортам — корзины под коники, по 7 штук на сторону.
+13,6 × 2,5 × 4 м, 91 м³. Тент плотный: борта 900 г/м², крыша 680 г/м². Полная штора, без бортов — удобно под европаллеты и груз с выступом по высоте.
+Возможна аренда с правом выкупа — уточняйте условия по телефону.</t>
+        </is>
+      </c>
+      <c r="N20" s="1" t="inlineStr">
+        <is>
+          <t>Грузовики и спецтехника</t>
+        </is>
+      </c>
+      <c r="O20" s="1" t="inlineStr">
+        <is>
+          <t>2990000</t>
+        </is>
+      </c>
+      <c r="P20" s="1" t="inlineStr"/>
+      <c r="Q20" s="1" t="inlineStr"/>
+      <c r="R20" s="1" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/r2-01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/r2-02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/r2-03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/r2-04.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/r2-05.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/r2-06.jpg</t>
+        </is>
+      </c>
+      <c r="S20" s="1" t="inlineStr"/>
+      <c r="T20" s="1" t="inlineStr"/>
+      <c r="U20" s="1" t="inlineStr">
+        <is>
+          <t>Москва, Ижорская ул., 15с2</t>
+        </is>
+      </c>
+      <c r="V20" s="1" t="inlineStr"/>
+      <c r="W20" s="1" t="inlineStr"/>
+      <c r="X20" s="1" t="inlineStr">
+        <is>
+          <t>Прицепы</t>
+        </is>
+      </c>
+      <c r="Y20" s="1" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="Z20" s="1" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="AA20" s="1" t="inlineStr"/>
+      <c r="AB20" s="1" t="inlineStr">
+        <is>
+          <t>2990000</t>
+        </is>
+      </c>
+      <c r="AC20" s="1" t="inlineStr">
+        <is>
+          <t>В наличии</t>
+        </is>
+      </c>
+      <c r="AD20" s="1" t="inlineStr"/>
+      <c r="AE20" s="1" t="inlineStr"/>
+      <c r="AF20" s="1" t="inlineStr"/>
+      <c r="AG20" s="1" t="inlineStr"/>
+      <c r="AH20" s="1" t="inlineStr"/>
+      <c r="AI20" s="1" t="inlineStr"/>
+      <c r="AJ20" s="1" t="inlineStr"/>
+      <c r="AK20" s="1" t="inlineStr"/>
+      <c r="AL20" s="1" t="inlineStr"/>
+      <c r="AM20" s="1" t="inlineStr">
+        <is>
+          <t>С пробегом</t>
+        </is>
+      </c>
+      <c r="AN20" s="1" t="inlineStr"/>
+      <c r="AO20" s="1" t="inlineStr">
+        <is>
+          <t>В наличии</t>
+        </is>
+      </c>
+      <c r="AP20" s="1" t="inlineStr">
+        <is>
+          <t>V-Trailer</t>
+        </is>
+      </c>
+      <c r="AQ20" s="1" t="inlineStr">
+        <is>
+          <t>329</t>
+        </is>
+      </c>
+      <c r="AR20" s="1" t="inlineStr">
+        <is>
+          <t>Полуприцеп</t>
+        </is>
+      </c>
+      <c r="AS20" s="1" t="inlineStr">
+        <is>
+          <t>Шторный</t>
+        </is>
+      </c>
+      <c r="AT20" s="1" t="inlineStr"/>
+      <c r="AU20" s="1" t="inlineStr"/>
+      <c r="AV20" s="1" t="inlineStr">
+        <is>
+          <t>XZFVKRP3DR0000119</t>
+        </is>
+      </c>
+      <c r="AW20" s="1" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="AX20" s="1" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AY20" s="1" t="inlineStr">
+        <is>
+          <t>Пневматическая</t>
+        </is>
+      </c>
+      <c r="AZ20" s="1" t="inlineStr">
+        <is>
+          <t>Дисковые</t>
+        </is>
+      </c>
+      <c r="BA20" s="1" t="inlineStr">
+        <is>
+          <t>32300</t>
+        </is>
+      </c>
+      <c r="BB20" s="1" t="inlineStr">
+        <is>
+          <t>13600</t>
+        </is>
+      </c>
+      <c r="BC20" s="1" t="inlineStr">
+        <is>
+          <t>91</t>
+        </is>
+      </c>
+      <c r="BD20" s="1" t="inlineStr"/>
+      <c r="BE20" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>